<commit_message>
chore: refresh SAT cache + report (2026-09-13)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-12</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-13</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-12</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-14)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-13</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-14</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -679,37 +679,37 @@
         <v>7</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>11</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>4</v>
@@ -745,7 +745,7 @@
         <v>6</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>8</v>
@@ -754,19 +754,19 @@
         <v>8</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>6</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>11</v>
@@ -775,13 +775,13 @@
         <v>11</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>16</v>
@@ -817,43 +817,43 @@
         <v>13</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="M6" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>13</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>13</v>
       </c>
       <c r="Q6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="R6" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="T6" s="4" t="n">
+      <c r="U6" s="4" t="n">
         <v>12</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>12</v>
@@ -888,41 +888,43 @@
       <c r="H7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="J7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="M7" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P7" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O7" s="6" t="inlineStr"/>
+      <c r="P7" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="Q7" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -955,28 +957,28 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>6</v>
@@ -985,16 +987,16 @@
         <v>6</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -1023,31 +1025,31 @@
         <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>3</v>
@@ -1056,13 +1058,13 @@
         <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -1098,34 +1100,34 @@
         <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>1</v>
@@ -1134,7 +1136,7 @@
         <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1170,28 +1172,28 @@
         <v>11</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="L11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N11" s="6" t="n">
         <v>9</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>5</v>
@@ -1200,7 +1202,7 @@
         <v>5</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>7</v>
@@ -1235,13 +1237,13 @@
       <c r="G12" s="4" t="inlineStr"/>
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>1</v>
@@ -1249,10 +1251,10 @@
       <c r="M12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O12" s="4" t="inlineStr"/>
+      <c r="N12" s="4" t="inlineStr"/>
+      <c r="O12" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="P12" s="4" t="n">
         <v>2</v>
       </c>
@@ -1260,17 +1262,15 @@
         <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="U12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="U12" s="4" t="inlineStr"/>
       <c r="V12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1306,43 +1306,43 @@
         <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="R13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="T13" s="6" t="n">
         <v>6</v>
-      </c>
-      <c r="S13" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="T13" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -1375,19 +1375,19 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>1</v>
@@ -1399,22 +1399,22 @@
         <v>1</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -1451,37 +1451,37 @@
         <v>10</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R15" s="6" t="n">
         <v>1</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>5</v>
@@ -1515,9 +1515,11 @@
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr"/>
+      <c r="N16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="O16" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>3</v>
@@ -1526,13 +1528,13 @@
         <v>3</v>
       </c>
       <c r="R16" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S16" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U16" s="4" t="n">
         <v>3</v>
@@ -1570,7 +1572,9 @@
       </c>
       <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr"/>
-      <c r="K17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1663,7 +1667,9 @@
       <c r="M19" s="6" t="inlineStr"/>
       <c r="N19" s="6" t="inlineStr"/>
       <c r="O19" s="6" t="inlineStr"/>
-      <c r="P19" s="6" t="inlineStr"/>
+      <c r="P19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q19" s="6" t="n">
         <v>1</v>
       </c>
@@ -1676,9 +1682,7 @@
       <c r="T19" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U19" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="U19" s="6" t="inlineStr"/>
       <c r="V19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1711,7 +1715,7 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>1</v>
@@ -1719,31 +1723,31 @@
       <c r="K20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L20" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" s="4" t="inlineStr"/>
+      <c r="N20" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="O20" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R20" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="R20" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="S20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>1</v>
@@ -1776,22 +1780,22 @@
         <v>1</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>2</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P21" s="6" t="n">
         <v>1</v>
@@ -1799,12 +1803,12 @@
       <c r="Q21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="R21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="R21" s="6" t="inlineStr"/>
       <c r="S21" s="6" t="inlineStr"/>
       <c r="T21" s="6" t="inlineStr"/>
-      <c r="U21" s="6" t="inlineStr"/>
+      <c r="U21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V21" s="6" t="n">
         <v>1</v>
       </c>
@@ -1839,43 +1843,43 @@
         <v>17</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="L22" s="4" t="n">
         <v>18</v>
       </c>
       <c r="M22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="P22" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="N22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="O22" s="4" t="n">
+      <c r="Q22" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="R22" s="4" t="n">
         <v>19</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="V22" s="4" t="n">
         <v>18</v>
@@ -1907,43 +1911,43 @@
         <v>84</v>
       </c>
       <c r="I23" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="K23" s="8" t="n">
         <v>86</v>
       </c>
-      <c r="J23" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="K23" s="8" t="n">
+      <c r="L23" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="L23" s="8" t="n">
-        <v>86</v>
-      </c>
       <c r="M23" s="8" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="O23" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="P23" s="8" t="n">
         <v>99</v>
       </c>
       <c r="Q23" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="T23" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="R23" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="U23" s="8" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="V23" s="8" t="n">
         <v>94</v>
@@ -1992,7 +1996,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-13</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-14</t>
         </is>
       </c>
     </row>
@@ -2034,72 +2038,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -2128,43 +2132,43 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="I4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>17</v>
-      </c>
       <c r="K4" s="4" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="N4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="P4" s="4" t="n">
+      <c r="Q4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="S4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="R4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>22</v>
-      </c>
       <c r="T4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>18</v>
@@ -2195,22 +2199,22 @@
         <v>11</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="M5" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>15</v>
@@ -2222,16 +2226,16 @@
         <v>15</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="R5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="T5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>14</v>
@@ -2274,7 +2278,7 @@
         <v>2</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>1</v>
@@ -2283,22 +2287,22 @@
         <v>1</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>5</v>
@@ -2344,22 +2348,22 @@
         <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>3</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="P7" s="6" t="inlineStr"/>
       <c r="Q7" s="6" t="inlineStr"/>
       <c r="R7" s="6" t="inlineStr"/>
-      <c r="S7" s="6" t="inlineStr"/>
+      <c r="S7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>2</v>
@@ -2399,34 +2403,34 @@
         <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="M8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="O8" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="Q8" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="R8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>5</v>
@@ -2470,25 +2474,25 @@
         <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>3</v>
@@ -2522,10 +2526,10 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>3</v>
@@ -2534,7 +2538,7 @@
         <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>5</v>
@@ -2546,19 +2550,19 @@
         <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>7</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>4</v>
@@ -2589,34 +2593,34 @@
         <v>40</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>38</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K11" s="10" t="n">
         <v>39</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="M11" s="10" t="n">
         <v>41</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="P11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="Q11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>43</v>
       </c>
       <c r="R11" s="10" t="n">
         <v>44</v>
@@ -2625,7 +2629,7 @@
         <v>44</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>43</v>
@@ -2656,43 +2660,43 @@
         <v>84</v>
       </c>
       <c r="H12" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>81</v>
+      </c>
+      <c r="J12" s="8" t="n">
         <v>86</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>84</v>
-      </c>
-      <c r="J12" s="8" t="n">
+      <c r="K12" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="K12" s="8" t="n">
-        <v>86</v>
-      </c>
       <c r="L12" s="8" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="O12" s="8" t="n">
         <v>99</v>
       </c>
       <c r="P12" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="S12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="Q12" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="T12" s="8" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>94</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-15)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-14</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-15</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -676,43 +676,43 @@
         <v>7</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>11</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="S4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="V4" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -751,19 +751,19 @@
         <v>8</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>6</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>11</v>
@@ -772,16 +772,16 @@
         <v>11</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>15</v>
@@ -817,43 +817,43 @@
         <v>13</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="L6" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>13</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>13</v>
       </c>
       <c r="P6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="Q6" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="S6" s="4" t="n">
+      <c r="T6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="T6" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="U6" s="4" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>16</v>
@@ -892,33 +892,33 @@
         <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="L7" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="K7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="M7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O7" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="N7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="P7" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>5</v>
@@ -960,22 +960,22 @@
         <v>4</v>
       </c>
       <c r="J8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="K8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L8" s="4" t="n">
+      <c r="N8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O8" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>6</v>
@@ -984,16 +984,16 @@
         <v>6</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>2</v>
@@ -1028,43 +1028,43 @@
         <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="O9" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="N9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="O9" s="6" t="n">
-        <v>3</v>
-      </c>
       <c r="P9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="S9" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="T9" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="Q9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="R9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="S9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="T9" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="U9" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -1097,34 +1097,34 @@
         <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>1</v>
@@ -1136,7 +1136,7 @@
         <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1169,43 +1169,43 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="K11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M11" s="6" t="n">
         <v>9</v>
-      </c>
-      <c r="L11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="T11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="U11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>8</v>
@@ -1240,7 +1240,7 @@
         <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>1</v>
@@ -1248,10 +1248,10 @@
       <c r="L12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="M12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="inlineStr"/>
+      <c r="N12" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="O12" s="4" t="n">
         <v>2</v>
       </c>
@@ -1259,17 +1259,15 @@
         <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="T12" s="4" t="inlineStr"/>
       <c r="U12" s="4" t="inlineStr"/>
       <c r="V12" s="4" t="inlineStr"/>
     </row>
@@ -1303,43 +1301,43 @@
         <v>3</v>
       </c>
       <c r="I13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="J13" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="K13" s="6" t="n">
-        <v>3</v>
-      </c>
       <c r="L13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="M13" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="M13" s="6" t="n">
-        <v>3</v>
-      </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="Q13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S13" s="6" t="n">
         <v>6</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="S13" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>3</v>
@@ -1375,16 +1373,16 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>1</v>
@@ -1396,16 +1394,16 @@
         <v>1</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>3</v>
@@ -1448,40 +1446,40 @@
         <v>10</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O15" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="O15" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="P15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R15" s="6" t="n">
         <v>4</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>1</v>
       </c>
       <c r="S15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>9</v>
@@ -1514,9 +1512,11 @@
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
-      <c r="M16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="N16" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O16" s="4" t="n">
         <v>3</v>
@@ -1525,13 +1525,13 @@
         <v>3</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R16" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>3</v>
@@ -1571,7 +1571,9 @@
         <v>1</v>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1602,9 +1604,7 @@
       <c r="T17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1638,7 +1638,9 @@
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
-      <c r="U18" s="4" t="inlineStr"/>
+      <c r="U18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1666,7 +1668,9 @@
       <c r="L19" s="6" t="inlineStr"/>
       <c r="M19" s="6" t="inlineStr"/>
       <c r="N19" s="6" t="inlineStr"/>
-      <c r="O19" s="6" t="inlineStr"/>
+      <c r="O19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P19" s="6" t="n">
         <v>1</v>
       </c>
@@ -1679,9 +1683,7 @@
       <c r="S19" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="T19" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="T19" s="6" t="inlineStr"/>
       <c r="U19" s="6" t="inlineStr"/>
       <c r="V19" s="6" t="inlineStr"/>
     </row>
@@ -1720,31 +1722,31 @@
       <c r="J20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K20" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="4" t="inlineStr"/>
-      <c r="M20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="N20" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q20" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="Q20" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="R20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>1</v>
@@ -1777,22 +1779,22 @@
         <v>1</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>2</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O21" s="6" t="n">
         <v>1</v>
@@ -1800,12 +1802,12 @@
       <c r="P21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q21" s="6" t="inlineStr"/>
       <c r="R21" s="6" t="inlineStr"/>
       <c r="S21" s="6" t="inlineStr"/>
-      <c r="T21" s="6" t="inlineStr"/>
+      <c r="T21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U21" s="6" t="n">
         <v>1</v>
       </c>
@@ -1843,43 +1845,43 @@
         <v>17</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K22" s="4" t="n">
         <v>18</v>
       </c>
       <c r="L22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="O22" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="M22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="N22" s="4" t="n">
+      <c r="P22" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>19</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="V22" s="4" t="n">
         <v>15</v>
@@ -1911,46 +1913,46 @@
         <v>84</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="J23" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="K23" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="K23" s="8" t="n">
-        <v>86</v>
-      </c>
       <c r="L23" s="8" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="O23" s="8" t="n">
         <v>99</v>
       </c>
       <c r="P23" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="S23" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="Q23" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="T23" s="8" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1996,7 +1998,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-14</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-15</t>
         </is>
       </c>
     </row>
@@ -2038,72 +2040,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -2132,43 +2134,43 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="M4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="N4" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="O4" s="4" t="n">
+      <c r="P4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="R4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="Q4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>22</v>
-      </c>
       <c r="S4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>16</v>
@@ -2202,16 +2204,16 @@
         <v>11</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="L5" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>15</v>
@@ -2223,22 +2225,22 @@
         <v>15</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="Q5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="S5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>14</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -2275,7 +2277,7 @@
         <v>2</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>1</v>
@@ -2284,25 +2286,25 @@
         <v>1</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>4</v>
@@ -2345,22 +2347,22 @@
         <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>3</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="6" t="inlineStr"/>
       <c r="Q7" s="6" t="inlineStr"/>
-      <c r="R7" s="6" t="inlineStr"/>
+      <c r="R7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="S7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>2</v>
@@ -2400,34 +2402,34 @@
         <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="L8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="N8" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="P8" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="Q8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>5</v>
@@ -2471,31 +2473,31 @@
         <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>2</v>
@@ -2526,7 +2528,7 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>3</v>
@@ -2535,7 +2537,7 @@
         <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>5</v>
@@ -2547,22 +2549,22 @@
         <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>7</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>5</v>
@@ -2596,28 +2598,28 @@
         <v>38</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>39</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="L11" s="10" t="n">
         <v>41</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="O11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="P11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>43</v>
       </c>
       <c r="Q11" s="10" t="n">
         <v>44</v>
@@ -2626,10 +2628,10 @@
         <v>44</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>48</v>
@@ -2660,46 +2662,46 @@
         <v>84</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="I12" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="J12" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="J12" s="8" t="n">
-        <v>86</v>
-      </c>
       <c r="K12" s="8" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>99</v>
       </c>
       <c r="O12" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="R12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="P12" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="S12" s="8" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-16)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-15</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-16</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -673,46 +673,46 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>11</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="R4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="V4" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -748,19 +748,19 @@
         <v>8</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>6</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>11</v>
@@ -769,19 +769,19 @@
         <v>11</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>15</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>16</v>
@@ -817,43 +817,43 @@
         <v>13</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>13</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>13</v>
       </c>
       <c r="O6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="P6" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="R6" s="4" t="n">
+      <c r="S6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="S6" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="T6" s="4" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>11</v>
@@ -889,39 +889,39 @@
         <v>9</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="K7" s="6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="L7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N7" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="M7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="O7" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>9</v>
@@ -957,22 +957,22 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>6</v>
@@ -981,22 +981,22 @@
         <v>6</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -1025,25 +1025,25 @@
         <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>3</v>
@@ -1052,19 +1052,19 @@
         <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>7</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -1097,31 +1097,31 @@
         <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>1</v>
@@ -1136,7 +1136,7 @@
         <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1172,43 +1172,43 @@
         <v>9</v>
       </c>
       <c r="J11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L11" s="6" t="n">
         <v>9</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L11" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="N11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="T11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="U11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="O11" s="6" t="n">
+      <c r="V11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="V11" s="6" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -1237,7 +1237,7 @@
       <c r="G12" s="4" t="inlineStr"/>
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>1</v>
@@ -1245,10 +1245,10 @@
       <c r="K12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="N12" s="4" t="n">
         <v>2</v>
       </c>
@@ -1256,19 +1256,19 @@
         <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="S12" s="4" t="inlineStr"/>
       <c r="T12" s="4" t="inlineStr"/>
-      <c r="U12" s="4" t="inlineStr"/>
+      <c r="U12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V12" s="4" t="n">
         <v>1</v>
       </c>
@@ -1306,43 +1306,43 @@
         <v>3</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="P13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R13" s="6" t="n">
         <v>6</v>
-      </c>
-      <c r="Q13" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>3</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1375,13 +1375,13 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>1</v>
@@ -1393,16 +1393,16 @@
         <v>1</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>3</v>
@@ -1411,7 +1411,7 @@
         <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>2</v>
@@ -1445,43 +1445,43 @@
         <v>7</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P15" s="6" t="n">
         <v>1</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>8</v>
@@ -1513,9 +1513,11 @@
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
-      <c r="L16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="M16" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N16" s="4" t="n">
         <v>3</v>
@@ -1524,13 +1526,13 @@
         <v>3</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S16" s="4" t="n">
         <v>3</v>
@@ -1539,7 +1541,7 @@
         <v>3</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V16" s="4" t="n">
         <v>5</v>
@@ -1572,7 +1574,9 @@
       <c r="H17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1603,9 +1607,7 @@
       <c r="S17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="T17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
     </row>
@@ -1639,7 +1641,9 @@
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
-      <c r="T18" s="4" t="inlineStr"/>
+      <c r="T18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="U18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1669,7 +1673,9 @@
       <c r="K19" s="6" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr"/>
       <c r="M19" s="6" t="inlineStr"/>
-      <c r="N19" s="6" t="inlineStr"/>
+      <c r="N19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O19" s="6" t="n">
         <v>1</v>
       </c>
@@ -1682,9 +1688,7 @@
       <c r="R19" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="S19" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="S19" s="6" t="inlineStr"/>
       <c r="T19" s="6" t="inlineStr"/>
       <c r="U19" s="6" t="inlineStr"/>
       <c r="V19" s="6" t="inlineStr"/>
@@ -1721,31 +1725,31 @@
       <c r="I20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J20" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J20" s="4" t="inlineStr"/>
       <c r="K20" s="4" t="inlineStr"/>
-      <c r="L20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="M20" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O20" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P20" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="P20" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="Q20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>1</v>
@@ -1753,9 +1757,7 @@
       <c r="U20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="V20" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="V20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1781,19 +1783,19 @@
         <v>1</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>2</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>1</v>
@@ -1801,20 +1803,20 @@
       <c r="O21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="P21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="P21" s="6" t="inlineStr"/>
       <c r="Q21" s="6" t="inlineStr"/>
       <c r="R21" s="6" t="inlineStr"/>
-      <c r="S21" s="6" t="inlineStr"/>
+      <c r="S21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -1847,46 +1849,46 @@
         <v>17</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J22" s="4" t="n">
         <v>18</v>
       </c>
       <c r="K22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="N22" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="L22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="M22" s="4" t="n">
+      <c r="O22" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="P22" s="4" t="n">
         <v>19</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="U22" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="V22" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="V22" s="4" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="23">
@@ -1915,46 +1917,46 @@
         <v>84</v>
       </c>
       <c r="I23" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="J23" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="J23" s="8" t="n">
-        <v>86</v>
-      </c>
       <c r="K23" s="8" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="N23" s="8" t="n">
         <v>99</v>
       </c>
       <c r="O23" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="R23" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="P23" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="S23" s="8" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -2000,7 +2002,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-15</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-16</t>
         </is>
       </c>
     </row>
@@ -2042,72 +2044,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -2136,40 +2138,40 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="L4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="N4" s="4" t="n">
+      <c r="O4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="Q4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>22</v>
-      </c>
       <c r="R4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>16</v>
@@ -2203,16 +2205,16 @@
         <v>11</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="K5" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>15</v>
@@ -2224,25 +2226,25 @@
         <v>15</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="P5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="R5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>13</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -2276,7 +2278,7 @@
         <v>2</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>1</v>
@@ -2285,31 +2287,31 @@
         <v>1</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -2346,28 +2348,28 @@
         <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>3</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="N7" s="6" t="inlineStr"/>
       <c r="O7" s="6" t="inlineStr"/>
       <c r="P7" s="6" t="inlineStr"/>
-      <c r="Q7" s="6" t="inlineStr"/>
+      <c r="Q7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>3</v>
@@ -2401,34 +2403,34 @@
         <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="K8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="M8" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="N8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="O8" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="P8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>5</v>
@@ -2472,34 +2474,34 @@
         <v>1</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>5</v>
@@ -2536,7 +2538,7 @@
         <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>5</v>
@@ -2548,22 +2550,22 @@
         <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>7</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>5</v>
@@ -2597,28 +2599,28 @@
         <v>40</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>39</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K11" s="10" t="n">
         <v>41</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="N11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="O11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>43</v>
       </c>
       <c r="P11" s="10" t="n">
         <v>44</v>
@@ -2627,16 +2629,16 @@
         <v>44</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12">
@@ -2664,46 +2666,46 @@
         <v>84</v>
       </c>
       <c r="H12" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="I12" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>86</v>
-      </c>
       <c r="J12" s="8" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="M12" s="8" t="n">
         <v>99</v>
       </c>
       <c r="N12" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="Q12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="O12" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="R12" s="8" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-17)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-16</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-17</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -676,43 +676,43 @@
         <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>11</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -745,19 +745,19 @@
         <v>6</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>6</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>11</v>
@@ -766,25 +766,25 @@
         <v>11</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="S5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="T5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="U5" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -817,46 +817,46 @@
         <v>13</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>13</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>13</v>
       </c>
       <c r="N6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="O6" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="Q6" s="4" t="n">
+      <c r="R6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="R6" s="4" t="n">
-        <v>13</v>
-      </c>
       <c r="S6" s="4" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -888,43 +888,43 @@
       <c r="H7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="I7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="J7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="K7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M7" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="N7" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -957,19 +957,19 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>6</v>
@@ -978,25 +978,25 @@
         <v>6</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -1025,22 +1025,22 @@
         <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>3</v>
@@ -1049,19 +1049,19 @@
         <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>7</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>6</v>
@@ -1097,28 +1097,28 @@
         <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>1</v>
@@ -1133,10 +1133,10 @@
         <v>1</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -1169,43 +1169,43 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K11" s="6" t="n">
         <v>9</v>
-      </c>
-      <c r="J11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="M11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="T11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="N11" s="6" t="n">
+      <c r="U11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>9</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>8</v>
@@ -1242,10 +1242,10 @@
       <c r="J12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="M12" s="4" t="n">
         <v>2</v>
       </c>
@@ -1253,25 +1253,23 @@
         <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="R12" s="4" t="inlineStr"/>
       <c r="S12" s="4" t="inlineStr"/>
-      <c r="T12" s="4" t="inlineStr"/>
+      <c r="T12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="U12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="V12" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="V12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1303,37 +1301,37 @@
         <v>3</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>3</v>
@@ -1378,7 +1376,7 @@
         <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>1</v>
@@ -1390,16 +1388,16 @@
         <v>1</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>3</v>
@@ -1408,13 +1406,13 @@
         <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -1445,43 +1443,43 @@
         <v>7</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O15" s="6" t="n">
         <v>1</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>7</v>
@@ -1512,9 +1510,11 @@
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="L16" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M16" s="4" t="n">
         <v>3</v>
@@ -1523,13 +1523,13 @@
         <v>3</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R16" s="4" t="n">
         <v>3</v>
@@ -1538,10 +1538,10 @@
         <v>3</v>
       </c>
       <c r="T16" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V16" s="4" t="n">
         <v>6</v>
@@ -1604,9 +1604,7 @@
       <c r="R17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="S17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
@@ -1640,7 +1638,9 @@
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
-      <c r="S18" s="4" t="inlineStr"/>
+      <c r="S18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="T18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1672,7 +1672,9 @@
       <c r="J19" s="6" t="inlineStr"/>
       <c r="K19" s="6" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr"/>
-      <c r="M19" s="6" t="inlineStr"/>
+      <c r="M19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N19" s="6" t="n">
         <v>1</v>
       </c>
@@ -1685,9 +1687,7 @@
       <c r="Q19" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="R19" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="R19" s="6" t="inlineStr"/>
       <c r="S19" s="6" t="inlineStr"/>
       <c r="T19" s="6" t="inlineStr"/>
       <c r="U19" s="6" t="inlineStr"/>
@@ -1722,31 +1722,31 @@
       <c r="H20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I20" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I20" s="4" t="inlineStr"/>
       <c r="J20" s="4" t="inlineStr"/>
-      <c r="K20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="L20" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S20" s="4" t="n">
         <v>1</v>
@@ -1754,10 +1754,10 @@
       <c r="T20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="U20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V20" s="4" t="inlineStr"/>
+      <c r="U20" s="4" t="inlineStr"/>
+      <c r="V20" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1783,16 +1783,16 @@
         <v>1</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>2</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>1</v>
@@ -1800,20 +1800,20 @@
       <c r="N21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="O21" s="6" t="inlineStr"/>
       <c r="P21" s="6" t="inlineStr"/>
       <c r="Q21" s="6" t="inlineStr"/>
-      <c r="R21" s="6" t="inlineStr"/>
+      <c r="R21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="S21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>5</v>
@@ -1852,40 +1852,40 @@
         <v>18</v>
       </c>
       <c r="J22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="M22" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="K22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="L22" s="4" t="n">
+      <c r="N22" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="O22" s="4" t="n">
         <v>19</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="V22" s="4" t="n">
         <v>14</v>
@@ -1917,43 +1917,43 @@
         <v>84</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="M23" s="8" t="n">
         <v>99</v>
       </c>
       <c r="N23" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="Q23" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="O23" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="R23" s="8" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="V23" s="8" t="n">
         <v>105</v>
@@ -2002,7 +2002,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-16</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-17</t>
         </is>
       </c>
     </row>
@@ -2044,72 +2044,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -2138,43 +2138,43 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="M4" s="4" t="n">
+      <c r="N4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="P4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>22</v>
-      </c>
       <c r="Q4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>18</v>
@@ -2205,13 +2205,13 @@
         <v>11</v>
       </c>
       <c r="H5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="I5" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="J5" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>15</v>
@@ -2223,25 +2223,25 @@
         <v>15</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="O5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="Q5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>13</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>14</v>
@@ -2275,7 +2275,7 @@
         <v>2</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>1</v>
@@ -2284,31 +2284,31 @@
         <v>1</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>5</v>
@@ -2345,31 +2345,31 @@
         <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>3</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="M7" s="6" t="inlineStr"/>
       <c r="N7" s="6" t="inlineStr"/>
       <c r="O7" s="6" t="inlineStr"/>
-      <c r="P7" s="6" t="inlineStr"/>
+      <c r="P7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>4</v>
@@ -2400,34 +2400,34 @@
         <v>6</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="L8" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>5</v>
@@ -2471,34 +2471,34 @@
         <v>1</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>5</v>
@@ -2535,7 +2535,7 @@
         <v>3</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>5</v>
@@ -2547,28 +2547,28 @@
         <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>7</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>6</v>
@@ -2602,22 +2602,22 @@
         <v>39</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>41</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="M11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>43</v>
       </c>
       <c r="O11" s="10" t="n">
         <v>44</v>
@@ -2626,16 +2626,16 @@
         <v>44</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="S11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="T11" s="10" t="n">
         <v>48</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>50</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>48</v>
@@ -2666,43 +2666,43 @@
         <v>84</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>99</v>
       </c>
       <c r="M12" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="P12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="N12" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="Q12" s="8" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>105</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-18)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-17</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-18</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -673,46 +673,46 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>11</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -745,16 +745,16 @@
         <v>6</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>6</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>11</v>
@@ -763,25 +763,25 @@
         <v>11</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="R5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="S5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="T5" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>19</v>
@@ -814,49 +814,49 @@
         <v>17</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>13</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="Q6" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="V6" s="4" t="n">
         <v>13</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="V6" s="4" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -888,43 +888,45 @@
       <c r="H7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="J7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L7" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="M7" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -954,7 +956,7 @@
         <v>7</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>6</v>
@@ -963,37 +965,37 @@
         <v>5</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>4</v>
@@ -1025,19 +1027,19 @@
         <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>3</v>
@@ -1046,22 +1048,22 @@
         <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>7</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>3</v>
@@ -1097,25 +1099,25 @@
         <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>1</v>
@@ -1130,13 +1132,13 @@
         <v>1</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1169,46 +1171,46 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="L11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="S11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="M11" s="6" t="n">
+      <c r="T11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="N11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="S11" s="6" t="n">
+      <c r="U11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="V11" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="V11" s="6" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -1239,10 +1241,10 @@
       <c r="I12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="L12" s="4" t="n">
         <v>2</v>
       </c>
@@ -1250,24 +1252,24 @@
         <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="Q12" s="4" t="inlineStr"/>
       <c r="R12" s="4" t="inlineStr"/>
-      <c r="S12" s="4" t="inlineStr"/>
+      <c r="S12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="T12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>4</v>
@@ -1303,34 +1305,34 @@
         <v>3</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>3</v>
@@ -1339,10 +1341,10 @@
         <v>3</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -1375,7 +1377,7 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>1</v>
@@ -1387,16 +1389,16 @@
         <v>1</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>3</v>
@@ -1405,16 +1407,16 @@
         <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -1445,40 +1447,40 @@
         <v>7</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>1</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U15" s="6" t="n">
         <v>7</v>
@@ -1511,9 +1513,11 @@
       <c r="G16" s="4" t="inlineStr"/>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="K16" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L16" s="4" t="n">
         <v>3</v>
@@ -1528,7 +1532,7 @@
         <v>3</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>2</v>
@@ -1537,16 +1541,16 @@
         <v>2</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T16" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
@@ -1603,9 +1607,7 @@
       <c r="Q17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="R17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
@@ -1639,7 +1641,9 @@
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
-      <c r="R18" s="4" t="inlineStr"/>
+      <c r="R18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1673,12 +1677,14 @@
       <c r="I19" s="6" t="inlineStr"/>
       <c r="J19" s="6" t="inlineStr"/>
       <c r="K19" s="6" t="inlineStr"/>
-      <c r="L19" s="6" t="inlineStr"/>
+      <c r="L19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M19" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O19" s="6" t="n">
         <v>2</v>
@@ -1687,7 +1693,7 @@
         <v>2</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R19" s="6" t="n">
         <v>1</v>
@@ -1696,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U19" s="6" t="n">
         <v>1</v>
@@ -1733,27 +1739,29 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="inlineStr"/>
-      <c r="J20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="K20" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>1</v>
@@ -1761,10 +1769,10 @@
       <c r="S20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="T20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U20" s="4" t="inlineStr"/>
+      <c r="T20" s="4" t="inlineStr"/>
+      <c r="U20" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="V20" s="4" t="n">
         <v>2</v>
       </c>
@@ -1793,13 +1801,13 @@
         <v>1</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>1</v>
@@ -1807,23 +1815,23 @@
       <c r="M21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="N21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="N21" s="6" t="inlineStr"/>
       <c r="O21" s="6" t="inlineStr"/>
       <c r="P21" s="6" t="inlineStr"/>
-      <c r="Q21" s="6" t="inlineStr"/>
+      <c r="Q21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>3</v>
@@ -1859,43 +1867,43 @@
         <v>17</v>
       </c>
       <c r="I22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="L22" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="J22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="K22" s="4" t="n">
+      <c r="M22" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="L22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="N22" s="4" t="n">
         <v>19</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="V22" s="4" t="n">
         <v>17</v>
@@ -1927,46 +1935,46 @@
         <v>84</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="L23" s="8" t="n">
         <v>99</v>
       </c>
       <c r="M23" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="P23" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="N23" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="Q23" s="8" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="S23" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -2012,7 +2020,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-17</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-18</t>
         </is>
       </c>
     </row>
@@ -2054,72 +2062,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -2148,46 +2156,46 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>21</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="L4" s="4" t="n">
+      <c r="M4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="O4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="N4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>22</v>
-      </c>
       <c r="P4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
@@ -2215,10 +2223,10 @@
         <v>11</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>15</v>
@@ -2230,28 +2238,28 @@
         <v>15</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="N5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="P5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>13</v>
       </c>
       <c r="S5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>13</v>
@@ -2282,7 +2290,7 @@
         <v>2</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>1</v>
@@ -2291,37 +2299,37 @@
         <v>1</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -2352,31 +2360,31 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>3</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr"/>
       <c r="N7" s="6" t="inlineStr"/>
-      <c r="O7" s="6" t="inlineStr"/>
+      <c r="O7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>4</v>
@@ -2410,31 +2418,31 @@
         <v>6</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="K8" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>5</v>
@@ -2478,34 +2486,34 @@
         <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>5</v>
@@ -2542,7 +2550,7 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>5</v>
@@ -2554,28 +2562,28 @@
         <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>7</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>6</v>
@@ -2609,22 +2617,22 @@
         <v>40</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>41</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="M11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>43</v>
       </c>
       <c r="N11" s="10" t="n">
         <v>44</v>
@@ -2633,19 +2641,19 @@
         <v>44</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="R11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="S11" s="10" t="n">
+      <c r="T11" s="10" t="n">
         <v>50</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>48</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>50</v>
@@ -2676,46 +2684,46 @@
         <v>84</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="K12" s="8" t="n">
         <v>99</v>
       </c>
       <c r="L12" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="O12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="M12" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="P12" s="8" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-19)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-18</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-19</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-18</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-20)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-19</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-19</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-21)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:W23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -522,12 +522,13 @@
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-20</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-21</t>
         </is>
       </c>
     </row>
@@ -642,6 +643,11 @@
           <t>2026-09-18</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -714,6 +720,9 @@
       <c r="V4" s="4" t="n">
         <v>4</v>
       </c>
+      <c r="W4" s="4" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -786,6 +795,9 @@
       <c r="V5" s="6" t="n">
         <v>20</v>
       </c>
+      <c r="W5" s="6" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -858,6 +870,9 @@
       <c r="V6" s="4" t="n">
         <v>17</v>
       </c>
+      <c r="W6" s="4" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -928,6 +943,9 @@
       <c r="V7" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="W7" s="6" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -999,6 +1017,9 @@
       </c>
       <c r="V8" s="4" t="n">
         <v>6</v>
+      </c>
+      <c r="W8" s="4" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -1068,6 +1089,9 @@
       <c r="V9" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="W9" s="6" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1140,6 +1164,9 @@
       <c r="V10" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="W10" s="4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1210,6 +1237,9 @@
         <v>10</v>
       </c>
       <c r="V11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="W11" s="6" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1274,6 +1304,9 @@
       <c r="V12" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="W12" s="4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1346,6 +1379,9 @@
       <c r="V13" s="6" t="n">
         <v>7</v>
       </c>
+      <c r="W13" s="6" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1416,6 +1452,9 @@
         <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="W14" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1486,6 +1525,9 @@
         <v>7</v>
       </c>
       <c r="V15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="W15" s="6" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1550,6 +1592,9 @@
         <v>4</v>
       </c>
       <c r="V16" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="W16" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1612,6 +1657,7 @@
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
+      <c r="W17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1654,6 +1700,7 @@
         <v>1</v>
       </c>
       <c r="V18" s="4" t="inlineStr"/>
+      <c r="W18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1706,6 +1753,7 @@
         <v>1</v>
       </c>
       <c r="V19" s="6" t="inlineStr"/>
+      <c r="W19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1772,6 +1820,9 @@
         <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="W20" s="4" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1834,6 +1885,9 @@
       <c r="V21" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="W21" s="6" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1904,6 +1958,9 @@
         <v>17</v>
       </c>
       <c r="V22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="W22" s="4" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1974,10 +2031,13 @@
       <c r="V23" s="8" t="n">
         <v>101</v>
       </c>
+      <c r="W23" s="8" t="n">
+        <v>101</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A1:W1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1989,7 +2049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2013,12 +2073,13 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-20</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-21</t>
         </is>
       </c>
     </row>
@@ -2128,6 +2189,11 @@
           <t>2026-09-18</t>
         </is>
       </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -2195,6 +2261,9 @@
       <c r="U4" s="4" t="n">
         <v>21</v>
       </c>
+      <c r="V4" s="4" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2262,6 +2331,9 @@
       <c r="U5" s="6" t="n">
         <v>13</v>
       </c>
+      <c r="V5" s="6" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2327,6 +2399,9 @@
         <v>6</v>
       </c>
       <c r="U6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="V6" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -2390,6 +2465,9 @@
       <c r="U7" s="6" t="n">
         <v>4</v>
       </c>
+      <c r="V7" s="6" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -2457,6 +2535,9 @@
       <c r="U8" s="4" t="n">
         <v>6</v>
       </c>
+      <c r="V8" s="4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2522,6 +2603,9 @@
       <c r="U9" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="V9" s="6" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -2589,6 +2673,9 @@
       <c r="U10" s="4" t="n">
         <v>6</v>
       </c>
+      <c r="V10" s="4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -2656,6 +2743,9 @@
       <c r="U11" s="10" t="n">
         <v>41</v>
       </c>
+      <c r="V11" s="10" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -2723,10 +2813,13 @@
       <c r="U12" s="8" t="n">
         <v>101</v>
       </c>
+      <c r="V12" s="8" t="n">
+        <v>101</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A1:V1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-22)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-21</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-22</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -679,49 +679,49 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>11</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="W4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -757,10 +757,10 @@
         <v>6</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>11</v>
@@ -769,34 +769,34 @@
         <v>11</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="R5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="S5" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="T5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="U5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="V5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="U5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>20</v>
-      </c>
       <c r="W5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -829,49 +829,49 @@
         <v>12</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="L6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>12</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>11</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="Q6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="R6" s="4" t="n">
+      <c r="U6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="V6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="W6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="V6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="W6" s="4" t="n">
-        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -904,47 +904,47 @@
         <v>9</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="L7" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>4</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W7" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -977,13 +977,13 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>6</v>
@@ -992,31 +992,31 @@
         <v>6</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="O8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="V8" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>9</v>
@@ -1048,16 +1048,16 @@
         <v>4</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>4</v>
@@ -1066,28 +1066,28 @@
         <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W9" s="6" t="n">
         <v>3</v>
@@ -1123,22 +1123,22 @@
         <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>1</v>
@@ -1153,19 +1153,19 @@
         <v>1</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1198,49 +1198,49 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>9</v>
       </c>
       <c r="K11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="R11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="L11" s="6" t="n">
+      <c r="S11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="M11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="R11" s="6" t="n">
+      <c r="T11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="U11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="V11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="S11" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="V11" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="W11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -1268,10 +1268,10 @@
       </c>
       <c r="G12" s="4" t="inlineStr"/>
       <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="K12" s="4" t="n">
         <v>2</v>
       </c>
@@ -1279,33 +1279,33 @@
         <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="P12" s="4" t="inlineStr"/>
       <c r="Q12" s="4" t="inlineStr"/>
-      <c r="R12" s="4" t="inlineStr"/>
+      <c r="R12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -1338,31 +1338,31 @@
         <v>3</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>3</v>
@@ -1371,13 +1371,13 @@
         <v>3</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="W13" s="6" t="n">
         <v>5</v>
@@ -1422,16 +1422,16 @@
         <v>1</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>3</v>
@@ -1440,22 +1440,22 @@
         <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -1486,43 +1486,43 @@
         <v>7</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M15" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T15" s="6" t="n">
         <v>7</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>4</v>
@@ -1554,9 +1554,11 @@
       </c>
       <c r="G16" s="4" t="inlineStr"/>
       <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="J16" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K16" s="4" t="n">
         <v>3</v>
@@ -1571,7 +1573,7 @@
         <v>3</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>2</v>
@@ -1580,7 +1582,7 @@
         <v>2</v>
       </c>
       <c r="R16" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S16" s="4" t="n">
         <v>4</v>
@@ -1589,10 +1591,10 @@
         <v>4</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V16" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W16" s="4" t="n">
         <v>1</v>
@@ -1649,9 +1651,7 @@
       <c r="P17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
@@ -1686,7 +1686,9 @@
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
-      <c r="Q18" s="4" t="inlineStr"/>
+      <c r="Q18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="R18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1696,9 +1698,7 @@
       <c r="T18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="U18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
       <c r="W18" s="4" t="inlineStr"/>
     </row>
@@ -1721,12 +1721,14 @@
       <c r="H19" s="6" t="inlineStr"/>
       <c r="I19" s="6" t="inlineStr"/>
       <c r="J19" s="6" t="inlineStr"/>
-      <c r="K19" s="6" t="inlineStr"/>
+      <c r="K19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L19" s="6" t="n">
         <v>1</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>2</v>
@@ -1735,7 +1737,7 @@
         <v>2</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>1</v>
@@ -1744,14 +1746,12 @@
         <v>1</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="U19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="U19" s="6" t="inlineStr"/>
       <c r="V19" s="6" t="inlineStr"/>
       <c r="W19" s="6" t="inlineStr"/>
     </row>
@@ -1784,27 +1784,29 @@
       <c r="H20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="J20" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>1</v>
@@ -1812,15 +1814,15 @@
       <c r="R20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="S20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T20" s="4" t="inlineStr"/>
+      <c r="S20" s="4" t="inlineStr"/>
+      <c r="T20" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="U20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>1</v>
@@ -1853,7 +1855,7 @@
         <v>2</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>1</v>
@@ -1861,23 +1863,23 @@
       <c r="L21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="M21" s="6" t="inlineStr"/>
       <c r="N21" s="6" t="inlineStr"/>
       <c r="O21" s="6" t="inlineStr"/>
-      <c r="P21" s="6" t="inlineStr"/>
+      <c r="P21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U21" s="6" t="n">
         <v>3</v>
@@ -1919,49 +1921,49 @@
         <v>17</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="J22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="L22" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="K22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="L22" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="M22" s="4" t="n">
         <v>19</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="T22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="U22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="V22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="W22" s="4" t="n">
         <v>14</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="V22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="W22" s="4" t="n">
-        <v>13</v>
       </c>
     </row>
     <row r="23">
@@ -1990,46 +1992,46 @@
         <v>84</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="K23" s="8" t="n">
         <v>99</v>
       </c>
       <c r="L23" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="O23" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="M23" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="P23" s="8" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="Q23" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="R23" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="S23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="T23" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="U23" s="8" t="n">
         <v>101</v>
       </c>
-      <c r="T23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>108</v>
-      </c>
       <c r="V23" s="8" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>100</v>
@@ -2079,7 +2081,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-21</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-22</t>
         </is>
       </c>
     </row>
@@ -2121,77 +2123,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -2223,43 +2225,43 @@
         <v>21</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="N4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>22</v>
-      </c>
       <c r="O4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="S4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>18</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>21</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>18</v>
@@ -2290,7 +2292,7 @@
         <v>11</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>15</v>
@@ -2302,28 +2304,28 @@
         <v>15</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="O5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>13</v>
       </c>
       <c r="R5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>13</v>
@@ -2332,7 +2334,7 @@
         <v>13</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -2366,37 +2368,37 @@
         <v>1</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>7</v>
@@ -2430,31 +2432,31 @@
         <v>2</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>3</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="K7" s="6" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr"/>
-      <c r="N7" s="6" t="inlineStr"/>
+      <c r="N7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>4</v>
@@ -2497,25 +2499,25 @@
         <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>5</v>
@@ -2530,10 +2532,10 @@
         <v>5</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>7</v>
@@ -2562,34 +2564,34 @@
         <v>1</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>5</v>
@@ -2598,13 +2600,13 @@
         <v>5</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -2641,28 +2643,28 @@
         <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>7</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>6</v>
@@ -2671,10 +2673,10 @@
         <v>6</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -2705,16 +2707,16 @@
         <v>41</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="L11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>43</v>
       </c>
       <c r="M11" s="10" t="n">
         <v>44</v>
@@ -2723,28 +2725,28 @@
         <v>44</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="Q11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="R11" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="R11" s="10" t="n">
+      <c r="S11" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="S11" s="10" t="n">
-        <v>48</v>
-      </c>
       <c r="T11" s="10" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="U11" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="V11" s="10" t="n">
         <v>41</v>
-      </c>
-      <c r="V11" s="10" t="n">
-        <v>42</v>
       </c>
     </row>
     <row r="12">
@@ -2772,46 +2774,46 @@
         <v>84</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="J12" s="8" t="n">
         <v>99</v>
       </c>
       <c r="K12" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="N12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="L12" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="O12" s="8" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="R12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="T12" s="8" t="n">
         <v>101</v>
       </c>
-      <c r="S12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>108</v>
-      </c>
       <c r="U12" s="8" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-23)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-22</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-23</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -679,49 +679,49 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>11</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="L4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="V4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="W4" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="W4" s="4" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -754,10 +754,10 @@
         <v>6</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>11</v>
@@ -766,37 +766,37 @@
         <v>11</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="U5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="V5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="P5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="W5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -829,43 +829,43 @@
         <v>12</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>12</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>11</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="P6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="Q6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="S6" s="4" t="n">
+      <c r="T6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>15</v>
@@ -903,45 +903,45 @@
       <c r="H7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="I7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="K7" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>4</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>4</v>
@@ -977,10 +977,10 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>6</v>
@@ -989,37 +989,37 @@
         <v>6</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="N8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="U8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="O8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="V8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="W8" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="W8" s="4" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -1051,10 +1051,10 @@
         <v>4</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>4</v>
@@ -1063,31 +1063,31 @@
         <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W9" s="6" t="n">
         <v>4</v>
@@ -1123,19 +1123,19 @@
         <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>1</v>
@@ -1150,22 +1150,22 @@
         <v>1</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1201,43 +1201,43 @@
         <v>9</v>
       </c>
       <c r="J11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="K11" s="6" t="n">
+      <c r="R11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="L11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q11" s="6" t="n">
+      <c r="S11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="T11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="U11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="R11" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="V11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>7</v>
@@ -1268,7 +1268,9 @@
       </c>
       <c r="G12" s="4" t="inlineStr"/>
       <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="J12" s="4" t="n">
         <v>2</v>
       </c>
@@ -1276,33 +1278,33 @@
         <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="O12" s="4" t="inlineStr"/>
       <c r="P12" s="4" t="inlineStr"/>
-      <c r="Q12" s="4" t="inlineStr"/>
+      <c r="Q12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="R12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>3</v>
@@ -1338,28 +1340,28 @@
         <v>3</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>3</v>
@@ -1368,13 +1370,13 @@
         <v>3</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>5</v>
@@ -1419,16 +1421,16 @@
         <v>1</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>3</v>
@@ -1437,25 +1439,25 @@
         <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -1486,46 +1488,46 @@
         <v>7</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L15" s="6" t="n">
         <v>1</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S15" s="6" t="n">
         <v>7</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="U15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>3</v>
@@ -1555,7 +1557,7 @@
       <c r="G16" s="4" t="inlineStr"/>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J16" s="4" t="n">
         <v>3</v>
@@ -1570,7 +1572,7 @@
         <v>3</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O16" s="4" t="n">
         <v>2</v>
@@ -1579,7 +1581,7 @@
         <v>2</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R16" s="4" t="n">
         <v>4</v>
@@ -1588,15 +1590,15 @@
         <v>4</v>
       </c>
       <c r="T16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U16" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="V16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="W16" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="V16" s="4" t="inlineStr"/>
+      <c r="W16" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1646,9 +1648,7 @@
       <c r="O17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="P17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
@@ -1683,7 +1683,9 @@
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
-      <c r="P18" s="4" t="inlineStr"/>
+      <c r="P18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1693,9 +1695,7 @@
       <c r="S18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="T18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
       <c r="W18" s="4" t="inlineStr"/>
@@ -1718,12 +1718,14 @@
       <c r="G19" s="6" t="inlineStr"/>
       <c r="H19" s="6" t="inlineStr"/>
       <c r="I19" s="6" t="inlineStr"/>
-      <c r="J19" s="6" t="inlineStr"/>
+      <c r="J19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K19" s="6" t="n">
         <v>1</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M19" s="6" t="n">
         <v>2</v>
@@ -1732,7 +1734,7 @@
         <v>2</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P19" s="6" t="n">
         <v>1</v>
@@ -1741,14 +1743,12 @@
         <v>1</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="T19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="T19" s="6" t="inlineStr"/>
       <c r="U19" s="6" t="inlineStr"/>
       <c r="V19" s="6" t="inlineStr"/>
       <c r="W19" s="6" t="inlineStr"/>
@@ -1783,25 +1783,25 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>1</v>
@@ -1809,19 +1809,17 @@
       <c r="Q20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S20" s="4" t="inlineStr"/>
+      <c r="R20" s="4" t="inlineStr"/>
+      <c r="S20" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="V20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="V20" s="4" t="inlineStr"/>
       <c r="W20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
@@ -1848,7 +1846,7 @@
         <v>1</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>1</v>
@@ -1856,23 +1854,23 @@
       <c r="K21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="L21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr"/>
       <c r="N21" s="6" t="inlineStr"/>
-      <c r="O21" s="6" t="inlineStr"/>
+      <c r="O21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T21" s="6" t="n">
         <v>3</v>
@@ -1881,7 +1879,7 @@
         <v>3</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>4</v>
@@ -1917,49 +1915,49 @@
         <v>17</v>
       </c>
       <c r="I22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="K22" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="J22" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="K22" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="L22" s="4" t="n">
         <v>19</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="Q22" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="S22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="T22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="U22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="V22" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="W22" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="V22" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="W22" s="4" t="n">
-        <v>14</v>
       </c>
     </row>
     <row r="23">
@@ -1988,49 +1986,49 @@
         <v>84</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="J23" s="8" t="n">
         <v>99</v>
       </c>
       <c r="K23" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="N23" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="L23" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="O23" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="T23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="U23" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="V23" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="W23" s="8" t="n">
         <v>99</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="V23" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="W23" s="8" t="n">
-        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -2077,7 +2075,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-22</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-23</t>
         </is>
       </c>
     </row>
@@ -2119,77 +2117,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -2218,43 +2216,43 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="I4" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="J4" s="4" t="n">
+      <c r="K4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="M4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>22</v>
-      </c>
       <c r="N4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="R4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>18</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>21</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>18</v>
@@ -2297,28 +2295,28 @@
         <v>15</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="N5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>13</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>13</v>
@@ -2327,10 +2325,10 @@
         <v>13</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -2361,37 +2359,37 @@
         <v>1</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>7</v>
@@ -2431,25 +2429,25 @@
         <v>3</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="J7" s="6" t="inlineStr"/>
       <c r="K7" s="6" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr"/>
-      <c r="M7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>4</v>
@@ -2461,7 +2459,7 @@
         <v>4</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>3</v>
@@ -2492,25 +2490,25 @@
         <v>6</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>5</v>
@@ -2525,13 +2523,13 @@
         <v>5</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>6</v>
@@ -2563,28 +2561,28 @@
         <v>2</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>5</v>
@@ -2593,10 +2591,10 @@
         <v>5</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>4</v>
@@ -2636,28 +2634,28 @@
         <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>7</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>6</v>
@@ -2666,10 +2664,10 @@
         <v>6</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>6</v>
@@ -2700,16 +2698,16 @@
         <v>40</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="J11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="K11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>43</v>
       </c>
       <c r="L11" s="10" t="n">
         <v>44</v>
@@ -2718,28 +2716,28 @@
         <v>44</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="P11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q11" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="Q11" s="10" t="n">
+      <c r="R11" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="R11" s="10" t="n">
-        <v>48</v>
-      </c>
       <c r="S11" s="10" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>39</v>
@@ -2770,49 +2768,49 @@
         <v>84</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="I12" s="8" t="n">
         <v>99</v>
       </c>
       <c r="J12" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="M12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="K12" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="N12" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="T12" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="U12" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="V12" s="8" t="n">
         <v>99</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="V12" s="8" t="n">
-        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-24)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-23</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-24</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -682,46 +682,46 @@
         <v>11</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>7</v>
       </c>
       <c r="W4" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -754,7 +754,7 @@
         <v>6</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>11</v>
@@ -763,37 +763,37 @@
         <v>11</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="U5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="V5" s="6" t="n">
         <v>12</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>12</v>
@@ -832,43 +832,43 @@
         <v>12</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>12</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>11</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="O6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="P6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="R6" s="4" t="n">
+      <c r="S6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>15</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>14</v>
@@ -903,45 +903,47 @@
       <c r="H7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="J7" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>4</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="S7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="U7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="V7" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="V7" s="6" t="n">
-        <v>4</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>8</v>
@@ -977,7 +979,7 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>6</v>
@@ -986,37 +988,37 @@
         <v>6</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="M8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="N8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="U8" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>8</v>
@@ -1048,10 +1050,10 @@
         <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>3</v>
@@ -1060,37 +1062,37 @@
         <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1126,13 +1128,13 @@
         <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>2</v>
@@ -1147,22 +1149,22 @@
         <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>2</v>
@@ -1198,49 +1200,49 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="P11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="J11" s="6" t="n">
+      <c r="Q11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="K11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="L11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P11" s="6" t="n">
+      <c r="R11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="T11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="Q11" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="U11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="W11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -1275,39 +1277,39 @@
         <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N12" s="4" t="inlineStr"/>
       <c r="O12" s="4" t="inlineStr"/>
-      <c r="P12" s="4" t="inlineStr"/>
+      <c r="P12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -1340,25 +1342,25 @@
         <v>3</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>3</v>
@@ -1367,22 +1369,22 @@
         <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -1418,16 +1420,16 @@
         <v>1</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>3</v>
@@ -1436,28 +1438,28 @@
         <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -1488,46 +1490,46 @@
         <v>7</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K15" s="6" t="n">
         <v>1</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R15" s="6" t="n">
         <v>7</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="T15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>6</v>
@@ -1569,7 +1571,7 @@
         <v>3</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N16" s="4" t="n">
         <v>2</v>
@@ -1578,7 +1580,7 @@
         <v>2</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>4</v>
@@ -1587,14 +1589,12 @@
         <v>4</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T16" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="U16" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
       <c r="W16" s="4" t="inlineStr"/>
     </row>
@@ -1643,9 +1643,7 @@
       <c r="N17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
@@ -1653,7 +1651,9 @@
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
-      <c r="W17" s="6" t="inlineStr"/>
+      <c r="W17" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1680,7 +1680,9 @@
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
-      <c r="O18" s="4" t="inlineStr"/>
+      <c r="O18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1690,9 +1692,7 @@
       <c r="R18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="S18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
@@ -1715,12 +1715,14 @@
       <c r="F19" s="6" t="inlineStr"/>
       <c r="G19" s="6" t="inlineStr"/>
       <c r="H19" s="6" t="inlineStr"/>
-      <c r="I19" s="6" t="inlineStr"/>
+      <c r="I19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J19" s="6" t="n">
         <v>1</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>2</v>
@@ -1729,7 +1731,7 @@
         <v>2</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O19" s="6" t="n">
         <v>1</v>
@@ -1738,14 +1740,12 @@
         <v>1</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="S19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="S19" s="6" t="inlineStr"/>
       <c r="T19" s="6" t="inlineStr"/>
       <c r="U19" s="6" t="inlineStr"/>
       <c r="V19" s="6" t="inlineStr"/>
@@ -1781,22 +1781,22 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>1</v>
@@ -1804,19 +1804,17 @@
       <c r="P20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R20" s="4" t="inlineStr"/>
+      <c r="Q20" s="4" t="inlineStr"/>
+      <c r="R20" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="S20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="U20" s="4" t="inlineStr"/>
       <c r="V20" s="4" t="inlineStr"/>
       <c r="W20" s="4" t="inlineStr"/>
     </row>
@@ -1849,23 +1847,23 @@
       <c r="J21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="K21" s="6" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr"/>
       <c r="M21" s="6" t="inlineStr"/>
-      <c r="N21" s="6" t="inlineStr"/>
+      <c r="N21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S21" s="6" t="n">
         <v>3</v>
@@ -1874,13 +1872,13 @@
         <v>3</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W21" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -1913,49 +1911,49 @@
         <v>17</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K22" s="4" t="n">
         <v>19</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q22" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="S22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="T22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="U22" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="V22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="W22" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="V22" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="W22" s="4" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="23">
@@ -1987,46 +1985,46 @@
         <v>99</v>
       </c>
       <c r="J23" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="M23" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="K23" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="L23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="N23" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="T23" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="U23" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="V23" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="O23" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="V23" s="8" t="n">
+      <c r="W23" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="W23" s="8" t="n">
-        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -2073,7 +2071,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-23</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-24</t>
         </is>
       </c>
     </row>
@@ -2115,77 +2113,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -2214,46 +2212,46 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="L4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>22</v>
-      </c>
       <c r="M4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>16</v>
@@ -2290,28 +2288,28 @@
         <v>15</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="M5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>13</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>13</v>
@@ -2320,10 +2318,10 @@
         <v>13</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>17</v>
@@ -2354,37 +2352,37 @@
         <v>2</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>7</v>
@@ -2396,7 +2394,7 @@
         <v>7</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -2424,25 +2422,25 @@
         <v>2</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="I7" s="6" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr"/>
       <c r="K7" s="6" t="inlineStr"/>
-      <c r="L7" s="6" t="inlineStr"/>
+      <c r="L7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>4</v>
@@ -2454,7 +2452,7 @@
         <v>4</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>3</v>
@@ -2488,43 +2486,43 @@
         <v>6</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="T8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>7</v>
@@ -2556,28 +2554,28 @@
         <v>1</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>5</v>
@@ -2586,16 +2584,16 @@
         <v>5</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>2</v>
@@ -2629,28 +2627,28 @@
         <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>7</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>6</v>
@@ -2659,16 +2657,16 @@
         <v>6</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -2696,13 +2694,13 @@
         <v>40</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="J11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>43</v>
       </c>
       <c r="K11" s="10" t="n">
         <v>44</v>
@@ -2711,31 +2709,31 @@
         <v>44</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="O11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="P11" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="P11" s="10" t="n">
+      <c r="Q11" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="Q11" s="10" t="n">
-        <v>48</v>
-      </c>
       <c r="R11" s="10" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="S11" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="T11" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="U11" s="10" t="n">
         <v>41</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>39</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>41</v>
@@ -2769,46 +2767,46 @@
         <v>99</v>
       </c>
       <c r="I12" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="L12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="J12" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="M12" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="T12" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="U12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="N12" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="U12" s="8" t="n">
+      <c r="V12" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="V12" s="8" t="n">
-        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-25)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-24</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-25</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -679,49 +679,49 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="V4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="W4" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="W4" s="4" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -760,43 +760,43 @@
         <v>11</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="U5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="V5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="W5" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="W5" s="6" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -829,49 +829,49 @@
         <v>12</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>12</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>11</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="N6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="O6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q6" s="4" t="n">
+      <c r="R6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>15</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="W6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -904,49 +904,49 @@
         <v>9</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>4</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="R7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="U7" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="S7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="V7" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="W7" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -985,40 +985,40 @@
         <v>6</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="M8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="T8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="V8" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>8</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>9</v>
@@ -1050,7 +1050,7 @@
         <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>3</v>
@@ -1059,40 +1059,40 @@
         <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1125,13 +1125,13 @@
         <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>2</v>
@@ -1146,28 +1146,28 @@
         <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -1200,46 +1200,46 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="J11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="L11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>7</v>
-      </c>
       <c r="O11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="P11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="P11" s="6" t="n">
-        <v>9</v>
-      </c>
       <c r="Q11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="R11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="T11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>5</v>
@@ -1274,42 +1274,42 @@
         <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M12" s="4" t="inlineStr"/>
       <c r="N12" s="4" t="inlineStr"/>
-      <c r="O12" s="4" t="inlineStr"/>
+      <c r="O12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>5</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1345,19 +1345,19 @@
         <v>6</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>3</v>
@@ -1366,25 +1366,25 @@
         <v>3</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1417,16 +1417,16 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>3</v>
@@ -1435,22 +1435,22 @@
         <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>3</v>
@@ -1459,7 +1459,7 @@
         <v>3</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -1490,46 +1490,46 @@
         <v>7</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>1</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="O15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="V15" s="6" t="n">
         <v>9</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>6</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>9</v>
@@ -1568,7 +1568,7 @@
         <v>3</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M16" s="4" t="n">
         <v>2</v>
@@ -1577,7 +1577,7 @@
         <v>2</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>4</v>
@@ -1586,14 +1586,12 @@
         <v>4</v>
       </c>
       <c r="R16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="T16" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
       <c r="W16" s="4" t="inlineStr"/>
@@ -1640,9 +1638,7 @@
       <c r="M17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="N17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
@@ -1650,7 +1646,9 @@
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
-      <c r="V17" s="6" t="inlineStr"/>
+      <c r="V17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="W17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1679,7 +1677,9 @@
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="inlineStr"/>
+      <c r="N18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1689,13 +1689,13 @@
       <c r="Q18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
-      <c r="V18" s="4" t="inlineStr"/>
+      <c r="V18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="W18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1721,7 +1721,7 @@
         <v>1</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>2</v>
@@ -1730,7 +1730,7 @@
         <v>2</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>1</v>
@@ -1739,14 +1739,12 @@
         <v>1</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="R19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="R19" s="6" t="inlineStr"/>
       <c r="S19" s="6" t="inlineStr"/>
       <c r="T19" s="6" t="inlineStr"/>
       <c r="U19" s="6" t="inlineStr"/>
@@ -1783,19 +1781,19 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>1</v>
@@ -1803,21 +1801,21 @@
       <c r="O20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q20" s="4" t="inlineStr"/>
+      <c r="P20" s="4" t="inlineStr"/>
+      <c r="Q20" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="R20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="T20" s="4" t="inlineStr"/>
       <c r="U20" s="4" t="inlineStr"/>
-      <c r="V20" s="4" t="inlineStr"/>
+      <c r="V20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="W20" s="4" t="n">
         <v>1</v>
       </c>
@@ -1848,23 +1846,23 @@
       <c r="I21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="J21" s="6" t="inlineStr"/>
       <c r="K21" s="6" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr"/>
-      <c r="M21" s="6" t="inlineStr"/>
+      <c r="M21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R21" s="6" t="n">
         <v>3</v>
@@ -1873,13 +1871,13 @@
         <v>3</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>2</v>
@@ -1915,43 +1913,43 @@
         <v>17</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J22" s="4" t="n">
         <v>19</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Q22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="S22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="T22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="R22" s="4" t="n">
+      <c r="U22" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>14</v>
       </c>
       <c r="V22" s="4" t="n">
         <v>17</v>
@@ -1986,46 +1984,46 @@
         <v>84</v>
       </c>
       <c r="I23" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="L23" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="J23" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="K23" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="L23" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="M23" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="T23" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="U23" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="N23" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>97</v>
-      </c>
       <c r="V23" s="8" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>103</v>
@@ -2075,7 +2073,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-24</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-25</t>
         </is>
       </c>
     </row>
@@ -2117,77 +2115,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -2216,46 +2214,46 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>22</v>
-      </c>
       <c r="L4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="T4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>16</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>17</v>
@@ -2289,28 +2287,28 @@
         <v>15</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="L5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>13</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>13</v>
@@ -2319,16 +2317,16 @@
         <v>13</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
@@ -2359,31 +2357,31 @@
         <v>2</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>7</v>
@@ -2395,7 +2393,7 @@
         <v>7</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>6</v>
@@ -2425,23 +2423,23 @@
       <c r="G7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>4</v>
@@ -2453,7 +2451,7 @@
         <v>4</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>3</v>
@@ -2490,19 +2488,19 @@
         <v>6</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>5</v>
@@ -2517,13 +2515,13 @@
         <v>5</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>7</v>
@@ -2532,7 +2530,7 @@
         <v>7</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -2558,25 +2556,25 @@
         <v>1</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>5</v>
@@ -2585,19 +2583,19 @@
         <v>5</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>3</v>
@@ -2628,28 +2626,28 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>7</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>6</v>
@@ -2658,16 +2656,16 @@
         <v>6</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>5</v>
@@ -2698,10 +2696,10 @@
         <v>40</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="I11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="I11" s="10" t="n">
-        <v>43</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>44</v>
@@ -2710,34 +2708,34 @@
         <v>44</v>
       </c>
       <c r="L11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>41</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="S11" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="T11" s="10" t="n">
+        <v>41</v>
+      </c>
+      <c r="U11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>41</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>39</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>41</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>44</v>
@@ -2768,46 +2766,46 @@
         <v>84</v>
       </c>
       <c r="H12" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="K12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="L12" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="T12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="M12" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>97</v>
-      </c>
       <c r="U12" s="8" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>103</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-26)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-25</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-26</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-25</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-27)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-26</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-27</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-26</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-28)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-27</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-28</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -679,49 +679,49 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>7</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W4" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -757,46 +757,46 @@
         <v>11</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="U5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="V5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="K5" s="6" t="n">
+      <c r="W5" s="6" t="n">
         <v>12</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="W5" s="6" t="n">
-        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -829,49 +829,49 @@
         <v>12</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="M6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="N6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="P6" s="4" t="n">
+      <c r="Q6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>15</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="W6" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -907,46 +907,46 @@
         <v>5</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="Q7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="T7" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="R7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="U7" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="W7" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -982,43 +982,43 @@
         <v>6</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="L8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="S8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="U8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="T8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="U8" s="4" t="n">
+      <c r="V8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="W8" s="4" t="n">
         <v>8</v>
@@ -1056,34 +1056,34 @@
         <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>3</v>
@@ -1125,10 +1125,10 @@
         <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>2</v>
@@ -1143,22 +1143,22 @@
         <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>2</v>
@@ -1167,7 +1167,7 @@
         <v>2</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1206,43 +1206,43 @@
         <v>5</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="O11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="O11" s="6" t="n">
-        <v>9</v>
-      </c>
       <c r="P11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="R11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="Q11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="S11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>5</v>
       </c>
       <c r="W11" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -1271,36 +1271,36 @@
       <c r="G12" s="4" t="inlineStr"/>
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="L12" s="4" t="inlineStr"/>
       <c r="M12" s="4" t="inlineStr"/>
-      <c r="N12" s="4" t="inlineStr"/>
+      <c r="N12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U12" s="4" t="n">
         <v>5</v>
@@ -1309,7 +1309,7 @@
         <v>5</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -1342,19 +1342,19 @@
         <v>3</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>3</v>
@@ -1363,28 +1363,28 @@
         <v>3</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1420,10 +1420,10 @@
         <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>3</v>
@@ -1432,22 +1432,22 @@
         <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>3</v>
@@ -1459,7 +1459,7 @@
         <v>3</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -1493,46 +1493,46 @@
         <v>1</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="O15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="V15" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="W15" s="6" t="n">
         <v>9</v>
-      </c>
-      <c r="W15" s="6" t="n">
-        <v>13</v>
       </c>
     </row>
     <row r="16">
@@ -1565,7 +1565,7 @@
         <v>3</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L16" s="4" t="n">
         <v>2</v>
@@ -1574,7 +1574,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O16" s="4" t="n">
         <v>4</v>
@@ -1583,14 +1583,12 @@
         <v>4</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R16" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="S16" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
@@ -1635,9 +1633,7 @@
       <c r="L17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="M17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
@@ -1645,7 +1641,9 @@
       <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
-      <c r="U17" s="6" t="inlineStr"/>
+      <c r="U17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1676,7 +1674,9 @@
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1686,16 +1686,14 @@
       <c r="P18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
-      <c r="U18" s="4" t="inlineStr"/>
-      <c r="V18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="U18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V18" s="4" t="inlineStr"/>
       <c r="W18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1716,7 +1714,7 @@
       <c r="G19" s="6" t="inlineStr"/>
       <c r="H19" s="6" t="inlineStr"/>
       <c r="I19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>2</v>
@@ -1725,7 +1723,7 @@
         <v>2</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M19" s="6" t="n">
         <v>1</v>
@@ -1734,14 +1732,12 @@
         <v>1</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="Q19" s="6" t="inlineStr"/>
       <c r="R19" s="6" t="inlineStr"/>
       <c r="S19" s="6" t="inlineStr"/>
       <c r="T19" s="6" t="inlineStr"/>
@@ -1779,16 +1775,16 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M20" s="4" t="n">
         <v>1</v>
@@ -1796,26 +1792,26 @@
       <c r="N20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="O20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P20" s="4" t="inlineStr"/>
+      <c r="O20" s="4" t="inlineStr"/>
+      <c r="P20" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="Q20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="S20" s="4" t="inlineStr"/>
       <c r="T20" s="4" t="inlineStr"/>
-      <c r="U20" s="4" t="inlineStr"/>
+      <c r="U20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -1841,23 +1837,23 @@
       <c r="H21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I21" s="6" t="inlineStr"/>
       <c r="J21" s="6" t="inlineStr"/>
       <c r="K21" s="6" t="inlineStr"/>
-      <c r="L21" s="6" t="inlineStr"/>
+      <c r="L21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>3</v>
@@ -1866,19 +1862,19 @@
         <v>3</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W21" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1914,46 +1910,46 @@
         <v>19</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="P22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="S22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="Q22" s="4" t="n">
+      <c r="T22" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>14</v>
       </c>
       <c r="U22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="W22" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23">
@@ -1982,49 +1978,49 @@
         <v>84</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="K23" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="T23" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="U23" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="V23" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="W23" s="8" t="n">
         <v>98</v>
-      </c>
-      <c r="L23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="V23" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="W23" s="8" t="n">
-        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2071,7 +2067,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-27</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-28</t>
         </is>
       </c>
     </row>
@@ -2113,77 +2109,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -2212,46 +2208,46 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="I4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>22</v>
-      </c>
       <c r="K4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="S4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="T4" s="4" t="n">
-        <v>16</v>
-      </c>
       <c r="U4" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>20</v>
@@ -2282,28 +2278,28 @@
         <v>11</v>
       </c>
       <c r="H5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="I5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>16</v>
-      </c>
       <c r="K5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>13</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>13</v>
@@ -2312,19 +2308,19 @@
         <v>13</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -2352,31 +2348,31 @@
         <v>2</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>7</v>
@@ -2388,13 +2384,13 @@
         <v>7</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -2423,18 +2419,20 @@
       </c>
       <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>4</v>
@@ -2446,7 +2444,7 @@
         <v>4</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>3</v>
@@ -2458,7 +2456,7 @@
         <v>3</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -2486,16 +2484,16 @@
         <v>6</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>5</v>
@@ -2510,13 +2508,13 @@
         <v>5</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>7</v>
@@ -2525,7 +2523,7 @@
         <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>6</v>
@@ -2554,22 +2552,22 @@
         <v>1</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>5</v>
@@ -2578,19 +2576,19 @@
         <v>5</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>3</v>
@@ -2624,25 +2622,25 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>7</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>6</v>
@@ -2651,16 +2649,16 @@
         <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>5</v>
@@ -2694,7 +2692,7 @@
         <v>40</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>44</v>
@@ -2703,40 +2701,40 @@
         <v>44</v>
       </c>
       <c r="K11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>41</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="S11" s="10" t="n">
+        <v>41</v>
+      </c>
+      <c r="T11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="L11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q11" s="10" t="n">
+      <c r="U11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="V11" s="10" t="n">
         <v>41</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>39</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>41</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="V11" s="10" t="n">
-        <v>46</v>
       </c>
     </row>
     <row r="12">
@@ -2764,49 +2762,49 @@
         <v>84</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="J12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="T12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="U12" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="V12" s="8" t="n">
         <v>98</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="V12" s="8" t="n">
-        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-29)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-28</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-29</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -682,46 +682,46 @@
         <v>6</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="R4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="V4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="S4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="W4" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -754,49 +754,49 @@
         <v>6</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>11</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>10</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="W5" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -829,49 +829,49 @@
         <v>12</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="L6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="O6" s="4" t="n">
+      <c r="P6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>15</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>9</v>
       </c>
       <c r="W6" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -904,49 +904,49 @@
         <v>9</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="P7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="S7" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="Q7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="T7" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>15</v>
       </c>
       <c r="W7" s="6" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -979,49 +979,49 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="Q8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="K8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="R8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="S8" s="4" t="n">
+      <c r="U8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="V8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="T8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="W8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -1053,34 +1053,34 @@
         <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>3</v>
@@ -1092,7 +1092,7 @@
         <v>3</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1125,7 +1125,7 @@
         <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>2</v>
@@ -1140,22 +1140,22 @@
         <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>2</v>
@@ -1164,10 +1164,10 @@
         <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1203,37 +1203,37 @@
         <v>5</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="N11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="N11" s="6" t="n">
-        <v>9</v>
-      </c>
       <c r="O11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="P11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="R11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>5</v>
@@ -1274,30 +1274,30 @@
         <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K12" s="4" t="inlineStr"/>
       <c r="L12" s="4" t="inlineStr"/>
-      <c r="M12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>5</v>
@@ -1306,10 +1306,10 @@
         <v>5</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1345,13 +1345,13 @@
         <v>7</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>3</v>
@@ -1360,31 +1360,31 @@
         <v>3</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1417,10 +1417,10 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>3</v>
@@ -1429,22 +1429,22 @@
         <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>3</v>
@@ -1456,10 +1456,10 @@
         <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -1490,46 +1490,46 @@
         <v>7</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="M15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="N15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="U15" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>3</v>
@@ -1562,7 +1562,7 @@
         <v>3</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K16" s="4" t="n">
         <v>2</v>
@@ -1571,7 +1571,7 @@
         <v>2</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N16" s="4" t="n">
         <v>4</v>
@@ -1580,14 +1580,12 @@
         <v>4</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R16" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
@@ -1630,9 +1628,7 @@
       <c r="K17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="L17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
@@ -1640,7 +1636,9 @@
       <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
-      <c r="T17" s="6" t="inlineStr"/>
+      <c r="T17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1673,7 +1671,9 @@
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="inlineStr"/>
+      <c r="L18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1683,16 +1683,14 @@
       <c r="O18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
-      <c r="T18" s="4" t="inlineStr"/>
-      <c r="U18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="T18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
       <c r="W18" s="4" t="inlineStr"/>
     </row>
@@ -1720,7 +1718,7 @@
         <v>2</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>1</v>
@@ -1729,14 +1727,12 @@
         <v>1</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="P19" s="6" t="inlineStr"/>
       <c r="Q19" s="6" t="inlineStr"/>
       <c r="R19" s="6" t="inlineStr"/>
       <c r="S19" s="6" t="inlineStr"/>
@@ -1775,13 +1771,13 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L20" s="4" t="n">
         <v>1</v>
@@ -1789,26 +1785,26 @@
       <c r="M20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O20" s="4" t="inlineStr"/>
+      <c r="N20" s="4" t="inlineStr"/>
+      <c r="O20" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="P20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="R20" s="4" t="inlineStr"/>
       <c r="S20" s="4" t="inlineStr"/>
-      <c r="T20" s="4" t="inlineStr"/>
+      <c r="T20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="U20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W20" s="4" t="n">
         <v>4</v>
@@ -1839,18 +1835,20 @@
       </c>
       <c r="I21" s="6" t="inlineStr"/>
       <c r="J21" s="6" t="inlineStr"/>
-      <c r="K21" s="6" t="inlineStr"/>
+      <c r="K21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P21" s="6" t="n">
         <v>3</v>
@@ -1859,19 +1857,19 @@
         <v>3</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>1</v>
@@ -1907,49 +1905,49 @@
         <v>17</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="O22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="R22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="P22" s="4" t="n">
+      <c r="S22" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>14</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="W22" s="4" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23">
@@ -1978,49 +1976,49 @@
         <v>84</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K23" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="S23" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="L23" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>97</v>
-      </c>
       <c r="T23" s="8" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="W23" s="8" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -2067,7 +2065,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-28</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-29</t>
         </is>
       </c>
     </row>
@@ -2109,77 +2107,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -2208,49 +2206,49 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="S4" s="4" t="n">
-        <v>16</v>
-      </c>
       <c r="T4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="V4" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -2278,25 +2276,25 @@
         <v>11</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>13</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>13</v>
@@ -2305,22 +2303,22 @@
         <v>13</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -2348,46 +2346,46 @@
         <v>2</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="K6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="O6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="P6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="T6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>5</v>
@@ -2418,18 +2416,20 @@
         <v>2</v>
       </c>
       <c r="H7" s="6" t="inlineStr"/>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>4</v>
@@ -2441,7 +2441,7 @@
         <v>4</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>3</v>
@@ -2453,7 +2453,7 @@
         <v>3</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>2</v>
@@ -2484,46 +2484,46 @@
         <v>6</v>
       </c>
       <c r="H8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="U8" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>3</v>
@@ -2555,16 +2555,16 @@
         <v>2</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>5</v>
@@ -2573,25 +2573,25 @@
         <v>5</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>2</v>
@@ -2625,19 +2625,19 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>6</v>
@@ -2646,22 +2646,22 @@
         <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q10" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="S10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="U10" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>6</v>
@@ -2698,43 +2698,43 @@
         <v>44</v>
       </c>
       <c r="J11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>41</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>41</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>41</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="R11" s="10" t="n">
+      <c r="T11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="U11" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="V11" s="10" t="n">
         <v>39</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>41</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="V11" s="10" t="n">
-        <v>40</v>
       </c>
     </row>
     <row r="12">
@@ -2762,49 +2762,49 @@
         <v>84</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J12" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="R12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="K12" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>97</v>
-      </c>
       <c r="S12" s="8" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="V12" s="8" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-09-30)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-29</t>
+          <t>Evolución abiertas SAT por estado — 2026-09-30</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -679,46 +679,46 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>7</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>7</v>
@@ -754,49 +754,49 @@
         <v>6</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="S5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="W5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -829,49 +829,49 @@
         <v>12</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="N6" s="4" t="n">
+      <c r="O6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>15</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>9</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -904,49 +904,49 @@
         <v>9</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>4</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="O7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="R7" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="P7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="S7" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>15</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="W7" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -979,49 +979,49 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>6</v>
-      </c>
       <c r="Q8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="R8" s="4" t="n">
+      <c r="T8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="U8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="S8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="T8" s="4" t="n">
+      <c r="V8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="W8" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="W8" s="4" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -1050,34 +1050,34 @@
         <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>3</v>
@@ -1089,10 +1089,10 @@
         <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1137,22 +1137,22 @@
         <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>2</v>
@@ -1161,13 +1161,13 @@
         <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -1200,37 +1200,37 @@
         <v>8</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="M11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="M11" s="6" t="n">
-        <v>9</v>
-      </c>
       <c r="N11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="P11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="O11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="Q11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>5</v>
@@ -1271,30 +1271,30 @@
       <c r="G12" s="4" t="inlineStr"/>
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J12" s="4" t="inlineStr"/>
       <c r="K12" s="4" t="inlineStr"/>
-      <c r="L12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S12" s="4" t="n">
         <v>5</v>
@@ -1303,13 +1303,13 @@
         <v>5</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1342,13 +1342,13 @@
         <v>3</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>3</v>
@@ -1357,34 +1357,34 @@
         <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1417,7 +1417,7 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>3</v>
@@ -1426,22 +1426,22 @@
         <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>3</v>
@@ -1453,13 +1453,13 @@
         <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -1493,43 +1493,43 @@
         <v>4</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="L15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S15" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="M15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="T15" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>7</v>
@@ -1559,7 +1559,7 @@
       <c r="G16" s="4" t="inlineStr"/>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J16" s="4" t="n">
         <v>2</v>
@@ -1568,7 +1568,7 @@
         <v>2</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M16" s="4" t="n">
         <v>4</v>
@@ -1577,20 +1577,20 @@
         <v>4</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q16" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
-      <c r="W16" s="4" t="inlineStr"/>
+      <c r="W16" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1625,9 +1625,7 @@
       <c r="J17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="K17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
@@ -1635,7 +1633,9 @@
       <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
       <c r="R17" s="6" t="inlineStr"/>
-      <c r="S17" s="6" t="inlineStr"/>
+      <c r="S17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1646,7 +1646,7 @@
         <v>1</v>
       </c>
       <c r="W17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -1670,7 +1670,9 @@
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="4" t="inlineStr"/>
+      <c r="K18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1680,16 +1682,14 @@
       <c r="N18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="O18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
-      <c r="S18" s="4" t="inlineStr"/>
-      <c r="T18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="S18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
       <c r="W18" s="4" t="inlineStr"/>
@@ -1715,7 +1715,7 @@
         <v>2</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>1</v>
@@ -1724,14 +1724,12 @@
         <v>1</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="O19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="O19" s="6" t="inlineStr"/>
       <c r="P19" s="6" t="inlineStr"/>
       <c r="Q19" s="6" t="inlineStr"/>
       <c r="R19" s="6" t="inlineStr"/>
@@ -1771,10 +1769,10 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>1</v>
@@ -1782,26 +1780,26 @@
       <c r="L20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="M20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="inlineStr"/>
+      <c r="N20" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="O20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="Q20" s="4" t="inlineStr"/>
       <c r="R20" s="4" t="inlineStr"/>
-      <c r="S20" s="4" t="inlineStr"/>
+      <c r="S20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="T20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>4</v>
@@ -1834,18 +1832,20 @@
         <v>1</v>
       </c>
       <c r="I21" s="6" t="inlineStr"/>
-      <c r="J21" s="6" t="inlineStr"/>
+      <c r="J21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O21" s="6" t="n">
         <v>3</v>
@@ -1854,19 +1854,19 @@
         <v>3</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>1</v>
@@ -1905,49 +1905,49 @@
         <v>17</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="N22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="O22" s="4" t="n">
+      <c r="R22" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>14</v>
       </c>
       <c r="S22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="V22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="W22" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23">
@@ -1976,46 +1976,46 @@
         <v>84</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J23" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="R23" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="K23" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="L23" s="8" t="n">
+      <c r="S23" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="T23" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="U23" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="V23" s="8" t="n">
         <v>95</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="V23" s="8" t="n">
-        <v>91</v>
       </c>
       <c r="W23" s="8" t="n">
         <v>95</v>
@@ -2065,7 +2065,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-29</t>
+          <t>Evolución abiertas SAT por cadena — 2026-09-30</t>
         </is>
       </c>
     </row>
@@ -2107,77 +2107,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -2206,49 +2206,49 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="S4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="V4" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -2276,22 +2276,22 @@
         <v>11</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>13</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>13</v>
@@ -2300,25 +2300,25 @@
         <v>13</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="U5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="V5" s="6" t="n">
         <v>18</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -2346,25 +2346,25 @@
         <v>2</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>7</v>
@@ -2376,16 +2376,16 @@
         <v>7</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>6</v>
@@ -2415,18 +2415,20 @@
       <c r="G7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="I7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>4</v>
@@ -2438,7 +2440,7 @@
         <v>4</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>3</v>
@@ -2450,7 +2452,7 @@
         <v>3</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>2</v>
@@ -2484,10 +2486,10 @@
         <v>6</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>5</v>
@@ -2502,13 +2504,13 @@
         <v>5</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>7</v>
@@ -2517,16 +2519,16 @@
         <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -2552,16 +2554,16 @@
         <v>1</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>5</v>
@@ -2570,28 +2572,28 @@
         <v>5</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>3</v>
@@ -2622,19 +2624,19 @@
         <v>4</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>6</v>
@@ -2643,28 +2645,28 @@
         <v>6</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -2695,46 +2697,46 @@
         <v>44</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>41</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>41</v>
+      </c>
+      <c r="R11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>41</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>39</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>41</v>
-      </c>
       <c r="S11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>40</v>
       </c>
       <c r="V11" s="10" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12">
@@ -2762,46 +2764,46 @@
         <v>84</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I12" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="Q12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="J12" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="K12" s="8" t="n">
+      <c r="R12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="T12" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="U12" s="8" t="n">
         <v>95</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>91</v>
       </c>
       <c r="V12" s="8" t="n">
         <v>95</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-01)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W23"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -522,13 +522,12 @@
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-09-30</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-01</t>
         </is>
       </c>
     </row>
@@ -545,107 +544,102 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="W3" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -664,64 +658,61 @@
         <v>10</v>
       </c>
       <c r="D4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="V4" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="W4" s="4" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -736,68 +727,65 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="D5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>18</v>
-      </c>
       <c r="Q5" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="W5" s="6" t="n">
-        <v>13</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -811,67 +799,64 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="K6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="M6" s="4" t="n">
+      <c r="N6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>15</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>9</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="W6" s="4" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -886,67 +871,64 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="K7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="I7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="L7" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="N7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q7" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="O7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="R7" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>15</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="W7" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -961,67 +943,64 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="V8" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="W8" s="4" t="n">
-        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -1036,45 +1015,45 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E9" s="6" t="inlineStr"/>
       <c r="F9" s="6" t="inlineStr"/>
-      <c r="G9" s="6" t="inlineStr"/>
+      <c r="G9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="H9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>3</v>
@@ -1086,12 +1065,9 @@
         <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="W9" s="6" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1107,10 +1083,10 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>3</v>
@@ -1119,10 +1095,10 @@
         <v>3</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>2</v>
@@ -1134,22 +1110,22 @@
         <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>2</v>
@@ -1158,16 +1134,13 @@
         <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="W10" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1182,52 +1155,52 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="G11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="H11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K11" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="L11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="I11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="J11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="K11" s="6" t="n">
+      <c r="M11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="L11" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="P11" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>5</v>
@@ -1239,9 +1212,6 @@
         <v>5</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="W11" s="6" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1257,41 +1227,41 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="F12" s="4" t="inlineStr"/>
       <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="4" t="inlineStr"/>
       <c r="J12" s="4" t="inlineStr"/>
-      <c r="K12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>5</v>
@@ -1300,16 +1270,13 @@
         <v>5</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="W12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1330,22 +1297,22 @@
         <v>1</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
         <v>6</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>3</v>
@@ -1354,37 +1321,34 @@
         <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>3</v>
-      </c>
-      <c r="W13" s="6" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1399,16 +1363,16 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E14" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>2</v>
@@ -1423,22 +1387,22 @@
         <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>3</v>
@@ -1450,16 +1414,13 @@
         <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="W14" s="4" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15">
@@ -1473,65 +1434,64 @@
           <t>Devuelto a cliente</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr"/>
+      <c r="C15" s="6" t="n">
+        <v>13</v>
+      </c>
       <c r="D15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="S15" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="E15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="H15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="I15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="J15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>9</v>
-      </c>
       <c r="T15" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="W15" s="6" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1547,17 +1507,17 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="4" t="inlineStr"/>
-      <c r="F16" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="4" t="inlineStr"/>
-      <c r="H16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I16" s="4" t="n">
         <v>2</v>
       </c>
@@ -1565,7 +1525,7 @@
         <v>2</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L16" s="4" t="n">
         <v>4</v>
@@ -1574,21 +1534,18 @@
         <v>4</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P16" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
-      <c r="V16" s="4" t="inlineStr"/>
-      <c r="W16" s="4" t="n">
+      <c r="V16" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1604,7 +1561,7 @@
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D17" s="6" t="n">
         <v>1</v>
@@ -1612,19 +1569,17 @@
       <c r="E17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" s="6" t="inlineStr"/>
+      <c r="F17" s="6" t="inlineStr"/>
+      <c r="G17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H17" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
@@ -1632,7 +1587,9 @@
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
       <c r="Q17" s="6" t="inlineStr"/>
-      <c r="R17" s="6" t="inlineStr"/>
+      <c r="R17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="S17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1643,9 +1600,6 @@
         <v>1</v>
       </c>
       <c r="V17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="W17" s="6" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1660,16 +1614,16 @@
           <t>En reparación (online)</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="C18" s="4" t="inlineStr"/>
       <c r="D18" s="4" t="inlineStr"/>
       <c r="E18" s="4" t="inlineStr"/>
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" s="4" t="inlineStr"/>
+      <c r="J18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1679,20 +1633,17 @@
       <c r="M18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
-      <c r="R18" s="4" t="inlineStr"/>
-      <c r="S18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="R18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
-      <c r="W18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1712,7 +1663,7 @@
       <c r="G19" s="6" t="inlineStr"/>
       <c r="H19" s="6" t="inlineStr"/>
       <c r="I19" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>1</v>
@@ -1721,14 +1672,12 @@
         <v>1</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N19" s="6" t="inlineStr"/>
       <c r="O19" s="6" t="inlineStr"/>
       <c r="P19" s="6" t="inlineStr"/>
       <c r="Q19" s="6" t="inlineStr"/>
@@ -1737,7 +1686,6 @@
       <c r="T19" s="6" t="inlineStr"/>
       <c r="U19" s="6" t="inlineStr"/>
       <c r="V19" s="6" t="inlineStr"/>
-      <c r="W19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1751,25 +1699,25 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>1</v>
@@ -1777,34 +1725,31 @@
       <c r="K20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="N20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="P20" s="4" t="inlineStr"/>
       <c r="Q20" s="4" t="inlineStr"/>
-      <c r="R20" s="4" t="inlineStr"/>
+      <c r="R20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="W20" s="4" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1819,30 +1764,32 @@
           <t>Esperando respuesta cliente a presupuesto</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="C21" s="6" t="inlineStr"/>
       <c r="D21" s="6" t="inlineStr"/>
       <c r="E21" s="6" t="inlineStr"/>
-      <c r="F21" s="6" t="inlineStr"/>
+      <c r="F21" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="G21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I21" s="6" t="inlineStr"/>
+      <c r="I21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>3</v>
@@ -1851,27 +1798,24 @@
         <v>3</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U21" s="6" t="n">
         <v>1</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="W21" s="6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1887,67 +1831,64 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="J22" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="D22" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="E22" s="4" t="n">
+      <c r="K22" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="L22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="F22" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="G22" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="H22" s="4" t="n">
+      <c r="M22" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="I22" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="J22" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="K22" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="L22" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="M22" s="4" t="n">
+      <c r="N22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="P22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="N22" s="4" t="n">
+      <c r="Q22" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>14</v>
       </c>
       <c r="R22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="U22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="W22" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
@@ -1958,72 +1899,69 @@
         </is>
       </c>
       <c r="C23" s="8" t="n">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>129</v>
+        <v>96</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="I23" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="Q23" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="J23" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="K23" s="8" t="n">
+      <c r="R23" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="T23" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="U23" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="L23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="S23" s="8" t="n">
+      <c r="V23" s="8" t="n">
         <v>103</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="V23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="W23" s="8" t="n">
-        <v>100</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:W1"/>
+    <mergeCell ref="A1:V1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2035,7 +1973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2059,13 +1997,12 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-09-30</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-01</t>
         </is>
       </c>
     </row>
@@ -2077,107 +2014,102 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="V3" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -2188,67 +2120,64 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E4" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="F4" s="4" t="n">
         <v>18</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>13</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="P4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="Q4" s="4" t="n">
-        <v>16</v>
-      </c>
       <c r="R4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="S4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>18</v>
-      </c>
       <c r="U4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -2258,37 +2187,37 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F5" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="C5" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="G5" s="6" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>13</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>13</v>
@@ -2297,27 +2226,24 @@
         <v>13</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="V5" s="6" t="n">
         <v>19</v>
       </c>
     </row>
@@ -2331,64 +2257,61 @@
         <v>6</v>
       </c>
       <c r="C6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="D6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="H6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="I6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="M6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="N6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="R6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="S6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="U6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="V6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -2398,7 +2321,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -2410,22 +2333,22 @@
         <v>1</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>4</v>
@@ -2437,7 +2360,7 @@
         <v>4</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>3</v>
@@ -2449,15 +2372,12 @@
         <v>3</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>2</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="V7" s="6" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2468,66 +2388,63 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C8" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="G8" s="4" t="n">
+      <c r="O8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R8" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="S8" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="V8" s="4" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2541,26 +2458,26 @@
         <v>1</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E9" s="6" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="D9" s="6" t="inlineStr"/>
+      <c r="E9" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="F9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>5</v>
@@ -2569,34 +2486,31 @@
         <v>5</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>3</v>
-      </c>
-      <c r="V9" s="6" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -2606,34 +2520,34 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>4</v>
-      </c>
       <c r="H10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>6</v>
@@ -2642,30 +2556,27 @@
         <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O10" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="R10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="T10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="V10" s="4" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2676,67 +2587,64 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="C11" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="I11" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="D11" s="10" t="n">
-        <v>32</v>
-      </c>
-      <c r="E11" s="10" t="n">
-        <v>35</v>
-      </c>
-      <c r="F11" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="G11" s="10" t="n">
+      <c r="J11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>41</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>41</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>40</v>
-      </c>
-      <c r="H11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="I11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>48</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>41</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>39</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>41</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>46</v>
       </c>
       <c r="T11" s="10" t="n">
         <v>40</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>40</v>
-      </c>
-      <c r="V11" s="10" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12">
@@ -2746,72 +2654,69 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>129</v>
+        <v>96</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="G12" s="8" t="n">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="P12" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>94</v>
-      </c>
-      <c r="J12" s="8" t="n">
+      <c r="Q12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="T12" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="K12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="R12" s="8" t="n">
+      <c r="U12" s="8" t="n">
         <v>103</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="V12" s="8" t="n">
-        <v>100</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A1:U1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-02)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-01</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -673,40 +673,40 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="T4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>7</v>
@@ -745,43 +745,43 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>15</v>
-      </c>
       <c r="K5" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>20</v>
-      </c>
       <c r="O5" s="6" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>17</v>
@@ -817,46 +817,46 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="J6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="L6" s="4" t="n">
+      <c r="M6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>15</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>9</v>
       </c>
       <c r="T6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="U6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="V6" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -892,43 +892,43 @@
         <v>4</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="M7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P7" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="N7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="Q7" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>15</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -961,46 +961,46 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="O8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="P8" s="4" t="n">
+      <c r="R8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="T8" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1029,28 +1029,28 @@
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>3</v>
@@ -1062,10 +1062,10 @@
         <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>5</v>
@@ -1107,22 +1107,22 @@
         <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>2</v>
@@ -1131,16 +1131,16 @@
         <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -1173,46 +1173,46 @@
         <v>5</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="K11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="K11" s="6" t="n">
-        <v>9</v>
-      </c>
       <c r="L11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="N11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="M11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="N11" s="6" t="n">
+      <c r="O11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="T11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="U11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="V11" s="6" t="n">
         <v>6</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="V11" s="6" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -1241,24 +1241,26 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="inlineStr"/>
-      <c r="J12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>5</v>
@@ -1267,10 +1269,10 @@
         <v>5</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
         <v>2</v>
@@ -1309,7 +1311,7 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>3</v>
@@ -1318,34 +1320,34 @@
         <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>4</v>
@@ -1384,22 +1386,22 @@
         <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>3</v>
@@ -1411,7 +1413,7 @@
         <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>2</v>
@@ -1453,43 +1455,43 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="K15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="R15" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>12</v>
@@ -1522,7 +1524,7 @@
         <v>2</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K16" s="4" t="n">
         <v>4</v>
@@ -1531,14 +1533,12 @@
         <v>4</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O16" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
@@ -1574,9 +1574,7 @@
       <c r="H17" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I17" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
@@ -1584,7 +1582,9 @@
       <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
       <c r="P17" s="6" t="inlineStr"/>
-      <c r="Q17" s="6" t="inlineStr"/>
+      <c r="Q17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="R17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1595,7 +1595,7 @@
         <v>1</v>
       </c>
       <c r="U17" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V17" s="6" t="n">
         <v>3</v>
@@ -1618,7 +1618,9 @@
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="inlineStr"/>
+      <c r="I18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1628,16 +1630,14 @@
       <c r="L18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="M18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
-      <c r="Q18" s="4" t="inlineStr"/>
-      <c r="R18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
@@ -1667,14 +1667,12 @@
         <v>1</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="M19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M19" s="6" t="inlineStr"/>
       <c r="N19" s="6" t="inlineStr"/>
       <c r="O19" s="6" t="inlineStr"/>
       <c r="P19" s="6" t="inlineStr"/>
@@ -1720,35 +1718,35 @@
       <c r="J20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="M20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="O20" s="4" t="inlineStr"/>
       <c r="P20" s="4" t="inlineStr"/>
-      <c r="Q20" s="4" t="inlineStr"/>
+      <c r="Q20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="R20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -1778,13 +1776,13 @@
         <v>1</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>3</v>
@@ -1793,19 +1791,19 @@
         <v>3</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T21" s="6" t="n">
         <v>1</v>
@@ -1813,9 +1811,7 @@
       <c r="U21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="V21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="V21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1847,46 +1843,46 @@
         <v>11</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="L22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="O22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="M22" s="4" t="n">
+      <c r="P22" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>14</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="S22" s="4" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="T22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23">
@@ -1915,46 +1911,46 @@
         <v>100</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="S23" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="T23" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="K23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="L23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="O23" s="8" t="n">
+      <c r="U23" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="V23" s="8" t="n">
         <v>100</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="V23" s="8" t="n">
-        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -2000,7 +1996,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-01</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -2042,72 +2038,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -2136,46 +2132,46 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="O4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="Q4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="U4" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -2203,16 +2199,16 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>13</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>13</v>
@@ -2221,28 +2217,28 @@
         <v>13</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="Q5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="T5" s="6" t="n">
+      <c r="U5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -2270,43 +2266,43 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="Q6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="R6" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="T6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>4</v>
@@ -2340,10 +2336,10 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>4</v>
@@ -2355,7 +2351,7 @@
         <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>3</v>
@@ -2367,7 +2363,7 @@
         <v>3</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>2</v>
@@ -2376,7 +2372,7 @@
         <v>2</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -2416,13 +2412,13 @@
         <v>5</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>7</v>
@@ -2431,16 +2427,16 @@
         <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>5</v>
@@ -2469,10 +2465,10 @@
         <v>2</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>5</v>
@@ -2481,28 +2477,28 @@
         <v>5</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>3</v>
@@ -2536,13 +2532,13 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>6</v>
@@ -2551,28 +2547,28 @@
         <v>6</v>
       </c>
       <c r="M10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N10" s="4" t="n">
         <v>6</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="Q10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="S10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>8</v>
@@ -2603,46 +2599,46 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="J11" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="J11" s="10" t="n">
+      <c r="K11" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>48</v>
-      </c>
       <c r="L11" s="10" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="M11" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="O11" s="10" t="n">
         <v>41</v>
       </c>
-      <c r="N11" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>39</v>
-      </c>
       <c r="P11" s="10" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="S11" s="10" t="n">
         <v>40</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12">
@@ -2670,46 +2666,46 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="S12" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="J12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="N12" s="8" t="n">
+      <c r="T12" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="U12" s="8" t="n">
         <v>100</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-03)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-02</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-03</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-02</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-04)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-03</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-04</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-03</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-05)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-04</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-05</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -676,34 +676,34 @@
         <v>5</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>7</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>7</v>
@@ -712,7 +712,7 @@
         <v>7</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -745,46 +745,46 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>20</v>
-      </c>
       <c r="N5" s="6" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -817,43 +817,43 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>15</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>9</v>
       </c>
       <c r="S6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="T6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="U6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>12</v>
@@ -889,43 +889,43 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="L7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="O7" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="M7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="P7" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>15</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>6</v>
@@ -961,45 +961,45 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="N8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="O8" s="4" t="n">
+      <c r="Q8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="R8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="P8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="S8" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="V8" s="4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="U8" s="4" t="inlineStr"/>
+      <c r="V8" s="4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1027,25 +1027,25 @@
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>3</v>
@@ -1057,16 +1057,16 @@
         <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -1102,22 +1102,22 @@
         <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>2</v>
@@ -1126,19 +1126,19 @@
         <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1171,46 +1171,46 @@
         <v>5</v>
       </c>
       <c r="I11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="J11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="J11" s="6" t="n">
-        <v>9</v>
-      </c>
       <c r="K11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="L11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="N11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="T11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="U11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="O11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="V11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -1238,24 +1238,26 @@
       <c r="H12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>5</v>
@@ -1264,19 +1266,19 @@
         <v>5</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -1315,40 +1317,40 @@
         <v>3</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -1381,22 +1383,22 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>3</v>
@@ -1408,7 +1410,7 @@
         <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>2</v>
@@ -1417,10 +1419,10 @@
         <v>2</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -1453,46 +1455,46 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="P15" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="J15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="Q15" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
@@ -1519,7 +1521,7 @@
         <v>1</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J16" s="4" t="n">
         <v>4</v>
@@ -1528,14 +1530,12 @@
         <v>4</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N16" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
@@ -1579,7 +1579,9 @@
       <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
-      <c r="P17" s="6" t="inlineStr"/>
+      <c r="P17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="Q17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1590,7 +1592,7 @@
         <v>1</v>
       </c>
       <c r="T17" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U17" s="6" t="n">
         <v>3</v>
@@ -1625,16 +1627,14 @@
       <c r="K18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
-      <c r="P18" s="4" t="inlineStr"/>
-      <c r="Q18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="P18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
@@ -1662,14 +1662,12 @@
         <v>1</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="L19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="L19" s="6" t="inlineStr"/>
       <c r="M19" s="6" t="inlineStr"/>
       <c r="N19" s="6" t="inlineStr"/>
       <c r="O19" s="6" t="inlineStr"/>
@@ -1713,38 +1711,38 @@
       <c r="I20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="L20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N20" s="4" t="inlineStr"/>
       <c r="O20" s="4" t="inlineStr"/>
-      <c r="P20" s="4" t="inlineStr"/>
+      <c r="P20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
@@ -1771,13 +1769,13 @@
         <v>1</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>3</v>
@@ -1786,19 +1784,19 @@
         <v>3</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S21" s="6" t="n">
         <v>1</v>
@@ -1806,9 +1804,7 @@
       <c r="T21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="U21" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="U21" s="6" t="inlineStr"/>
       <c r="V21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1841,46 +1837,46 @@
         <v>11</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="N22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="L22" s="4" t="n">
+      <c r="O22" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>14</v>
       </c>
       <c r="P22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="R22" s="4" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="S22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="T22" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="U22" s="4" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23">
@@ -1909,46 +1905,46 @@
         <v>100</v>
       </c>
       <c r="I23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="S23" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="J23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="K23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="L23" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="O23" s="8" t="n">
+      <c r="T23" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="U23" s="8" t="n">
         <v>97</v>
       </c>
       <c r="V23" s="8" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1994,7 +1990,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-04</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-05</t>
         </is>
       </c>
     </row>
@@ -2036,72 +2032,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -2133,40 +2129,40 @@
         <v>16</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="N4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="P4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>17</v>
-      </c>
       <c r="T4" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>14</v>
@@ -2200,10 +2196,10 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="J5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>13</v>
@@ -2212,31 +2208,31 @@
         <v>13</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -2267,13 +2263,13 @@
         <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>7</v>
@@ -2285,25 +2281,25 @@
         <v>7</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -2331,10 +2327,10 @@
         <v>3</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>4</v>
@@ -2346,7 +2342,7 @@
         <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>3</v>
@@ -2358,7 +2354,7 @@
         <v>3</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>2</v>
@@ -2367,10 +2363,10 @@
         <v>2</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -2407,13 +2403,13 @@
         <v>5</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>7</v>
@@ -2422,22 +2418,22 @@
         <v>7</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -2463,7 +2459,7 @@
         <v>2</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>5</v>
@@ -2472,28 +2468,28 @@
         <v>5</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>3</v>
@@ -2533,7 +2529,7 @@
         <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>6</v>
@@ -2542,34 +2538,34 @@
         <v>6</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -2597,43 +2593,43 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="I11" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="I11" s="10" t="n">
+      <c r="J11" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>48</v>
-      </c>
       <c r="K11" s="10" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="L11" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>41</v>
       </c>
-      <c r="M11" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>39</v>
-      </c>
       <c r="O11" s="10" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="R11" s="10" t="n">
         <v>40</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>43</v>
@@ -2664,46 +2660,46 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="R12" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="N12" s="8" t="n">
+      <c r="S12" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="T12" s="8" t="n">
         <v>97</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-06)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-05</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-06</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>
@@ -673,34 +673,34 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>7</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>7</v>
@@ -745,43 +745,43 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>20</v>
-      </c>
       <c r="M5" s="6" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>21</v>
@@ -817,43 +817,43 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>15</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>9</v>
       </c>
       <c r="R6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="S6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="T6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>14</v>
@@ -889,43 +889,43 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>8</v>
       </c>
       <c r="K7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="N7" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="L7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="O7" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>15</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>5</v>
@@ -961,42 +961,42 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="M8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="N8" s="4" t="n">
+      <c r="P8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="O8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="R8" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="U8" s="4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="T8" s="4" t="inlineStr"/>
+      <c r="U8" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="V8" s="4" t="n">
         <v>2</v>
       </c>
@@ -1030,19 +1030,19 @@
         <v>6</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>3</v>
@@ -1054,16 +1054,16 @@
         <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>3</v>
@@ -1099,22 +1099,22 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>2</v>
@@ -1123,19 +1123,19 @@
         <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>5</v>
@@ -1171,43 +1171,43 @@
         <v>5</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="K11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="L11" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="M11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="T11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="N11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="U11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>6</v>
@@ -1242,19 +1242,19 @@
         <v>1</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>5</v>
@@ -1263,19 +1263,19 @@
         <v>5</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>2</v>
@@ -1314,40 +1314,40 @@
         <v>3</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>3</v>
@@ -1386,16 +1386,16 @@
         <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>3</v>
@@ -1407,7 +1407,7 @@
         <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>2</v>
@@ -1416,7 +1416,7 @@
         <v>2</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>3</v>
@@ -1455,43 +1455,43 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>7</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>11</v>
@@ -1527,14 +1527,12 @@
         <v>4</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M16" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
@@ -1578,7 +1576,9 @@
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
       <c r="N17" s="6" t="inlineStr"/>
-      <c r="O17" s="6" t="inlineStr"/>
+      <c r="O17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="P17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1589,7 +1589,7 @@
         <v>1</v>
       </c>
       <c r="S17" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T17" s="6" t="n">
         <v>3</v>
@@ -1624,16 +1624,14 @@
       <c r="J18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
-      <c r="O18" s="4" t="inlineStr"/>
-      <c r="P18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="O18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
@@ -1659,14 +1657,12 @@
       <c r="G19" s="6" t="inlineStr"/>
       <c r="H19" s="6" t="inlineStr"/>
       <c r="I19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K19" s="6" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr"/>
       <c r="M19" s="6" t="inlineStr"/>
       <c r="N19" s="6" t="inlineStr"/>
@@ -1708,38 +1704,38 @@
       <c r="H20" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="I20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="K20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M20" s="4" t="inlineStr"/>
       <c r="N20" s="4" t="inlineStr"/>
-      <c r="O20" s="4" t="inlineStr"/>
+      <c r="O20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>6</v>
@@ -1769,10 +1765,10 @@
         <v>1</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>3</v>
@@ -1781,19 +1777,19 @@
         <v>3</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R21" s="6" t="n">
         <v>1</v>
@@ -1801,10 +1797,10 @@
       <c r="S21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="T21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="U21" s="6" t="inlineStr"/>
+      <c r="T21" s="6" t="inlineStr"/>
+      <c r="U21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V21" s="6" t="n">
         <v>1</v>
       </c>
@@ -1839,43 +1835,43 @@
         <v>11</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="M22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="K22" s="4" t="n">
+      <c r="N22" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="L22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>14</v>
       </c>
       <c r="O22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="R22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="S22" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="T22" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="U22" s="4" t="n">
         <v>12</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>14</v>
       </c>
       <c r="V22" s="4" t="n">
         <v>12</v>
@@ -1907,43 +1903,43 @@
         <v>100</v>
       </c>
       <c r="I23" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="J23" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="K23" s="8" t="n">
         <v>101</v>
       </c>
-      <c r="J23" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="K23" s="8" t="n">
-        <v>108</v>
-      </c>
       <c r="L23" s="8" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="N23" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="R23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="S23" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="T23" s="8" t="n">
         <v>97</v>
       </c>
       <c r="U23" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="V23" s="8" t="n">
         <v>104</v>
@@ -1992,7 +1988,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-05</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-06</t>
         </is>
       </c>
     </row>
@@ -2034,72 +2030,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>
@@ -2128,40 +2124,40 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="M4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="O4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>17</v>
-      </c>
       <c r="S4" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>14</v>
@@ -2195,10 +2191,10 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="I5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>13</v>
@@ -2207,31 +2203,31 @@
         <v>13</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>16</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>19</v>
@@ -2262,13 +2258,13 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>7</v>
@@ -2280,25 +2276,25 @@
         <v>7</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>3</v>
@@ -2329,7 +2325,7 @@
         <v>3</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>4</v>
@@ -2341,7 +2337,7 @@
         <v>4</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>3</v>
@@ -2353,7 +2349,7 @@
         <v>3</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>2</v>
@@ -2362,10 +2358,10 @@
         <v>2</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>4</v>
@@ -2402,13 +2398,13 @@
         <v>5</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>7</v>
@@ -2417,22 +2413,22 @@
         <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>7</v>
@@ -2467,28 +2463,28 @@
         <v>5</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>3</v>
@@ -2528,7 +2524,7 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>6</v>
@@ -2537,34 +2533,34 @@
         <v>6</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>10</v>
@@ -2595,43 +2591,43 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="I11" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="I11" s="10" t="n">
-        <v>48</v>
-      </c>
       <c r="J11" s="10" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="K11" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="M11" s="10" t="n">
         <v>41</v>
       </c>
-      <c r="L11" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>39</v>
-      </c>
       <c r="N11" s="10" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="Q11" s="10" t="n">
         <v>40</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>44</v>
@@ -2662,43 +2658,43 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="J12" s="8" t="n">
         <v>101</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>108</v>
-      </c>
       <c r="K12" s="8" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="M12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="R12" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="S12" s="8" t="n">
         <v>97</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>104</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-07)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-06</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-07</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -673,46 +673,46 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>7</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="V4" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -745,46 +745,46 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>20</v>
-      </c>
       <c r="L5" s="6" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -811,52 +811,52 @@
         <v>17</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="K6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>14</v>
-      </c>
       <c r="O6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>9</v>
       </c>
       <c r="Q6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="R6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="S6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -892,43 +892,43 @@
         <v>8</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="U7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="V7" s="6" t="n">
         <v>10</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="V7" s="6" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -961,44 +961,44 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="M8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="M8" s="4" t="n">
+      <c r="N8" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>8</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>9</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="T8" s="4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="S8" s="4" t="inlineStr"/>
+      <c r="T8" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="U8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -1027,19 +1027,19 @@
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>3</v>
@@ -1051,19 +1051,19 @@
         <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>2</v>
@@ -1099,19 +1099,19 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>2</v>
@@ -1120,25 +1120,25 @@
         <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1165,19 +1165,19 @@
         <v>9</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>5</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>8</v>
@@ -1186,7 +1186,7 @@
         <v>7</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>5</v>
@@ -1201,16 +1201,16 @@
         <v>5</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -1239,19 +1239,19 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>5</v>
@@ -1260,22 +1260,22 @@
         <v>5</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>4</v>
@@ -1311,46 +1311,46 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1383,16 +1383,16 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>3</v>
@@ -1404,7 +1404,7 @@
         <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>2</v>
@@ -1413,16 +1413,16 @@
         <v>2</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -1458,43 +1458,43 @@
         <v>7</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="S15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="T15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="V15" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
@@ -1524,14 +1524,12 @@
         <v>4</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="L16" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
@@ -1575,7 +1573,9 @@
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
       <c r="M17" s="6" t="inlineStr"/>
-      <c r="N17" s="6" t="inlineStr"/>
+      <c r="N17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="O17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1586,7 +1586,7 @@
         <v>1</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S17" s="6" t="n">
         <v>3</v>
@@ -1621,16 +1621,14 @@
       <c r="I18" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="inlineStr"/>
-      <c r="O18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="N18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
@@ -1657,11 +1655,9 @@
       <c r="G19" s="6" t="inlineStr"/>
       <c r="H19" s="6" t="inlineStr"/>
       <c r="I19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J19" s="6" t="inlineStr"/>
       <c r="K19" s="6" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr"/>
       <c r="M19" s="6" t="inlineStr"/>
@@ -1704,41 +1700,43 @@
       <c r="H20" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="I20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="J20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L20" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" s="4" t="inlineStr"/>
+      <c r="N20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -1765,7 +1763,7 @@
         <v>1</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>3</v>
@@ -1774,19 +1772,19 @@
         <v>3</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>1</v>
@@ -1794,15 +1792,15 @@
       <c r="R21" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="S21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T21" s="6" t="inlineStr"/>
+      <c r="S21" s="6" t="inlineStr"/>
+      <c r="T21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U21" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1835,46 +1833,46 @@
         <v>11</v>
       </c>
       <c r="I22" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="L22" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="J22" s="4" t="n">
+      <c r="M22" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="K22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="L22" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>14</v>
       </c>
       <c r="N22" s="4" t="n">
         <v>17</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>12</v>
       </c>
       <c r="R22" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="S22" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="T22" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="S22" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>14</v>
-      </c>
       <c r="U22" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="V22" s="4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23">
@@ -1903,46 +1901,46 @@
         <v>100</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="M23" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="Q23" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="R23" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="S23" s="8" t="n">
         <v>97</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="U23" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="V23" s="8" t="n">
         <v>104</v>
-      </c>
-      <c r="V23" s="8" t="n">
-        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -1988,7 +1986,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-06</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-07</t>
         </is>
       </c>
     </row>
@@ -2030,72 +2028,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
     </row>
@@ -2124,37 +2122,37 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="L4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="N4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="N4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>17</v>
-      </c>
       <c r="R4" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>14</v>
@@ -2163,7 +2161,7 @@
         <v>14</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -2191,7 +2189,7 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>13</v>
@@ -2200,37 +2198,37 @@
         <v>13</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>16</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -2258,10 +2256,10 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>7</v>
@@ -2273,28 +2271,28 @@
         <v>7</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>4</v>
@@ -2334,7 +2332,7 @@
         <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>3</v>
@@ -2346,7 +2344,7 @@
         <v>3</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>2</v>
@@ -2355,10 +2353,10 @@
         <v>2</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>4</v>
@@ -2395,13 +2393,13 @@
         <v>5</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>7</v>
@@ -2410,28 +2408,28 @@
         <v>7</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -2460,28 +2458,28 @@
         <v>5</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>3</v>
@@ -2530,40 +2528,40 @@
         <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -2591,46 +2589,46 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="J11" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="L11" s="10" t="n">
         <v>41</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>39</v>
-      </c>
       <c r="M11" s="10" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="P11" s="10" t="n">
         <v>40</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="R11" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12">
@@ -2658,46 +2656,46 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="L12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q12" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="R12" s="8" t="n">
         <v>97</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="T12" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="U12" s="8" t="n">
         <v>104</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-08)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:V22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-07</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-08</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -673,28 +673,28 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>7</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>7</v>
@@ -706,13 +706,13 @@
         <v>7</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -745,46 +745,46 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="U5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="V5" s="6" t="n">
         <v>14</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -817,10 +817,10 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>14</v>
@@ -829,31 +829,31 @@
         <v>14</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>9</v>
       </c>
       <c r="P6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="Q6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="R6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>15</v>
@@ -889,46 +889,46 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>14</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="Q7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="U7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="V7" s="6" t="n">
         <v>10</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="V7" s="6" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -961,41 +961,41 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="M8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="N8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="O8" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="M8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="P8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="S8" s="4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="R8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>3</v>
@@ -1027,16 +1027,16 @@
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>3</v>
@@ -1048,25 +1048,25 @@
         <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1099,16 +1099,16 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>2</v>
@@ -1117,28 +1117,28 @@
         <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1171,43 +1171,43 @@
         <v>5</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="M11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="S11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>4</v>
@@ -1239,16 +1239,16 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>5</v>
@@ -1257,28 +1257,28 @@
         <v>5</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1311,46 +1311,46 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -1386,10 +1386,10 @@
         <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>3</v>
@@ -1401,7 +1401,7 @@
         <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>2</v>
@@ -1410,19 +1410,19 @@
         <v>2</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -1455,43 +1455,43 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="R15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="S15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="U15" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>6</v>
@@ -1521,14 +1521,12 @@
         <v>1</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K16" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
       <c r="N16" s="4" t="inlineStr"/>
@@ -1572,7 +1570,9 @@
       <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr"/>
-      <c r="M17" s="6" t="inlineStr"/>
+      <c r="M17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="N17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1583,7 +1583,7 @@
         <v>1</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R17" s="6" t="n">
         <v>3</v>
@@ -1595,7 +1595,7 @@
         <v>3</v>
       </c>
       <c r="U17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V17" s="6" t="n">
         <v>2</v>
@@ -1618,16 +1618,14 @@
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="M18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
@@ -1640,36 +1638,70 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Externa</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Pendiente agendar llamada</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr"/>
-      <c r="D19" s="6" t="inlineStr"/>
-      <c r="E19" s="6" t="inlineStr"/>
-      <c r="F19" s="6" t="inlineStr"/>
-      <c r="G19" s="6" t="inlineStr"/>
-      <c r="H19" s="6" t="inlineStr"/>
+          <t>Pendiente definir servicio externo</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="I19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="6" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K19" s="6" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr"/>
-      <c r="M19" s="6" t="inlineStr"/>
-      <c r="N19" s="6" t="inlineStr"/>
-      <c r="O19" s="6" t="inlineStr"/>
-      <c r="P19" s="6" t="inlineStr"/>
-      <c r="Q19" s="6" t="inlineStr"/>
-      <c r="R19" s="6" t="inlineStr"/>
-      <c r="S19" s="6" t="inlineStr"/>
-      <c r="T19" s="6" t="inlineStr"/>
-      <c r="U19" s="6" t="inlineStr"/>
-      <c r="V19" s="6" t="inlineStr"/>
+      <c r="M19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O19" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P19" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R19" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="S19" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="T19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="U19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="V19" s="6" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1679,64 +1711,60 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Pendiente definir servicio externo</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D20" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E20" s="4" t="n">
-        <v>3</v>
-      </c>
+          <t>Esperando respuesta cliente a presupuesto</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr"/>
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="4" t="inlineStr"/>
       <c r="F20" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" s="4" t="inlineStr"/>
-      <c r="M20" s="4" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="N20" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="R20" s="4" t="n">
-        <v>5</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="R20" s="4" t="inlineStr"/>
       <c r="S20" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="V20" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1747,200 +1775,136 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Esperando respuesta cliente a presupuesto</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr"/>
-      <c r="D21" s="6" t="inlineStr"/>
-      <c r="E21" s="6" t="inlineStr"/>
+          <t>Enviado a técnico externo</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>18</v>
+      </c>
       <c r="F21" s="6" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S21" s="6" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="S21" s="6" t="n">
+        <v>12</v>
+      </c>
       <c r="T21" s="6" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Externa</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Enviado a técnico externo</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="D22" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="E22" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="F22" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="G22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="H22" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="I22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="J22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="K22" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="L22" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="V22" s="4" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr"/>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr"/>
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Total abiertas</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n">
+      <c r="C22" s="8" t="n">
         <v>129</v>
       </c>
-      <c r="D23" s="8" t="n">
+      <c r="D22" s="8" t="n">
         <v>96</v>
       </c>
-      <c r="E23" s="8" t="n">
+      <c r="E22" s="8" t="n">
         <v>85</v>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="F22" s="8" t="n">
         <v>79</v>
       </c>
-      <c r="G23" s="8" t="n">
+      <c r="G22" s="8" t="n">
         <v>84</v>
       </c>
-      <c r="H23" s="8" t="n">
+      <c r="H22" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="I23" s="8" t="n">
+      <c r="I22" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="J22" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="K22" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="L22" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="M22" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="N22" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="O22" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="P22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q22" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="R22" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="S22" s="8" t="n">
+        <v>104</v>
+      </c>
+      <c r="T22" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="J23" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="K23" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="L23" s="8" t="n">
+      <c r="U22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="V22" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="Q23" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="R23" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="S23" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="T23" s="8" t="n">
-        <v>104</v>
-      </c>
-      <c r="U23" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="V23" s="8" t="n">
-        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1986,7 +1950,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-07</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2028,72 +1992,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2122,34 +2086,34 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="M4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>17</v>
-      </c>
       <c r="Q4" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>14</v>
@@ -2158,10 +2122,10 @@
         <v>14</v>
       </c>
       <c r="T4" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>14</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -2195,37 +2159,37 @@
         <v>13</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>16</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>16</v>
@@ -2256,7 +2220,7 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>7</v>
@@ -2268,31 +2232,31 @@
         <v>7</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>3</v>
@@ -2329,7 +2293,7 @@
         <v>4</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>3</v>
@@ -2341,7 +2305,7 @@
         <v>3</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>2</v>
@@ -2350,10 +2314,10 @@
         <v>2</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>4</v>
@@ -2390,13 +2354,13 @@
         <v>5</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>7</v>
@@ -2405,28 +2369,28 @@
         <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>5</v>
@@ -2455,28 +2419,28 @@
         <v>2</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>3</v>
@@ -2525,40 +2489,40 @@
         <v>6</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>9</v>
@@ -2589,46 +2553,46 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="K11" s="10" t="n">
         <v>41</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>39</v>
-      </c>
       <c r="L11" s="10" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="O11" s="10" t="n">
         <v>40</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="R11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="S11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="T11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="U11" s="10" t="n">
         <v>43</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>44</v>
       </c>
     </row>
     <row r="12">
@@ -2656,46 +2620,46 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="K12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="P12" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="Q12" s="8" t="n">
         <v>97</v>
       </c>
       <c r="R12" s="8" t="n">
+        <v>104</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="T12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="U12" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>104</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>108</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-09)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-08</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-09</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -673,25 +673,25 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>7</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>7</v>
@@ -703,13 +703,13 @@
         <v>7</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>6</v>
@@ -745,46 +745,46 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="R5" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>20</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -817,7 +817,7 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>14</v>
@@ -826,34 +826,34 @@
         <v>14</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>9</v>
       </c>
       <c r="O6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="P6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="Q6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="T6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>15</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>17</v>
@@ -889,43 +889,43 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>14</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>6</v>
@@ -961,44 +961,44 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="M8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="N8" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="L8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="O8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R8" s="4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="Q8" s="4" t="inlineStr"/>
+      <c r="R8" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="S8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -1027,13 +1027,13 @@
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>3</v>
@@ -1045,28 +1045,28 @@
         <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -1099,13 +1099,13 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>2</v>
@@ -1114,31 +1114,31 @@
         <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1171,43 +1171,43 @@
         <v>5</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="L11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="R11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>5</v>
@@ -1239,13 +1239,13 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>5</v>
@@ -1254,28 +1254,28 @@
         <v>5</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>1</v>
@@ -1311,46 +1311,46 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1383,10 +1383,10 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>3</v>
@@ -1398,7 +1398,7 @@
         <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>2</v>
@@ -1407,22 +1407,22 @@
         <v>2</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -1458,40 +1458,40 @@
         <v>4</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="Q15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="S15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="R15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="T15" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>4</v>
@@ -1521,11 +1521,9 @@
         <v>1</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="J16" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="4" t="inlineStr"/>
@@ -1569,7 +1567,9 @@
       <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr"/>
       <c r="K17" s="6" t="inlineStr"/>
-      <c r="L17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1580,7 +1580,7 @@
         <v>1</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>3</v>
@@ -1592,7 +1592,7 @@
         <v>3</v>
       </c>
       <c r="T17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U17" s="6" t="n">
         <v>2</v>
@@ -1621,10 +1621,10 @@
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="L18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
@@ -1665,33 +1665,33 @@
         <v>5</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="J19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J19" s="6" t="inlineStr"/>
       <c r="K19" s="6" t="inlineStr"/>
-      <c r="L19" s="6" t="inlineStr"/>
+      <c r="L19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="M19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O19" s="6" t="n">
         <v>4</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T19" s="6" t="n">
         <v>5</v>
@@ -1730,19 +1730,19 @@
         <v>3</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>1</v>
@@ -1750,15 +1750,15 @@
       <c r="P20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R20" s="4" t="inlineStr"/>
+      <c r="Q20" s="4" t="inlineStr"/>
+      <c r="R20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>1</v>
@@ -1797,46 +1797,46 @@
         <v>11</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>17</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="O21" s="6" t="n">
         <v>12</v>
       </c>
       <c r="P21" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q21" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="R21" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q21" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="R21" s="6" t="n">
+      <c r="S21" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="T21" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="S21" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="T21" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="U21" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22">
@@ -1865,43 +1865,43 @@
         <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="K22" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="L22" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="M22" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="N22" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="O22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="P22" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="L22" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="M22" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="N22" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="O22" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="P22" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="Q22" s="8" t="n">
         <v>97</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>98</v>
@@ -1950,7 +1950,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-08</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-09</t>
         </is>
       </c>
     </row>
@@ -1992,72 +1992,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
     </row>
@@ -2086,31 +2086,31 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>17</v>
-      </c>
       <c r="P4" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>14</v>
@@ -2119,10 +2119,10 @@
         <v>14</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>16</v>
@@ -2156,43 +2156,43 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>16</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -2229,31 +2229,31 @@
         <v>7</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>3</v>
@@ -2290,7 +2290,7 @@
         <v>4</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>3</v>
@@ -2302,7 +2302,7 @@
         <v>3</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>2</v>
@@ -2311,10 +2311,10 @@
         <v>2</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>4</v>
@@ -2323,7 +2323,7 @@
         <v>4</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>3</v>
@@ -2354,10 +2354,10 @@
         <v>5</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>7</v>
@@ -2366,34 +2366,34 @@
         <v>7</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -2419,25 +2419,25 @@
         <v>2</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>4</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>3</v>
@@ -2486,43 +2486,43 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="S10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="T10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>10</v>
@@ -2553,43 +2553,43 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="J11" s="10" t="n">
         <v>41</v>
       </c>
-      <c r="I11" s="10" t="n">
-        <v>42</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>39</v>
-      </c>
       <c r="K11" s="10" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="N11" s="10" t="n">
         <v>40</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="S11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="T11" s="10" t="n">
         <v>43</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>44</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>43</v>
@@ -2620,43 +2620,43 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="J12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="O12" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="P12" s="8" t="n">
         <v>97</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>98</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-10)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-09</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-10</t>
         </is>
       </c>
     </row>
@@ -1950,7 +1950,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-09</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-11)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-10</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-11</t>
         </is>
       </c>
     </row>
@@ -1950,7 +1950,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-10</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-12)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-11</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-12</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -673,22 +673,22 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>7</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>7</v>
@@ -700,19 +700,19 @@
         <v>7</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>6</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -745,46 +745,46 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>20</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -823,40 +823,40 @@
         <v>14</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>9</v>
       </c>
       <c r="N6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="O6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="P6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="T6" s="4" t="n">
-        <v>15</v>
-      </c>
       <c r="U6" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
@@ -889,46 +889,46 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>14</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="O7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="U7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="P7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="V7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -961,44 +961,44 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="L8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="M8" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="K8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="N8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q8" s="4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="P8" s="4" t="inlineStr"/>
+      <c r="Q8" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="R8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -1027,10 +1027,10 @@
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>3</v>
@@ -1042,25 +1042,25 @@
         <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>2</v>
@@ -1099,10 +1099,10 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>2</v>
@@ -1111,28 +1111,28 @@
         <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>1</v>
@@ -1171,43 +1171,43 @@
         <v>5</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="K11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="L11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="Q11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>7</v>
@@ -1239,10 +1239,10 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>5</v>
@@ -1251,31 +1251,31 @@
         <v>5</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>3</v>
@@ -1314,37 +1314,37 @@
         <v>5</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>5</v>
@@ -1383,7 +1383,7 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>3</v>
@@ -1395,7 +1395,7 @@
         <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>2</v>
@@ -1404,19 +1404,19 @@
         <v>2</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>4</v>
@@ -1455,46 +1455,46 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="P15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="R15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="S15" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -1520,9 +1520,7 @@
       <c r="H16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I16" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
@@ -1566,7 +1564,9 @@
       </c>
       <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr"/>
-      <c r="K17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1577,7 +1577,7 @@
         <v>1</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P17" s="6" t="n">
         <v>3</v>
@@ -1589,7 +1589,7 @@
         <v>3</v>
       </c>
       <c r="S17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T17" s="6" t="n">
         <v>2</v>
@@ -1598,7 +1598,7 @@
         <v>2</v>
       </c>
       <c r="V17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -1620,10 +1620,10 @@
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="K18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
@@ -1633,7 +1633,9 @@
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
-      <c r="V18" s="4" t="inlineStr"/>
+      <c r="V18" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1664,31 +1666,31 @@
       <c r="H19" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="I19" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="I19" s="6" t="inlineStr"/>
       <c r="J19" s="6" t="inlineStr"/>
-      <c r="K19" s="6" t="inlineStr"/>
+      <c r="K19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="L19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>4</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S19" s="6" t="n">
         <v>5</v>
@@ -1700,7 +1702,7 @@
         <v>5</v>
       </c>
       <c r="V19" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
@@ -1727,19 +1729,19 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>1</v>
@@ -1747,15 +1749,15 @@
       <c r="O20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q20" s="4" t="inlineStr"/>
+      <c r="P20" s="4" t="inlineStr"/>
+      <c r="Q20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="R20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>1</v>
@@ -1797,46 +1799,46 @@
         <v>11</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>17</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>12</v>
       </c>
       <c r="O21" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="P21" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q21" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="P21" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="Q21" s="6" t="n">
+      <c r="R21" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="S21" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="R21" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="S21" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="T21" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22">
@@ -1865,46 +1867,46 @@
         <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="J22" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="K22" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="L22" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="M22" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="N22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="O22" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="K22" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="L22" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="M22" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="N22" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="O22" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="P22" s="8" t="n">
         <v>97</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="S22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="T22" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="U22" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="T22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="U22" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="V22" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1950,7 +1952,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-11</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-12</t>
         </is>
       </c>
     </row>
@@ -1992,72 +1994,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
     </row>
@@ -2089,25 +2091,25 @@
         <v>17</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="K4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>17</v>
-      </c>
       <c r="O4" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>14</v>
@@ -2116,16 +2118,16 @@
         <v>14</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -2153,43 +2155,43 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>16</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>17</v>
@@ -2226,31 +2228,31 @@
         <v>7</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>3</v>
@@ -2259,7 +2261,7 @@
         <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -2287,7 +2289,7 @@
         <v>3</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>3</v>
@@ -2299,7 +2301,7 @@
         <v>3</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>2</v>
@@ -2308,10 +2310,10 @@
         <v>2</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>4</v>
@@ -2320,7 +2322,7 @@
         <v>4</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>3</v>
@@ -2354,7 +2356,7 @@
         <v>5</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>7</v>
@@ -2363,37 +2365,37 @@
         <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -2422,19 +2424,19 @@
         <v>4</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>3</v>
@@ -2455,7 +2457,7 @@
         <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>6</v>
@@ -2486,46 +2488,46 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="R10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="S10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -2553,46 +2555,46 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="M11" s="10" t="n">
         <v>40</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="O11" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="Q11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="R11" s="10" t="n">
+      <c r="T11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="U11" s="10" t="n">
         <v>46</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>45</v>
       </c>
     </row>
     <row r="12">
@@ -2620,46 +2622,46 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="I12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="N12" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="O12" s="8" t="n">
         <v>97</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="R12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="T12" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="S12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="U12" s="8" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-13)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-12</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-13</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -676,16 +676,16 @@
         <v>7</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>7</v>
@@ -697,20 +697,18 @@
         <v>7</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="U4" s="4" t="n">
-        <v>6</v>
-      </c>
+      <c r="U4" s="4" t="inlineStr"/>
       <c r="V4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -743,43 +741,43 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>20</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>17</v>
@@ -818,40 +816,40 @@
         <v>14</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>9</v>
       </c>
       <c r="M6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="N6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="O6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="R6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="S6" s="4" t="n">
-        <v>15</v>
-      </c>
       <c r="T6" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>18</v>
@@ -887,43 +885,43 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>14</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="N7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="T7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="O7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="U7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>9</v>
@@ -959,41 +957,41 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>9</v>
-      </c>
       <c r="M8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="P8" s="4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="O8" s="4" t="inlineStr"/>
+      <c r="P8" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="Q8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>3</v>
@@ -1025,7 +1023,7 @@
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>3</v>
@@ -1037,25 +1035,25 @@
         <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>2</v>
@@ -1097,7 +1095,7 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>2</v>
@@ -1106,28 +1104,28 @@
         <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>1</v>
@@ -1169,40 +1167,40 @@
         <v>5</v>
       </c>
       <c r="I11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="J11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="K11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="L11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="P11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>7</v>
@@ -1237,7 +1235,7 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>5</v>
@@ -1246,31 +1244,31 @@
         <v>5</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U12" s="4" t="n">
         <v>3</v>
@@ -1309,43 +1307,43 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>4</v>
@@ -1390,7 +1388,7 @@
         <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>2</v>
@@ -1399,25 +1397,25 @@
         <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>5</v>
@@ -1453,43 +1451,43 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="O15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="P15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="R15" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="T15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>2</v>
@@ -1561,7 +1559,9 @@
         <v>2</v>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1572,7 +1572,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O17" s="6" t="n">
         <v>3</v>
@@ -1584,7 +1584,7 @@
         <v>3</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S17" s="6" t="n">
         <v>2</v>
@@ -1593,7 +1593,7 @@
         <v>2</v>
       </c>
       <c r="U17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V17" s="6" t="n">
         <v>3</v>
@@ -1617,10 +1617,10 @@
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
@@ -1630,7 +1630,9 @@
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
-      <c r="U18" s="4" t="inlineStr"/>
+      <c r="U18" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V18" s="4" t="n">
         <v>1</v>
       </c>
@@ -1665,27 +1667,29 @@
         <v>5</v>
       </c>
       <c r="I19" s="6" t="inlineStr"/>
-      <c r="J19" s="6" t="inlineStr"/>
+      <c r="J19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="K19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M19" s="6" t="n">
         <v>4</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R19" s="6" t="n">
         <v>5</v>
@@ -1697,7 +1701,7 @@
         <v>5</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>8</v>
@@ -1727,16 +1731,16 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M20" s="4" t="n">
         <v>1</v>
@@ -1744,15 +1748,15 @@
       <c r="N20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="O20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P20" s="4" t="inlineStr"/>
+      <c r="O20" s="4" t="inlineStr"/>
+      <c r="P20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S20" s="4" t="n">
         <v>1</v>
@@ -1797,40 +1801,40 @@
         <v>11</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>17</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>12</v>
       </c>
       <c r="N21" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="O21" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="P21" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="O21" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="P21" s="6" t="n">
+      <c r="Q21" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="R21" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="Q21" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="R21" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="S21" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="U21" s="6" t="n">
         <v>22</v>
@@ -1865,43 +1869,43 @@
         <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="J22" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="K22" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="L22" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="M22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="N22" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="J22" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="K22" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="L22" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="M22" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="N22" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="O22" s="8" t="n">
         <v>97</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="R22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="S22" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="T22" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="S22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="T22" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="U22" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>106</v>
@@ -1950,7 +1954,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-12</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-13</t>
         </is>
       </c>
     </row>
@@ -1992,72 +1996,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -2086,25 +2090,25 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="I4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="J4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>17</v>
-      </c>
       <c r="N4" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>14</v>
@@ -2113,16 +2117,16 @@
         <v>14</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>18</v>
@@ -2153,40 +2157,40 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>16</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>17</v>
@@ -2223,31 +2227,31 @@
         <v>7</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>3</v>
@@ -2256,7 +2260,7 @@
         <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>4</v>
@@ -2296,7 +2300,7 @@
         <v>3</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>2</v>
@@ -2305,10 +2309,10 @@
         <v>2</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>4</v>
@@ -2317,7 +2321,7 @@
         <v>4</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>3</v>
@@ -2360,37 +2364,37 @@
         <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>4</v>
@@ -2419,19 +2423,19 @@
         <v>2</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>3</v>
@@ -2452,7 +2456,7 @@
         <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>6</v>
@@ -2489,40 +2493,40 @@
         <v>6</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="Q10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="R10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>8</v>
@@ -2553,43 +2557,43 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="L11" s="10" t="n">
         <v>40</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="O11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="R11" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="P11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="Q11" s="10" t="n">
+      <c r="S11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="T11" s="10" t="n">
         <v>46</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>45</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>46</v>
@@ -2620,43 +2624,43 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>109</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>91</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="M12" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="I12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>109</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>91</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>95</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>97</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="Q12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="S12" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="R12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="T12" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>106</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-14)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-13</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-14</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -673,16 +673,16 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>7</v>
@@ -694,21 +694,21 @@
         <v>7</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="T4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="U4" s="4" t="inlineStr"/>
+      <c r="T4" s="4" t="inlineStr"/>
+      <c r="U4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V4" s="4" t="n">
         <v>1</v>
       </c>
@@ -743,46 +743,46 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>20</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="S5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="U5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="T5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="U5" s="6" t="n">
-        <v>17</v>
-      </c>
       <c r="V5" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -815,46 +815,46 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>9</v>
       </c>
       <c r="L6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="N6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="Q6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="R6" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="R6" s="4" t="n">
-        <v>15</v>
-      </c>
       <c r="S6" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
@@ -887,43 +887,43 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>14</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="M7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="N7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="T7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>5</v>
@@ -959,41 +959,41 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="J8" s="4" t="n">
-        <v>10</v>
-      </c>
       <c r="K8" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="O8" s="4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="N8" s="4" t="inlineStr"/>
+      <c r="O8" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="P8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>8</v>
@@ -1034,25 +1034,25 @@
         <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>2</v>
@@ -1061,7 +1061,7 @@
         <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>3</v>
@@ -1103,28 +1103,28 @@
         <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>1</v>
@@ -1133,7 +1133,7 @@
         <v>1</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>2</v>
@@ -1169,7 +1169,7 @@
         <v>5</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>5</v>
@@ -1184,31 +1184,31 @@
         <v>5</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -1243,40 +1243,40 @@
         <v>5</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1309,46 +1309,46 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1387,7 +1387,7 @@
         <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>2</v>
@@ -1396,31 +1396,31 @@
         <v>2</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -1453,43 +1453,43 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="N15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="P15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="O15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="Q15" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>6</v>
@@ -1560,7 +1560,9 @@
       <c r="H17" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J17" s="6" t="n">
         <v>1</v>
       </c>
@@ -1571,7 +1573,7 @@
         <v>1</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>3</v>
@@ -1583,7 +1585,7 @@
         <v>3</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R17" s="6" t="n">
         <v>2</v>
@@ -1592,10 +1594,10 @@
         <v>2</v>
       </c>
       <c r="T17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V17" s="6" t="n">
         <v>4</v>
@@ -1618,10 +1620,10 @@
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
@@ -1631,10 +1633,10 @@
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
-      <c r="T18" s="4" t="inlineStr"/>
-      <c r="U18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="T18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1666,27 +1668,29 @@
       <c r="H19" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="I19" s="6" t="inlineStr"/>
+      <c r="I19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="J19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>5</v>
@@ -1698,10 +1702,10 @@
         <v>5</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>5</v>
@@ -1731,13 +1735,13 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L20" s="4" t="n">
         <v>1</v>
@@ -1745,15 +1749,15 @@
       <c r="M20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O20" s="4" t="inlineStr"/>
+      <c r="N20" s="4" t="inlineStr"/>
+      <c r="O20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>1</v>
@@ -1765,7 +1769,7 @@
         <v>1</v>
       </c>
       <c r="U20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V20" s="4" t="n">
         <v>2</v>
@@ -1804,43 +1808,43 @@
         <v>17</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>12</v>
       </c>
       <c r="M21" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="N21" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="O21" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="N21" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="O21" s="6" t="n">
+      <c r="P21" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q21" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="P21" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q21" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="R21" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="T21" s="6" t="n">
         <v>22</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22">
@@ -1869,46 +1873,46 @@
         <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="N22" s="8" t="n">
         <v>97</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="Q22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="R22" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="S22" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="R22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="S22" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="T22" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="U22" s="8" t="n">
         <v>106</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1954,7 +1958,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-13</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-14</t>
         </is>
       </c>
     </row>
@@ -1996,72 +2000,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -2090,22 +2094,22 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="I4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>17</v>
-      </c>
       <c r="M4" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>14</v>
@@ -2114,22 +2118,22 @@
         <v>14</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="R4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="U4" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -2157,37 +2161,37 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>16</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>17</v>
@@ -2224,31 +2228,31 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>3</v>
@@ -2257,13 +2261,13 @@
         <v>3</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -2297,7 +2301,7 @@
         <v>3</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>2</v>
@@ -2306,10 +2310,10 @@
         <v>2</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>4</v>
@@ -2318,7 +2322,7 @@
         <v>4</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>3</v>
@@ -2330,7 +2334,7 @@
         <v>3</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -2361,40 +2365,40 @@
         <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>5</v>
@@ -2423,16 +2427,16 @@
         <v>2</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>3</v>
@@ -2453,7 +2457,7 @@
         <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>6</v>
@@ -2490,43 +2494,43 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="P10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>7</v>
@@ -2557,46 +2561,46 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="K11" s="10" t="n">
         <v>40</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="Q11" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="O11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="P11" s="10" t="n">
+      <c r="R11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="Q11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>45</v>
-      </c>
       <c r="T11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12">
@@ -2624,46 +2628,46 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="M12" s="8" t="n">
         <v>97</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="P12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="R12" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="Q12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="S12" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="T12" s="8" t="n">
         <v>106</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-15)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-14</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-15</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -673,13 +673,13 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>7</v>
@@ -691,23 +691,23 @@
         <v>7</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="S4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="T4" s="4" t="inlineStr"/>
+      <c r="S4" s="4" t="inlineStr"/>
+      <c r="T4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="U4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>2</v>
@@ -743,46 +743,46 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>11</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>20</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="R5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="S5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="T5" s="6" t="n">
-        <v>17</v>
-      </c>
       <c r="U5" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -815,46 +815,46 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>9</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="L6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="M6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="P6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="Q6" s="4" t="n">
-        <v>15</v>
-      </c>
       <c r="R6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="S6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>19</v>
-      </c>
       <c r="V6" s="4" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -887,46 +887,46 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>14</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="L7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="R7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="M7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="S7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
@@ -959,44 +959,44 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J8" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="M8" s="4" t="inlineStr"/>
+      <c r="N8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="V8" s="4" t="n">
         <v>9</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N8" s="4" t="inlineStr"/>
-      <c r="O8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -1031,25 +1031,25 @@
         <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>2</v>
@@ -1058,10 +1058,10 @@
         <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>4</v>
@@ -1100,28 +1100,28 @@
         <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>1</v>
@@ -1130,13 +1130,13 @@
         <v>1</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1181,28 +1181,28 @@
         <v>5</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>5</v>
@@ -1240,43 +1240,43 @@
         <v>5</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1309,46 +1309,46 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1384,7 +1384,7 @@
         <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>2</v>
@@ -1393,34 +1393,34 @@
         <v>2</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -1453,43 +1453,43 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="M15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="O15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="N15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="P15" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="R15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>7</v>
@@ -1570,7 +1570,7 @@
         <v>1</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M17" s="6" t="n">
         <v>3</v>
@@ -1582,7 +1582,7 @@
         <v>3</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>2</v>
@@ -1591,16 +1591,16 @@
         <v>2</v>
       </c>
       <c r="S17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U17" s="6" t="n">
         <v>4</v>
       </c>
       <c r="V17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -1620,9 +1620,7 @@
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
@@ -1632,10 +1630,10 @@
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
-      <c r="S18" s="4" t="inlineStr"/>
-      <c r="T18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="S18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
     </row>
@@ -1669,25 +1667,25 @@
         <v>5</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>4</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P19" s="6" t="n">
         <v>5</v>
@@ -1699,13 +1697,13 @@
         <v>5</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>6</v>
@@ -1735,10 +1733,10 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>1</v>
@@ -1746,15 +1744,15 @@
       <c r="L20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="M20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="inlineStr"/>
+      <c r="N20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>1</v>
@@ -1766,12 +1764,12 @@
         <v>1</v>
       </c>
       <c r="T20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U20" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="V20" s="4" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="U20" s="4" t="inlineStr"/>
+      <c r="V20" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1803,43 +1801,43 @@
         <v>11</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>12</v>
       </c>
       <c r="L21" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="M21" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="N21" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="M21" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="N21" s="6" t="n">
+      <c r="O21" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="P21" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="O21" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="P21" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="Q21" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="S21" s="6" t="n">
         <v>22</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>13</v>
@@ -1871,46 +1869,46 @@
         <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="M22" s="8" t="n">
         <v>97</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="P22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q22" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="R22" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="Q22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="R22" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="S22" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="T22" s="8" t="n">
         <v>106</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1956,7 +1954,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-14</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-15</t>
         </is>
       </c>
     </row>
@@ -1998,72 +1996,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -2092,19 +2090,19 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="I4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>18</v>
-      </c>
       <c r="K4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>14</v>
@@ -2113,22 +2111,22 @@
         <v>14</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="Q4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>16</v>
@@ -2159,34 +2157,34 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>17</v>
@@ -2198,7 +2196,7 @@
         <v>17</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -2226,28 +2224,28 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>3</v>
@@ -2256,13 +2254,13 @@
         <v>3</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>2</v>
@@ -2296,7 +2294,7 @@
         <v>3</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>2</v>
@@ -2305,10 +2303,10 @@
         <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>4</v>
@@ -2317,7 +2315,7 @@
         <v>4</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>3</v>
@@ -2329,7 +2327,7 @@
         <v>3</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>4</v>
@@ -2360,46 +2358,46 @@
         <v>5</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -2428,10 +2426,10 @@
         <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>3</v>
@@ -2452,7 +2450,7 @@
         <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>6</v>
@@ -2461,7 +2459,7 @@
         <v>6</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>3</v>
@@ -2495,37 +2493,37 @@
         <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="O10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="P10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>7</v>
@@ -2559,46 +2557,46 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>40</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="P11" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="N11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="O11" s="10" t="n">
+      <c r="Q11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="R11" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="P11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>45</v>
-      </c>
       <c r="S11" s="10" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12">
@@ -2626,46 +2624,46 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>97</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="O12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="Q12" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="P12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="R12" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="S12" s="8" t="n">
         <v>106</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-16)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-15</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-16</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -673,10 +673,10 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>7</v>
@@ -688,30 +688,28 @@
         <v>7</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="R4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="S4" s="4" t="inlineStr"/>
+      <c r="R4" s="4" t="inlineStr"/>
+      <c r="S4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="T4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="V4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -746,43 +744,43 @@
         <v>11</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>20</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="R5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="S5" s="6" t="n">
-        <v>17</v>
-      </c>
       <c r="T5" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -818,43 +816,43 @@
         <v>9</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="K6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="L6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="O6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="P6" s="4" t="n">
+      <c r="Q6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="Q6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="R6" s="4" t="n">
+      <c r="V6" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="V6" s="4" t="n">
-        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -890,40 +888,40 @@
         <v>14</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="L7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="R7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>13</v>
@@ -959,44 +957,44 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="M8" s="4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="L8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="N8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -1028,25 +1026,25 @@
         <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>2</v>
@@ -1055,13 +1053,13 @@
         <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>6</v>
@@ -1097,28 +1095,28 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>1</v>
@@ -1127,16 +1125,16 @@
         <v>1</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1178,37 +1176,37 @@
         <v>5</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>5</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -1237,47 +1235,45 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="V12" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="V12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1309,46 +1305,46 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1381,7 +1377,7 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>2</v>
@@ -1390,37 +1386,37 @@
         <v>2</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -1453,46 +1449,46 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="L15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="N15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="M15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="O15" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -1567,7 +1563,7 @@
         <v>1</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L17" s="6" t="n">
         <v>3</v>
@@ -1579,7 +1575,7 @@
         <v>3</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P17" s="6" t="n">
         <v>2</v>
@@ -1588,19 +1584,19 @@
         <v>2</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T17" s="6" t="n">
         <v>4</v>
       </c>
       <c r="U17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -1629,10 +1625,10 @@
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
-      <c r="R18" s="4" t="inlineStr"/>
-      <c r="S18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="R18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
@@ -1667,22 +1663,22 @@
         <v>5</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>4</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O19" s="6" t="n">
         <v>5</v>
@@ -1694,19 +1690,19 @@
         <v>5</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="V19" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -1733,7 +1729,7 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>1</v>
@@ -1741,15 +1737,15 @@
       <c r="K20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="L20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>1</v>
@@ -1761,11 +1757,9 @@
         <v>1</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T20" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="T20" s="4" t="inlineStr"/>
       <c r="U20" s="4" t="inlineStr"/>
       <c r="V20" s="4" t="inlineStr"/>
     </row>
@@ -1799,40 +1793,40 @@
         <v>11</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>12</v>
       </c>
       <c r="K21" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="M21" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="L21" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="M21" s="6" t="n">
+      <c r="N21" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="O21" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="N21" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="O21" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="P21" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="R21" s="6" t="n">
         <v>22</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="U21" s="6" t="n">
         <v>13</v>
@@ -1867,46 +1861,46 @@
         <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>97</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="O22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="P22" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="Q22" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="P22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="Q22" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="R22" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="S22" s="8" t="n">
         <v>106</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1952,7 +1946,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-15</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-16</t>
         </is>
       </c>
     </row>
@@ -1994,72 +1988,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
     </row>
@@ -2088,16 +2082,16 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>14</v>
@@ -2106,28 +2100,28 @@
         <v>14</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="P4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="Q4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="S4" s="4" t="n">
+      <c r="T4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="U4" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -2155,31 +2149,31 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>17</v>
@@ -2191,10 +2185,10 @@
         <v>17</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -2222,25 +2216,25 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>3</v>
@@ -2249,13 +2243,13 @@
         <v>3</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>2</v>
@@ -2289,7 +2283,7 @@
         <v>3</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>2</v>
@@ -2298,10 +2292,10 @@
         <v>2</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>4</v>
@@ -2310,7 +2304,7 @@
         <v>4</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>3</v>
@@ -2322,7 +2316,7 @@
         <v>3</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>4</v>
@@ -2356,43 +2350,43 @@
         <v>5</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>1</v>
@@ -2421,10 +2415,10 @@
         <v>2</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>3</v>
@@ -2445,7 +2439,7 @@
         <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>6</v>
@@ -2454,10 +2448,10 @@
         <v>6</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>2</v>
@@ -2488,37 +2482,37 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="N10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="O10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>7</v>
@@ -2555,46 +2549,46 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>40</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="K11" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="O11" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="M11" s="10" t="n">
+      <c r="P11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="S11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="T11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="U11" s="10" t="n">
         <v>44</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>45</v>
       </c>
     </row>
     <row r="12">
@@ -2622,46 +2616,46 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="K12" s="8" t="n">
         <v>97</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="N12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="P12" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="O12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="Q12" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="R12" s="8" t="n">
         <v>106</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-17)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-16</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -1950,7 +1950,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-16</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-18)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-17</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-18</t>
         </is>
       </c>
     </row>
@@ -1950,7 +1950,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-17</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-19)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-18</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-19</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>7</v>
@@ -685,32 +685,32 @@
         <v>7</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="Q4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="R4" s="4" t="inlineStr"/>
+      <c r="Q4" s="4" t="inlineStr"/>
+      <c r="R4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -743,46 +743,46 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>20</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="Q5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="R5" s="6" t="n">
-        <v>17</v>
-      </c>
       <c r="S5" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="U5" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="V5" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -815,46 +815,46 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J6" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="J6" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="K6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="N6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="O6" s="4" t="n">
+      <c r="P6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="P6" s="4" t="n">
+      <c r="U6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="V6" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="V6" s="4" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -887,46 +887,46 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="J7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="P7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="K7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="Q7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -959,41 +959,41 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="L8" s="4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="K8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="M8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>3</v>
@@ -1025,25 +1025,25 @@
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>2</v>
@@ -1052,19 +1052,19 @@
         <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1097,25 +1097,25 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>1</v>
@@ -1124,16 +1124,16 @@
         <v>1</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>3</v>
@@ -1175,40 +1175,40 @@
         <v>5</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>5</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -1237,47 +1237,45 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="V12" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="V12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1309,46 +1307,46 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -1387,37 +1385,37 @@
         <v>2</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>3</v>
@@ -1453,43 +1451,43 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="K15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="M15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="L15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="N15" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>7</v>
@@ -1564,7 +1562,7 @@
         <v>1</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K17" s="6" t="n">
         <v>3</v>
@@ -1576,7 +1574,7 @@
         <v>3</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O17" s="6" t="n">
         <v>2</v>
@@ -1585,19 +1583,19 @@
         <v>2</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S17" s="6" t="n">
         <v>4</v>
       </c>
       <c r="T17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V17" s="6" t="n">
         <v>2</v>
@@ -1628,10 +1626,10 @@
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
-      <c r="Q18" s="4" t="inlineStr"/>
-      <c r="R18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="Q18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
@@ -1670,16 +1668,16 @@
         <v>4</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N19" s="6" t="n">
         <v>5</v>
@@ -1691,19 +1689,19 @@
         <v>5</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="V19" s="6" t="n">
         <v>2</v>
@@ -1738,15 +1736,15 @@
       <c r="J20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="K20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>1</v>
@@ -1758,14 +1756,14 @@
         <v>1</v>
       </c>
       <c r="R20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S20" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="S20" s="4" t="inlineStr"/>
       <c r="T20" s="4" t="inlineStr"/>
       <c r="U20" s="4" t="inlineStr"/>
-      <c r="V20" s="4" t="inlineStr"/>
+      <c r="V20" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1800,40 +1798,40 @@
         <v>12</v>
       </c>
       <c r="J21" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="L21" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="K21" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="L21" s="6" t="n">
+      <c r="M21" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="N21" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="M21" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="N21" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="O21" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>22</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="T21" s="6" t="n">
         <v>13</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>16</v>
@@ -1865,43 +1863,43 @@
         <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="K22" s="8" t="n">
         <v>97</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="M22" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="N22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="O22" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="P22" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="O22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="P22" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="Q22" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="R22" s="8" t="n">
         <v>106</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="V22" s="8" t="n">
         <v>95</v>
@@ -1950,7 +1948,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-18</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1992,72 +1990,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2086,13 +2084,13 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>14</v>
@@ -2101,28 +2099,28 @@
         <v>14</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="O4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="R4" s="4" t="n">
+      <c r="S4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="S4" s="4" t="n">
-        <v>16</v>
-      </c>
       <c r="T4" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>15</v>
@@ -2153,28 +2151,28 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>17</v>
@@ -2186,10 +2184,10 @@
         <v>17</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>13</v>
@@ -2220,22 +2218,22 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>3</v>
@@ -2244,19 +2242,19 @@
         <v>3</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>3</v>
@@ -2293,10 +2291,10 @@
         <v>2</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>4</v>
@@ -2305,7 +2303,7 @@
         <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>3</v>
@@ -2317,7 +2315,7 @@
         <v>3</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>4</v>
@@ -2354,40 +2352,40 @@
         <v>5</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>1</v>
@@ -2419,7 +2417,7 @@
         <v>2</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>3</v>
@@ -2440,7 +2438,7 @@
         <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>6</v>
@@ -2449,13 +2447,13 @@
         <v>6</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>3</v>
@@ -2486,43 +2484,43 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="M10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="N10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="P10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="T10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>10</v>
@@ -2556,40 +2554,40 @@
         <v>40</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="L11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="M11" s="10" t="n">
+      <c r="O11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="P11" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="N11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="P11" s="10" t="n">
+      <c r="Q11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="Q11" s="10" t="n">
+      <c r="T11" s="10" t="n">
         <v>46</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>45</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>46</v>
@@ -2620,43 +2618,43 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J12" s="8" t="n">
         <v>97</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="M12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="O12" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="N12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="P12" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="Q12" s="8" t="n">
         <v>106</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="U12" s="8" t="n">
         <v>95</v>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-20)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -527,7 +527,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-19</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-20</t>
         </is>
       </c>
     </row>
@@ -574,72 +574,72 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -682,32 +682,32 @@
         <v>7</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="P4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q4" s="4" t="inlineStr"/>
+      <c r="P4" s="4" t="inlineStr"/>
+      <c r="Q4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="R4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>3</v>
@@ -743,40 +743,40 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>20</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="P5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q5" s="6" t="n">
-        <v>17</v>
-      </c>
       <c r="R5" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>9</v>
@@ -815,46 +815,46 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="K6" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="U6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="L6" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="U6" s="4" t="n">
-        <v>16</v>
-      </c>
       <c r="V6" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -887,46 +887,46 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="O7" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="J7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="P7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="S7" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="U7" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="V7" s="6" t="n">
         <v>12</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="V7" s="6" t="n">
-        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -959,44 +959,44 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K8" s="4" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="L8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -1025,43 +1025,43 @@
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="S9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="L9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="M9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="O9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="R9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="S9" s="6" t="n">
-        <v>4</v>
-      </c>
       <c r="T9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>4</v>
@@ -1097,22 +1097,22 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>1</v>
@@ -1121,22 +1121,22 @@
         <v>1</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1172,43 +1172,43 @@
         <v>5</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="M11" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="S11" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="N11" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="T11" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -1240,40 +1240,40 @@
         <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V12" s="4" t="n">
         <v>2</v>
@@ -1309,43 +1309,43 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>3</v>
@@ -1384,37 +1384,37 @@
         <v>2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>3</v>
@@ -1453,46 +1453,46 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="J15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="L15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="K15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="M15" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="N15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="O15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>2</v>
-      </c>
       <c r="R15" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -1561,7 +1561,7 @@
         <v>2</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>3</v>
@@ -1573,7 +1573,7 @@
         <v>3</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>2</v>
@@ -1582,25 +1582,25 @@
         <v>2</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R17" s="6" t="n">
         <v>4</v>
       </c>
       <c r="S17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
@@ -1627,10 +1627,10 @@
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
-      <c r="P18" s="4" t="inlineStr"/>
-      <c r="Q18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="P18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
       <c r="T18" s="4" t="inlineStr"/>
@@ -1667,47 +1667,45 @@
         <v>5</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P19" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R19" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="M19" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N19" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O19" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P19" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q19" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="R19" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="S19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="V19" s="6" t="n">
-        <v>3</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="V19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1735,15 +1733,15 @@
       <c r="I20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="J20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>1</v>
@@ -1755,17 +1753,15 @@
         <v>1</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R20" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="R20" s="4" t="inlineStr"/>
       <c r="S20" s="4" t="inlineStr"/>
       <c r="T20" s="4" t="inlineStr"/>
-      <c r="U20" s="4" t="inlineStr"/>
-      <c r="V20" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="U20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="V20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1797,46 +1793,46 @@
         <v>11</v>
       </c>
       <c r="I21" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="K21" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="J21" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="K21" s="6" t="n">
+      <c r="L21" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="M21" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="L21" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="M21" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="N21" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="P21" s="6" t="n">
         <v>22</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="S21" s="6" t="n">
         <v>13</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22">
@@ -1865,46 +1861,46 @@
         <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J22" s="8" t="n">
         <v>97</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="M22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="N22" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="O22" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="N22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="O22" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="P22" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="Q22" s="8" t="n">
         <v>106</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="U22" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="V22" s="8" t="n">
         <v>95</v>
-      </c>
-      <c r="V22" s="8" t="n">
-        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1950,7 +1946,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-19</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-20</t>
         </is>
       </c>
     </row>
@@ -1992,72 +1988,72 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -2086,10 +2082,10 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>14</v>
@@ -2098,34 +2094,34 @@
         <v>14</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="N4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="P4" s="4" t="n">
+      <c r="R4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="T4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="U4" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -2153,25 +2149,25 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>17</v>
@@ -2183,13 +2179,13 @@
         <v>17</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>12</v>
@@ -2220,19 +2216,19 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>3</v>
@@ -2241,19 +2237,19 @@
         <v>3</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>3</v>
@@ -2290,10 +2286,10 @@
         <v>2</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>4</v>
@@ -2302,7 +2298,7 @@
         <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>3</v>
@@ -2314,7 +2310,7 @@
         <v>3</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>4</v>
@@ -2354,37 +2350,37 @@
         <v>5</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>1</v>
@@ -2437,7 +2433,7 @@
         <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>6</v>
@@ -2446,19 +2442,19 @@
         <v>6</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -2486,46 +2482,46 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>8</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="L10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="M10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="O10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="S10" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="P10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="T10" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="U10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="11">
@@ -2553,46 +2549,46 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="M11" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="L11" s="10" t="n">
+      <c r="N11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="O11" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="M11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="O11" s="10" t="n">
+      <c r="P11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="R11" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="P11" s="10" t="n">
+      <c r="S11" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="Q11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>45</v>
-      </c>
       <c r="T11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="U11" s="10" t="n">
         <v>46</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>50</v>
       </c>
     </row>
     <row r="12">
@@ -2620,46 +2616,46 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I12" s="8" t="n">
         <v>97</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="L12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="N12" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="M12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="O12" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="P12" s="8" t="n">
         <v>106</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="T12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="U12" s="8" t="n">
         <v>95</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-21)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V22"/>
+  <dimension ref="A1:W22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -522,12 +522,13 @@
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-20</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-21</t>
         </is>
       </c>
     </row>
@@ -642,6 +643,11 @@
           <t>2026-10-20</t>
         </is>
       </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -712,6 +718,9 @@
       <c r="V4" s="4" t="n">
         <v>2</v>
       </c>
+      <c r="W4" s="4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -784,6 +793,9 @@
       <c r="V5" s="6" t="n">
         <v>9</v>
       </c>
+      <c r="W5" s="6" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -856,6 +868,9 @@
       <c r="V6" s="4" t="n">
         <v>12</v>
       </c>
+      <c r="W6" s="4" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -928,6 +943,9 @@
       <c r="V7" s="6" t="n">
         <v>13</v>
       </c>
+      <c r="W7" s="6" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -997,6 +1015,9 @@
       </c>
       <c r="V8" s="4" t="n">
         <v>5</v>
+      </c>
+      <c r="W8" s="4" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -1066,6 +1087,9 @@
       <c r="V9" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="W9" s="6" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1138,6 +1162,9 @@
       <c r="V10" s="4" t="n">
         <v>5</v>
       </c>
+      <c r="W10" s="4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1209,6 +1236,9 @@
       </c>
       <c r="V11" s="6" t="n">
         <v>7</v>
+      </c>
+      <c r="W11" s="6" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -1276,6 +1306,9 @@
         <v>2</v>
       </c>
       <c r="V12" s="4" t="inlineStr"/>
+      <c r="W12" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1348,6 +1381,9 @@
       <c r="V13" s="6" t="n">
         <v>6</v>
       </c>
+      <c r="W13" s="6" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1420,6 +1456,9 @@
       <c r="V14" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="W14" s="4" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1490,6 +1529,9 @@
         <v>8</v>
       </c>
       <c r="V15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="W15" s="6" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1530,6 +1572,7 @@
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
+      <c r="W16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1598,6 +1641,9 @@
         <v>3</v>
       </c>
       <c r="V17" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="W17" s="6" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1634,6 +1680,7 @@
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
+      <c r="W18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1706,6 +1753,7 @@
       <c r="V19" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="W19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1762,6 +1810,7 @@
         <v>2</v>
       </c>
       <c r="V20" s="4" t="inlineStr"/>
+      <c r="W20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1833,6 +1882,9 @@
       </c>
       <c r="V21" s="6" t="n">
         <v>19</v>
+      </c>
+      <c r="W21" s="6" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="22">
@@ -1902,10 +1954,13 @@
       <c r="V22" s="8" t="n">
         <v>97</v>
       </c>
+      <c r="W22" s="8" t="n">
+        <v>96</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A1:W1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1917,7 +1972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1941,12 +1996,13 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-20</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2056,6 +2112,11 @@
           <t>2026-10-20</t>
         </is>
       </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -2123,6 +2184,9 @@
       <c r="U4" s="4" t="n">
         <v>17</v>
       </c>
+      <c r="V4" s="4" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2190,6 +2254,9 @@
       <c r="U5" s="6" t="n">
         <v>13</v>
       </c>
+      <c r="V5" s="6" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2257,6 +2324,9 @@
       <c r="U6" s="4" t="n">
         <v>2</v>
       </c>
+      <c r="V6" s="4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2324,6 +2394,9 @@
       <c r="U7" s="6" t="n">
         <v>5</v>
       </c>
+      <c r="V7" s="6" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -2391,6 +2464,9 @@
       <c r="U8" s="4" t="n">
         <v>3</v>
       </c>
+      <c r="V8" s="4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2456,6 +2532,9 @@
       <c r="U9" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="V9" s="6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -2523,6 +2602,9 @@
       <c r="U10" s="4" t="n">
         <v>10</v>
       </c>
+      <c r="V10" s="4" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -2590,6 +2672,9 @@
       <c r="U11" s="10" t="n">
         <v>45</v>
       </c>
+      <c r="V11" s="10" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -2657,10 +2742,13 @@
       <c r="U12" s="8" t="n">
         <v>97</v>
       </c>
+      <c r="V12" s="8" t="n">
+        <v>96</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A1:V1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-22)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-21</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-22</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -685,41 +685,41 @@
         <v>7</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="O4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="P4" s="4" t="inlineStr"/>
+      <c r="O4" s="4" t="inlineStr"/>
+      <c r="P4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="W4" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -752,37 +752,37 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>20</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="O5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>17</v>
-      </c>
       <c r="Q5" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>9</v>
@@ -827,46 +827,46 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="T6" s="4" t="n">
         <v>12</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="T6" s="4" t="n">
-        <v>16</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>13</v>
@@ -902,46 +902,46 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S7" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="U7" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="T7" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="V7" s="6" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>6</v>
@@ -976,48 +976,48 @@
       <c r="H8" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="K8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="N8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>8</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -1046,19 +1046,19 @@
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>2</v>
@@ -1067,28 +1067,28 @@
         <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1121,19 +1121,19 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>1</v>
@@ -1142,28 +1142,28 @@
         <v>1</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -1196,46 +1196,46 @@
         <v>5</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="P11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="T11" s="6" t="n">
         <v>7</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>5</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>10</v>
@@ -1267,46 +1267,46 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="U12" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="U12" s="4" t="inlineStr"/>
       <c r="V12" s="4" t="inlineStr"/>
-      <c r="W12" s="4" t="inlineStr"/>
+      <c r="W12" s="4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1341,46 +1341,46 @@
         <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -1413,37 +1413,37 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>3</v>
@@ -1452,10 +1452,10 @@
         <v>3</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -1488,43 +1488,43 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="K15" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="J15" s="6" t="n">
+      <c r="L15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="K15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="R15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="S15" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="S15" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="T15" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V15" s="6" t="n">
         <v>6</v>
@@ -1609,7 +1609,7 @@
         <v>3</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M17" s="6" t="n">
         <v>2</v>
@@ -1618,22 +1618,22 @@
         <v>2</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>4</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U17" s="6" t="n">
         <v>3</v>
@@ -1668,10 +1668,10 @@
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
-      <c r="O18" s="4" t="inlineStr"/>
-      <c r="P18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="O18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
@@ -1710,13 +1710,13 @@
         <v>5</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>5</v>
@@ -1728,30 +1728,30 @@
         <v>5</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U19" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="V19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="W19" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="V19" s="6" t="inlineStr"/>
+      <c r="W19" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1776,15 +1776,15 @@
       <c r="H20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M20" s="4" t="n">
         <v>1</v>
@@ -1796,17 +1796,15 @@
         <v>1</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q20" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="Q20" s="4" t="inlineStr"/>
       <c r="R20" s="4" t="inlineStr"/>
       <c r="S20" s="4" t="inlineStr"/>
-      <c r="T20" s="4" t="inlineStr"/>
-      <c r="U20" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="T20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="U20" s="4" t="inlineStr"/>
       <c r="V20" s="4" t="inlineStr"/>
       <c r="W20" s="4" t="inlineStr"/>
     </row>
@@ -1840,40 +1838,40 @@
         <v>11</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="J21" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="L21" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="K21" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="L21" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="M21" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="O21" s="6" t="n">
         <v>22</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="R21" s="6" t="n">
         <v>13</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="U21" s="6" t="n">
         <v>19</v>
@@ -1882,7 +1880,7 @@
         <v>19</v>
       </c>
       <c r="W21" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22">
@@ -1914,46 +1912,46 @@
         <v>97</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="L22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="M22" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="N22" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="M22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="N22" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="O22" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="P22" s="8" t="n">
         <v>106</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="V22" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="W22" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="W22" s="8" t="n">
-        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2000,7 +1998,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-21</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-22</t>
         </is>
       </c>
     </row>
@@ -2042,77 +2040,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2139,7 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I4" s="4" t="n">
         <v>14</v>
@@ -2150,34 +2148,34 @@
         <v>14</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="M4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="N4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="O4" s="4" t="n">
+      <c r="Q4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="S4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="T4" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>17</v>
@@ -2214,19 +2212,19 @@
         <v>17</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>17</v>
@@ -2238,22 +2236,22 @@
         <v>17</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="S5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="T5" s="6" t="n">
+      <c r="U5" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="U5" s="6" t="n">
+      <c r="V5" s="6" t="n">
         <v>13</v>
-      </c>
-      <c r="V5" s="6" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -2284,13 +2282,13 @@
         <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>3</v>
@@ -2299,31 +2297,31 @@
         <v>3</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -2351,10 +2349,10 @@
         <v>3</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>4</v>
@@ -2363,7 +2361,7 @@
         <v>4</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>3</v>
@@ -2375,7 +2373,7 @@
         <v>3</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>4</v>
@@ -2387,7 +2385,7 @@
         <v>4</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>5</v>
@@ -2424,31 +2422,31 @@
         <v>5</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>1</v>
@@ -2457,7 +2455,7 @@
         <v>1</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>3</v>
@@ -2504,7 +2502,7 @@
         <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>6</v>
@@ -2513,19 +2511,19 @@
         <v>6</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>2</v>
@@ -2562,25 +2560,25 @@
         <v>8</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="K10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="L10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>7</v>
@@ -2589,13 +2587,13 @@
         <v>7</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S10" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="T10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>12</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>10</v>
@@ -2629,49 +2627,49 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="L11" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="J11" s="10" t="n">
+      <c r="M11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="S11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="T11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="U11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="K11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="N11" s="10" t="n">
+      <c r="V11" s="10" t="n">
         <v>45</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="V11" s="10" t="n">
-        <v>44</v>
       </c>
     </row>
     <row r="12">
@@ -2702,46 +2700,46 @@
         <v>97</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="K12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="M12" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="L12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="N12" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="O12" s="8" t="n">
         <v>106</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="U12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="V12" s="8" t="n">
         <v>97</v>
-      </c>
-      <c r="V12" s="8" t="n">
-        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-23)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-22</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-23</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -682,35 +682,35 @@
         <v>7</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="N4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="O4" s="4" t="inlineStr"/>
+      <c r="N4" s="4" t="inlineStr"/>
+      <c r="O4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="P4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>2</v>
@@ -719,7 +719,7 @@
         <v>2</v>
       </c>
       <c r="W4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -752,34 +752,34 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>16</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>20</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="N5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="O5" s="6" t="n">
-        <v>17</v>
-      </c>
       <c r="P5" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>9</v>
@@ -794,7 +794,7 @@
         <v>9</v>
       </c>
       <c r="W5" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -827,49 +827,49 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="S6" s="4" t="n">
         <v>12</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="R6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="S6" s="4" t="n">
-        <v>16</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="W6" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -902,49 +902,49 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R7" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="T7" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="S7" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="U7" s="6" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="W7" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -976,48 +976,50 @@
       <c r="H8" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="I8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="J8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="M8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>8</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>8</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -1046,16 +1048,16 @@
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>2</v>
@@ -1064,31 +1066,31 @@
         <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -1121,16 +1123,16 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>1</v>
@@ -1139,28 +1141,28 @@
         <v>1</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>3</v>
@@ -1196,49 +1198,49 @@
         <v>5</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>6</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="O11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="S11" s="6" t="n">
         <v>7</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>5</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>10</v>
       </c>
       <c r="W11" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
@@ -1267,43 +1269,43 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="T12" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="T12" s="4" t="inlineStr"/>
       <c r="U12" s="4" t="inlineStr"/>
-      <c r="V12" s="4" t="inlineStr"/>
+      <c r="V12" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="W12" s="4" t="n">
         <v>4</v>
       </c>
@@ -1338,49 +1340,49 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -1416,31 +1418,31 @@
         <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>3</v>
@@ -1449,7 +1451,7 @@
         <v>3</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>5</v>
@@ -1488,46 +1490,46 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="P15" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="J15" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="K15" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="L15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="M15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="N15" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="O15" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="P15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="Q15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R15" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="R15" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="S15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="U15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="V15" s="6" t="n">
         <v>7</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>6</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>7</v>
@@ -1606,7 +1608,7 @@
         <v>3</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L17" s="6" t="n">
         <v>2</v>
@@ -1615,22 +1617,22 @@
         <v>2</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P17" s="6" t="n">
         <v>4</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T17" s="6" t="n">
         <v>3</v>
@@ -1642,7 +1644,7 @@
         <v>3</v>
       </c>
       <c r="W17" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1667,10 +1669,10 @@
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="inlineStr"/>
-      <c r="O18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="N18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
@@ -1710,10 +1712,10 @@
         <v>5</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K19" s="6" t="n">
         <v>5</v>
@@ -1725,33 +1727,31 @@
         <v>5</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T19" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="U19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="V19" s="6" t="inlineStr"/>
-      <c r="W19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="U19" s="6" t="inlineStr"/>
+      <c r="V19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="W19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1776,12 +1776,14 @@
       <c r="H20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L20" s="4" t="n">
         <v>1</v>
@@ -1793,20 +1795,20 @@
         <v>1</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P20" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="P20" s="4" t="inlineStr"/>
       <c r="Q20" s="4" t="inlineStr"/>
       <c r="R20" s="4" t="inlineStr"/>
-      <c r="S20" s="4" t="inlineStr"/>
-      <c r="T20" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="S20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T20" s="4" t="inlineStr"/>
       <c r="U20" s="4" t="inlineStr"/>
       <c r="V20" s="4" t="inlineStr"/>
-      <c r="W20" s="4" t="inlineStr"/>
+      <c r="W20" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1838,37 +1840,37 @@
         <v>11</v>
       </c>
       <c r="I21" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="K21" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="J21" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="K21" s="6" t="n">
-        <v>11</v>
-      </c>
       <c r="L21" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>22</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>13</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="T21" s="6" t="n">
         <v>19</v>
@@ -1880,7 +1882,7 @@
         <v>19</v>
       </c>
       <c r="W21" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22">
@@ -1909,49 +1911,49 @@
         <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="K22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="L22" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="M22" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="L22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="M22" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="N22" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="O22" s="8" t="n">
         <v>106</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="U22" s="8" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="V22" s="8" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="W22" s="8" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -1998,7 +2000,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-22</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-23</t>
         </is>
       </c>
     </row>
@@ -2040,77 +2042,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -2145,43 +2147,43 @@
         <v>14</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="L4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="N4" s="4" t="n">
+      <c r="P4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="R4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="S4" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -2209,19 +2211,19 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>17</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>14</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>17</v>
@@ -2233,22 +2235,22 @@
         <v>17</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="R5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="S5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="S5" s="6" t="n">
+      <c r="T5" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="T5" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="U5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>14</v>
@@ -2279,13 +2281,13 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>3</v>
@@ -2294,31 +2296,31 @@
         <v>3</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>2</v>
@@ -2349,7 +2351,7 @@
         <v>3</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>4</v>
@@ -2358,7 +2360,7 @@
         <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>3</v>
@@ -2370,7 +2372,7 @@
         <v>3</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>4</v>
@@ -2382,7 +2384,7 @@
         <v>4</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>5</v>
@@ -2419,31 +2421,31 @@
         <v>5</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>1</v>
@@ -2452,7 +2454,7 @@
         <v>1</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>3</v>
@@ -2461,7 +2463,7 @@
         <v>3</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -2499,7 +2501,7 @@
         <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>6</v>
@@ -2508,25 +2510,25 @@
         <v>6</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>1</v>
@@ -2557,25 +2559,25 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="J10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>7</v>
@@ -2584,13 +2586,13 @@
         <v>7</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="R10" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="S10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>12</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>10</v>
@@ -2627,49 +2629,49 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="K11" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="I11" s="10" t="n">
+      <c r="L11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="S11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="T11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>43</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="O11" s="10" t="n">
+      <c r="U11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="V11" s="10" t="n">
         <v>47</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="V11" s="10" t="n">
-        <v>48</v>
       </c>
     </row>
     <row r="12">
@@ -2697,49 +2699,49 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="J12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="L12" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="K12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="M12" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>106</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="U12" s="8" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="V12" s="8" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-24)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-23</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-24</t>
         </is>
       </c>
     </row>
@@ -1998,7 +1998,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-23</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-25)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-24</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-25</t>
         </is>
       </c>
     </row>
@@ -1998,7 +1998,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-24</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-26)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-25</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-26</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -679,35 +679,35 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="N4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr"/>
+      <c r="N4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="O4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>2</v>
@@ -716,7 +716,7 @@
         <v>2</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>5</v>
@@ -752,31 +752,31 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="L5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="M5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="N5" s="6" t="n">
-        <v>17</v>
-      </c>
       <c r="O5" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>9</v>
@@ -791,10 +791,10 @@
         <v>9</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="W5" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -827,49 +827,49 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="L6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="L6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="M6" s="4" t="n">
+      <c r="Q6" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="N6" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>15</v>
-      </c>
       <c r="R6" s="4" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="W6" s="4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
@@ -902,46 +902,46 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q7" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="S7" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="R7" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>14</v>
-      </c>
       <c r="T7" s="6" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>5</v>
@@ -977,40 +977,40 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O8" s="4" t="n">
         <v>7</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>8</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>8</v>
@@ -1019,7 +1019,7 @@
         <v>8</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -1048,13 +1048,13 @@
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>2</v>
@@ -1063,34 +1063,34 @@
         <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1123,13 +1123,13 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>1</v>
@@ -1138,34 +1138,34 @@
         <v>1</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1201,46 +1201,46 @@
         <v>6</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="N11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="R11" s="6" t="n">
         <v>7</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>5</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>10</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="W11" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -1269,42 +1269,42 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S12" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="S12" s="4" t="inlineStr"/>
       <c r="T12" s="4" t="inlineStr"/>
-      <c r="U12" s="4" t="inlineStr"/>
+      <c r="U12" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="V12" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>7</v>
@@ -1340,49 +1340,49 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -1415,31 +1415,31 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>3</v>
@@ -1448,7 +1448,7 @@
         <v>3</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>5</v>
@@ -1457,7 +1457,7 @@
         <v>5</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15">
@@ -1490,46 +1490,46 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q15" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="Q15" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="R15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="S15" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>6</v>
-      </c>
       <c r="V15" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>5</v>
@@ -1605,7 +1605,7 @@
         <v>3</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K17" s="6" t="n">
         <v>2</v>
@@ -1614,22 +1614,22 @@
         <v>2</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O17" s="6" t="n">
         <v>4</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S17" s="6" t="n">
         <v>3</v>
@@ -1640,9 +1640,7 @@
       <c r="U17" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="V17" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1666,10 +1664,10 @@
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="M18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
@@ -1710,7 +1708,7 @@
         <v>5</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>5</v>
@@ -1722,33 +1720,31 @@
         <v>5</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S19" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="T19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="U19" s="6" t="inlineStr"/>
-      <c r="V19" s="6" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="T19" s="6" t="inlineStr"/>
+      <c r="U19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="V19" s="6" t="inlineStr"/>
       <c r="W19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1775,10 +1771,10 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" s="4" t="n">
         <v>1</v>
@@ -1790,20 +1786,20 @@
         <v>1</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O20" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O20" s="4" t="inlineStr"/>
       <c r="P20" s="4" t="inlineStr"/>
       <c r="Q20" s="4" t="inlineStr"/>
-      <c r="R20" s="4" t="inlineStr"/>
-      <c r="S20" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="R20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S20" s="4" t="inlineStr"/>
       <c r="T20" s="4" t="inlineStr"/>
       <c r="U20" s="4" t="inlineStr"/>
-      <c r="V20" s="4" t="inlineStr"/>
+      <c r="V20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="W20" s="4" t="n">
         <v>1</v>
       </c>
@@ -1838,34 +1834,34 @@
         <v>11</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>22</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="P21" s="6" t="n">
         <v>13</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="S21" s="6" t="n">
         <v>19</v>
@@ -1877,10 +1873,10 @@
         <v>19</v>
       </c>
       <c r="V21" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="W21" s="6" t="n">
         <v>19</v>
-      </c>
-      <c r="W21" s="6" t="n">
-        <v>18</v>
       </c>
     </row>
     <row r="22">
@@ -1909,49 +1905,49 @@
         <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="J22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="K22" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="L22" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="K22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="L22" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="M22" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="N22" s="8" t="n">
         <v>106</v>
       </c>
       <c r="O22" s="8" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="Q22" s="8" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="S22" s="8" t="n">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="U22" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="V22" s="8" t="n">
         <v>96</v>
       </c>
-      <c r="V22" s="8" t="n">
+      <c r="W22" s="8" t="n">
         <v>99</v>
-      </c>
-      <c r="W22" s="8" t="n">
-        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1998,7 +1994,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-25</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2040,77 +2036,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -2142,40 +2138,40 @@
         <v>14</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="M4" s="4" t="n">
+      <c r="O4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="R4" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>16</v>
@@ -2209,16 +2205,16 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="L5" s="6" t="n">
         <v>17</v>
@@ -2230,28 +2226,28 @@
         <v>17</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="Q5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="R5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="R5" s="6" t="n">
+      <c r="S5" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="S5" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="T5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -2279,10 +2275,10 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>3</v>
@@ -2291,31 +2287,31 @@
         <v>3</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>2</v>
@@ -2355,7 +2351,7 @@
         <v>4</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>3</v>
@@ -2367,7 +2363,7 @@
         <v>3</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>4</v>
@@ -2379,7 +2375,7 @@
         <v>4</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>5</v>
@@ -2422,25 +2418,25 @@
         <v>7</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>1</v>
@@ -2449,7 +2445,7 @@
         <v>1</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>3</v>
@@ -2458,7 +2454,7 @@
         <v>3</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>4</v>
@@ -2496,7 +2492,7 @@
         <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>6</v>
@@ -2505,28 +2501,28 @@
         <v>6</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>3</v>
@@ -2560,19 +2556,19 @@
         <v>10</v>
       </c>
       <c r="I10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>7</v>
@@ -2581,13 +2577,13 @@
         <v>7</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="Q10" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="R10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>12</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>10</v>
@@ -2596,10 +2592,10 @@
         <v>10</v>
       </c>
       <c r="U10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="V10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="V10" s="4" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -2627,49 +2623,49 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="I11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="I11" s="10" t="n">
+      <c r="J11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="L11" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="J11" s="10" t="n">
+      <c r="M11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="R11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="K11" s="10" t="n">
+      <c r="T11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="U11" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="L11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>48</v>
-      </c>
       <c r="V11" s="10" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12">
@@ -2697,49 +2693,49 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="K12" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="J12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="L12" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="M12" s="8" t="n">
         <v>106</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="Q12" s="8" t="n">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="S12" s="8" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="T12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="U12" s="8" t="n">
         <v>96</v>
       </c>
-      <c r="U12" s="8" t="n">
+      <c r="V12" s="8" t="n">
         <v>99</v>
-      </c>
-      <c r="V12" s="8" t="n">
-        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-27)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-26</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-27</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -679,32 +679,32 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="M4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>2</v>
@@ -713,10 +713,10 @@
         <v>2</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>7</v>
@@ -752,28 +752,28 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>16</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="M5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="L5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="M5" s="6" t="n">
-        <v>17</v>
-      </c>
       <c r="N5" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>9</v>
@@ -788,13 +788,13 @@
         <v>9</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W5" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -827,46 +827,46 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="J6" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="K6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="K6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="L6" s="4" t="n">
+      <c r="P6" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>15</v>
-      </c>
       <c r="Q6" s="4" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="W6" s="4" t="n">
         <v>18</v>
@@ -902,49 +902,49 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="M7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="U7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="V7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="N7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="V7" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="W7" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -977,37 +977,37 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="N8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="S8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>8</v>
@@ -1016,10 +1016,10 @@
         <v>8</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -1048,10 +1048,10 @@
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>2</v>
@@ -1060,37 +1060,37 @@
         <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1123,10 +1123,10 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
         <v>1</v>
@@ -1135,37 +1135,37 @@
         <v>1</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -1198,49 +1198,49 @@
         <v>5</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N11" s="6" t="n">
         <v>5</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>10</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="W11" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -1272,42 +1272,42 @@
         <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R12" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="R12" s="4" t="inlineStr"/>
       <c r="S12" s="4" t="inlineStr"/>
-      <c r="T12" s="4" t="inlineStr"/>
+      <c r="T12" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="U12" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -1343,46 +1343,46 @@
         <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -1415,28 +1415,28 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>3</v>
@@ -1445,7 +1445,7 @@
         <v>3</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T14" s="4" t="n">
         <v>5</v>
@@ -1457,7 +1457,7 @@
         <v>5</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -1490,49 +1490,49 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="S15" s="6" t="n">
         <v>6</v>
       </c>
       <c r="T15" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U15" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V15" s="6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="W15" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
@@ -1602,7 +1602,7 @@
         <v>2</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>2</v>
@@ -1611,22 +1611,22 @@
         <v>2</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N17" s="6" t="n">
         <v>4</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R17" s="6" t="n">
         <v>3</v>
@@ -1637,9 +1637,7 @@
       <c r="T17" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="U17" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="6" t="inlineStr"/>
     </row>
@@ -1663,10 +1661,10 @@
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="L18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
       <c r="P18" s="4" t="inlineStr"/>
@@ -1717,34 +1715,34 @@
         <v>5</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R19" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="S19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T19" s="6" t="inlineStr"/>
-      <c r="U19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="V19" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="S19" s="6" t="inlineStr"/>
+      <c r="T19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="U19" s="6" t="inlineStr"/>
+      <c r="V19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="W19" s="6" t="n">
         <v>1</v>
       </c>
@@ -1773,7 +1771,7 @@
         <v>1</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J20" s="4" t="n">
         <v>1</v>
@@ -1785,20 +1783,20 @@
         <v>1</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N20" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="N20" s="4" t="inlineStr"/>
       <c r="O20" s="4" t="inlineStr"/>
       <c r="P20" s="4" t="inlineStr"/>
-      <c r="Q20" s="4" t="inlineStr"/>
-      <c r="R20" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="Q20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R20" s="4" t="inlineStr"/>
       <c r="S20" s="4" t="inlineStr"/>
       <c r="T20" s="4" t="inlineStr"/>
-      <c r="U20" s="4" t="inlineStr"/>
+      <c r="U20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="V20" s="4" t="n">
         <v>1</v>
       </c>
@@ -1836,31 +1834,31 @@
         <v>11</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>22</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="O21" s="6" t="n">
         <v>13</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="R21" s="6" t="n">
         <v>19</v>
@@ -1872,10 +1870,10 @@
         <v>19</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="V21" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="W21" s="6" t="n">
         <v>21</v>
@@ -1907,49 +1905,49 @@
         <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="J22" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="K22" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="J22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="K22" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="L22" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="M22" s="8" t="n">
         <v>106</v>
       </c>
       <c r="N22" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="O22" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="P22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q22" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="R22" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="S22" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="T22" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="U22" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="V22" s="8" t="n">
         <v>106</v>
       </c>
-      <c r="O22" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="P22" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="Q22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="R22" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="S22" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="T22" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="U22" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="V22" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="W22" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -1996,7 +1994,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-26</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-27</t>
         </is>
       </c>
     </row>
@@ -2038,77 +2036,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -2137,46 +2135,46 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="L4" s="4" t="n">
+      <c r="N4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="Q4" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="V4" s="4" t="n">
         <v>20</v>
@@ -2207,13 +2205,13 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>17</v>
@@ -2225,31 +2223,31 @@
         <v>17</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="P5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="Q5" s="6" t="n">
+      <c r="R5" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="R5" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="S5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -2277,7 +2275,7 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>3</v>
@@ -2286,31 +2284,31 @@
         <v>3</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>2</v>
@@ -2350,7 +2348,7 @@
         <v>4</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>3</v>
@@ -2362,7 +2360,7 @@
         <v>3</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
         <v>4</v>
@@ -2374,7 +2372,7 @@
         <v>4</v>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R7" s="6" t="n">
         <v>5</v>
@@ -2386,7 +2384,7 @@
         <v>5</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V7" s="6" t="n">
         <v>6</v>
@@ -2417,25 +2415,25 @@
         <v>5</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>1</v>
@@ -2444,7 +2442,7 @@
         <v>1</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>3</v>
@@ -2453,13 +2451,13 @@
         <v>3</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -2491,7 +2489,7 @@
         <v>3</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>6</v>
@@ -2500,28 +2498,28 @@
         <v>6</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>3</v>
@@ -2555,34 +2553,34 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="I10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="K10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O10" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="L10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="P10" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>12</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>10</v>
@@ -2591,10 +2589,10 @@
         <v>10</v>
       </c>
       <c r="T10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="U10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>10</v>
@@ -2625,49 +2623,49 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="K11" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="I11" s="10" t="n">
+      <c r="L11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="R11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="J11" s="10" t="n">
+      <c r="S11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="T11" s="10" t="n">
         <v>43</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>48</v>
       </c>
       <c r="U11" s="10" t="n">
         <v>43</v>
       </c>
       <c r="V11" s="10" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12">
@@ -2695,49 +2693,49 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="J12" s="8" t="n">
         <v>108</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="J12" s="8" t="n">
-        <v>98</v>
-      </c>
       <c r="K12" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>106</v>
       </c>
       <c r="M12" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="T12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="U12" s="8" t="n">
         <v>106</v>
       </c>
-      <c r="N12" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>96</v>
-      </c>
       <c r="V12" s="8" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-28)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-27</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-28</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -679,29 +679,29 @@
         <v>7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="K4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="L4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="M4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>2</v>
@@ -710,13 +710,13 @@
         <v>2</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>3</v>
@@ -755,22 +755,22 @@
         <v>16</v>
       </c>
       <c r="J5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="K5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>17</v>
-      </c>
       <c r="M5" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P5" s="6" t="n">
         <v>9</v>
@@ -785,13 +785,13 @@
         <v>9</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="W5" s="6" t="n">
         <v>11</v>
@@ -827,43 +827,43 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="J6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="K6" s="4" t="n">
+      <c r="O6" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="L6" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>15</v>
-      </c>
       <c r="P6" s="4" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>18</v>
@@ -902,46 +902,46 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="U7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="M7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="V7" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W7" s="6" t="n">
         <v>7</v>
@@ -977,34 +977,34 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="R8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>8</v>
@@ -1013,7 +1013,7 @@
         <v>8</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>5</v>
@@ -1048,7 +1048,7 @@
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>2</v>
@@ -1057,40 +1057,40 @@
         <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1123,7 +1123,7 @@
         <v>7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>1</v>
@@ -1132,37 +1132,37 @@
         <v>1</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>5</v>
@@ -1198,46 +1198,46 @@
         <v>5</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>5</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S11" s="6" t="n">
         <v>10</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>2</v>
@@ -1269,45 +1269,45 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q12" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="Q12" s="4" t="inlineStr"/>
       <c r="R12" s="4" t="inlineStr"/>
-      <c r="S12" s="4" t="inlineStr"/>
+      <c r="S12" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="T12" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -1340,49 +1340,49 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="W13" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -1415,25 +1415,25 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>3</v>
@@ -1442,7 +1442,7 @@
         <v>3</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="S14" s="4" t="n">
         <v>5</v>
@@ -1454,10 +1454,10 @@
         <v>5</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -1490,46 +1490,46 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>4</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="U15" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="V15" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>10</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>8</v>
@@ -1608,22 +1608,22 @@
         <v>2</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M17" s="6" t="n">
         <v>4</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>3</v>
@@ -1634,9 +1634,7 @@
       <c r="S17" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="T17" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
       <c r="W17" s="6" t="inlineStr"/>
@@ -1660,10 +1658,10 @@
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="K18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
@@ -1712,34 +1710,34 @@
         <v>5</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="R19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S19" s="6" t="inlineStr"/>
-      <c r="T19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="U19" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="R19" s="6" t="inlineStr"/>
+      <c r="S19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="T19" s="6" t="inlineStr"/>
+      <c r="U19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="V19" s="6" t="n">
         <v>1</v>
       </c>
@@ -1780,20 +1778,20 @@
         <v>1</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M20" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="M20" s="4" t="inlineStr"/>
       <c r="N20" s="4" t="inlineStr"/>
       <c r="O20" s="4" t="inlineStr"/>
-      <c r="P20" s="4" t="inlineStr"/>
-      <c r="Q20" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="P20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q20" s="4" t="inlineStr"/>
       <c r="R20" s="4" t="inlineStr"/>
       <c r="S20" s="4" t="inlineStr"/>
-      <c r="T20" s="4" t="inlineStr"/>
+      <c r="T20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="U20" s="4" t="n">
         <v>1</v>
       </c>
@@ -1834,28 +1832,28 @@
         <v>11</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>22</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="N21" s="6" t="n">
         <v>13</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>19</v>
@@ -1867,16 +1865,16 @@
         <v>19</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="V21" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="W21" s="6" t="n">
         <v>21</v>
-      </c>
-      <c r="W21" s="6" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="22">
@@ -1905,49 +1903,49 @@
         <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>106</v>
       </c>
       <c r="M22" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="N22" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="O22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="P22" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="Q22" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="R22" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="S22" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="T22" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="U22" s="8" t="n">
         <v>106</v>
       </c>
-      <c r="N22" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="O22" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="P22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="Q22" s="8" t="n">
+      <c r="V22" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="R22" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="S22" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="T22" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="U22" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="V22" s="8" t="n">
-        <v>106</v>
-      </c>
       <c r="W22" s="8" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1994,7 +1992,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-27</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-28</t>
         </is>
       </c>
     </row>
@@ -2036,77 +2034,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -2135,43 +2133,43 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="K4" s="4" t="n">
+      <c r="M4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="O4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="P4" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="U4" s="4" t="n">
         <v>20</v>
@@ -2205,10 +2203,10 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>17</v>
@@ -2220,31 +2218,31 @@
         <v>17</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="O5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="P5" s="6" t="n">
+      <c r="Q5" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Q5" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="R5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>17</v>
@@ -2281,31 +2279,31 @@
         <v>3</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S6" s="4" t="n">
         <v>2</v>
@@ -2314,7 +2312,7 @@
         <v>2</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>3</v>
@@ -2345,7 +2343,7 @@
         <v>3</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I7" s="6" t="n">
         <v>3</v>
@@ -2357,7 +2355,7 @@
         <v>3</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>4</v>
@@ -2369,7 +2367,7 @@
         <v>4</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>5</v>
@@ -2381,7 +2379,7 @@
         <v>5</v>
       </c>
       <c r="T7" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U7" s="6" t="n">
         <v>6</v>
@@ -2415,22 +2413,22 @@
         <v>5</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>1</v>
@@ -2439,7 +2437,7 @@
         <v>1</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>3</v>
@@ -2448,13 +2446,13 @@
         <v>3</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>5</v>
@@ -2486,7 +2484,7 @@
         <v>3</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>6</v>
@@ -2495,28 +2493,28 @@
         <v>6</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>3</v>
@@ -2553,31 +2551,31 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>10</v>
       </c>
       <c r="J10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N10" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="K10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="O10" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="P10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>12</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>10</v>
@@ -2586,16 +2584,16 @@
         <v>10</v>
       </c>
       <c r="S10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="T10" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="T10" s="4" t="n">
+      <c r="U10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="U10" s="4" t="n">
+      <c r="V10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="V10" s="4" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -2623,49 +2621,49 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="Q11" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="I11" s="10" t="n">
+      <c r="R11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="S11" s="10" t="n">
         <v>43</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="S11" s="10" t="n">
-        <v>48</v>
       </c>
       <c r="T11" s="10" t="n">
         <v>43</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="V11" s="10" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12">
@@ -2693,49 +2691,49 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K12" s="8" t="n">
         <v>106</v>
       </c>
       <c r="L12" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="T12" s="8" t="n">
         <v>106</v>
       </c>
-      <c r="M12" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="P12" s="8" t="n">
+      <c r="U12" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="Q12" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>106</v>
-      </c>
       <c r="V12" s="8" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-29)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-28</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-29</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
@@ -681,24 +681,24 @@
       <c r="I4" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="L4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>2</v>
@@ -707,19 +707,19 @@
         <v>2</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="W4" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -752,22 +752,22 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="K5" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="J5" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="K5" s="6" t="n">
-        <v>17</v>
-      </c>
       <c r="L5" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="O5" s="6" t="n">
         <v>9</v>
@@ -782,19 +782,19 @@
         <v>9</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="W5" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -827,40 +827,40 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="M6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="N6" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="K6" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>15</v>
-      </c>
       <c r="O6" s="4" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>18</v>
@@ -869,7 +869,7 @@
         <v>18</v>
       </c>
       <c r="W6" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -902,49 +902,49 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="T7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="L7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="U7" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W7" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -977,31 +977,31 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q8" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>8</v>
@@ -1010,7 +1010,7 @@
         <v>8</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>5</v>
@@ -1019,7 +1019,7 @@
         <v>5</v>
       </c>
       <c r="W8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -1054,43 +1054,43 @@
         <v>2</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -1129,40 +1129,40 @@
         <v>1</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="W10" s="4" t="n">
         <v>2</v>
@@ -1198,43 +1198,43 @@
         <v>5</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>5</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="R11" s="6" t="n">
         <v>10</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V11" s="6" t="n">
         <v>2</v>
@@ -1269,42 +1269,42 @@
         <v>1</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P12" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="P12" s="4" t="inlineStr"/>
       <c r="Q12" s="4" t="inlineStr"/>
-      <c r="R12" s="4" t="inlineStr"/>
+      <c r="R12" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="S12" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="W12" s="4" t="n">
         <v>5</v>
@@ -1343,43 +1343,43 @@
         <v>5</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="R13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="W13" s="6" t="n">
         <v>8</v>
@@ -1418,19 +1418,19 @@
         <v>4</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>3</v>
@@ -1439,7 +1439,7 @@
         <v>3</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>5</v>
@@ -1451,13 +1451,13 @@
         <v>5</v>
       </c>
       <c r="U14" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V14" s="4" t="n">
         <v>7</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -1493,43 +1493,43 @@
         <v>4</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="T15" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="U15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="Q15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="V15" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>7</v>
@@ -1572,7 +1572,9 @@
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
       <c r="V16" s="4" t="inlineStr"/>
-      <c r="W16" s="4" t="inlineStr"/>
+      <c r="W16" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1605,22 +1607,22 @@
         <v>2</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L17" s="6" t="n">
         <v>4</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P17" s="6" t="n">
         <v>3</v>
@@ -1631,9 +1633,7 @@
       <c r="R17" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="S17" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
       <c r="V17" s="6" t="inlineStr"/>
@@ -1657,10 +1657,10 @@
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" s="4" t="inlineStr"/>
-      <c r="K18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
       <c r="N18" s="4" t="inlineStr"/>
@@ -1707,34 +1707,34 @@
         <v>5</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="R19" s="6" t="inlineStr"/>
-      <c r="S19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="T19" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Q19" s="6" t="inlineStr"/>
+      <c r="R19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S19" s="6" t="inlineStr"/>
+      <c r="T19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="U19" s="6" t="n">
         <v>1</v>
       </c>
@@ -1775,29 +1775,27 @@
         <v>1</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="4" t="inlineStr"/>
       <c r="N20" s="4" t="inlineStr"/>
-      <c r="O20" s="4" t="inlineStr"/>
-      <c r="P20" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="O20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P20" s="4" t="inlineStr"/>
       <c r="Q20" s="4" t="inlineStr"/>
       <c r="R20" s="4" t="inlineStr"/>
-      <c r="S20" s="4" t="inlineStr"/>
+      <c r="S20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="T20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="U20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="V20" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="V20" s="4" t="inlineStr"/>
       <c r="W20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
@@ -1830,25 +1828,25 @@
         <v>11</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>22</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>13</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="P21" s="6" t="n">
         <v>19</v>
@@ -1860,19 +1858,19 @@
         <v>19</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="T21" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="U21" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="V21" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="V21" s="6" t="n">
-        <v>20</v>
-      </c>
       <c r="W21" s="6" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22">
@@ -1901,49 +1899,49 @@
         <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K22" s="8" t="n">
         <v>106</v>
       </c>
       <c r="L22" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="M22" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="N22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="O22" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="P22" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="Q22" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="R22" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="S22" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="T22" s="8" t="n">
         <v>106</v>
       </c>
-      <c r="M22" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="N22" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="O22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="P22" s="8" t="n">
+      <c r="U22" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="Q22" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="R22" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="S22" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="T22" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="U22" s="8" t="n">
-        <v>106</v>
-      </c>
       <c r="V22" s="8" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="W22" s="8" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -1990,7 +1988,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-28</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-29</t>
         </is>
       </c>
     </row>
@@ -2032,77 +2030,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
     </row>
@@ -2131,40 +2129,40 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="I4" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="J4" s="4" t="n">
+      <c r="L4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="N4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="O4" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="T4" s="4" t="n">
         <v>20</v>
@@ -2173,7 +2171,7 @@
         <v>20</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
@@ -2201,7 +2199,7 @@
         <v>19</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="I5" s="6" t="n">
         <v>17</v>
@@ -2213,37 +2211,37 @@
         <v>17</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="N5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="O5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="O5" s="6" t="n">
+      <c r="P5" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="P5" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="Q5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="U5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -2274,31 +2272,31 @@
         <v>3</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>2</v>
@@ -2307,7 +2305,7 @@
         <v>2</v>
       </c>
       <c r="T6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
         <v>3</v>
@@ -2350,7 +2348,7 @@
         <v>3</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>4</v>
@@ -2362,7 +2360,7 @@
         <v>4</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P7" s="6" t="n">
         <v>5</v>
@@ -2374,7 +2372,7 @@
         <v>5</v>
       </c>
       <c r="S7" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>6</v>
@@ -2411,19 +2409,19 @@
         <v>5</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>1</v>
@@ -2432,7 +2430,7 @@
         <v>1</v>
       </c>
       <c r="O8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>3</v>
@@ -2441,19 +2439,19 @@
         <v>3</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="T8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="U8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="V8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -2479,7 +2477,7 @@
         <v>2</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>6</v>
@@ -2488,28 +2486,28 @@
         <v>6</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="S9" s="6" t="n">
         <v>3</v>
@@ -2518,7 +2516,7 @@
         <v>3</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>5</v>
@@ -2552,25 +2550,25 @@
         <v>10</v>
       </c>
       <c r="I10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M10" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="J10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="N10" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="O10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>12</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>10</v>
@@ -2579,16 +2577,16 @@
         <v>10</v>
       </c>
       <c r="R10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="S10" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="S10" s="4" t="n">
+      <c r="T10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="T10" s="4" t="n">
-        <v>10</v>
-      </c>
       <c r="U10" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="V10" s="4" t="n">
         <v>11</v>
@@ -2619,46 +2617,46 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="N11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="P11" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="Q11" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="R11" s="10" t="n">
         <v>43</v>
-      </c>
-      <c r="I11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="O11" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="P11" s="10" t="n">
-        <v>45</v>
-      </c>
-      <c r="Q11" s="10" t="n">
-        <v>44</v>
-      </c>
-      <c r="R11" s="10" t="n">
-        <v>48</v>
       </c>
       <c r="S11" s="10" t="n">
         <v>43</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="U11" s="10" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>38</v>
@@ -2689,49 +2687,49 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="J12" s="8" t="n">
         <v>106</v>
       </c>
       <c r="K12" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="S12" s="8" t="n">
         <v>106</v>
       </c>
-      <c r="L12" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="O12" s="8" t="n">
+      <c r="T12" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="P12" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="S12" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="T12" s="8" t="n">
-        <v>106</v>
-      </c>
       <c r="U12" s="8" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="V12" s="8" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-30)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-29</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-30</t>
         </is>
       </c>
     </row>
@@ -575,77 +575,77 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -678,24 +678,24 @@
       <c r="H4" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="I4" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>2</v>
@@ -704,22 +704,22 @@
         <v>2</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="T4" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W4" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -752,19 +752,19 @@
         <v>13</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N5" s="6" t="n">
         <v>9</v>
@@ -779,22 +779,22 @@
         <v>9</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T5" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="V5" s="6" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="W5" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -827,37 +827,37 @@
         <v>8</v>
       </c>
       <c r="I6" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="M6" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="J6" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>15</v>
-      </c>
       <c r="N6" s="4" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>12</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="R6" s="4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>18</v>
@@ -866,10 +866,10 @@
         <v>18</v>
       </c>
       <c r="V6" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="W6" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -902,49 +902,49 @@
         <v>8</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="S7" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="K7" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="M7" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="N7" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="O7" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>5</v>
-      </c>
       <c r="T7" s="6" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="U7" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="V7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="W7" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="W7" s="6" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -977,28 +977,28 @@
         <v>11</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>8</v>
@@ -1007,19 +1007,19 @@
         <v>8</v>
       </c>
       <c r="S8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="V8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="T8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="V8" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="W8" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -1051,37 +1051,37 @@
         <v>2</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="R9" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U9" s="6" t="n">
         <v>2</v>
@@ -1090,7 +1090,7 @@
         <v>2</v>
       </c>
       <c r="W9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1126,46 +1126,46 @@
         <v>1</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q10" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V10" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W10" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -1201,43 +1201,43 @@
         <v>7</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>5</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O11" s="6" t="n">
         <v>7</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>10</v>
       </c>
       <c r="R11" s="6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="S11" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="T11" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="U11" s="6" t="n">
         <v>2</v>
       </c>
       <c r="V11" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W11" s="6" t="n">
         <v>3</v>
@@ -1272,42 +1272,42 @@
         <v>3</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>1</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O12" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O12" s="4" t="inlineStr"/>
       <c r="P12" s="4" t="inlineStr"/>
-      <c r="Q12" s="4" t="inlineStr"/>
+      <c r="Q12" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="R12" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S12" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="T12" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="U12" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="V12" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="W12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -1340,46 +1340,46 @@
         <v>2</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>2</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="R13" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T13" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U13" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="V13" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W13" s="6" t="n">
         <v>7</v>
@@ -1415,19 +1415,19 @@
         <v>2</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N14" s="4" t="n">
         <v>3</v>
@@ -1436,7 +1436,7 @@
         <v>3</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>5</v>
@@ -1448,16 +1448,16 @@
         <v>5</v>
       </c>
       <c r="T14" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U14" s="4" t="n">
         <v>7</v>
       </c>
       <c r="V14" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="W14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -1490,46 +1490,46 @@
         <v>10</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="S15" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="T15" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="P15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>10</v>
-      </c>
       <c r="U15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="V15" s="6" t="n">
         <v>8</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>7</v>
       </c>
       <c r="W15" s="6" t="n">
         <v>8</v>
@@ -1571,7 +1571,9 @@
       <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr"/>
       <c r="U16" s="4" t="inlineStr"/>
-      <c r="V16" s="4" t="inlineStr"/>
+      <c r="V16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="W16" s="4" t="n">
         <v>1</v>
       </c>
@@ -1604,22 +1606,22 @@
         <v>2</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K17" s="6" t="n">
         <v>4</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M17" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N17" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O17" s="6" t="n">
         <v>3</v>
@@ -1630,9 +1632,7 @@
       <c r="Q17" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="R17" s="6" t="n">
-        <v>3</v>
-      </c>
+      <c r="R17" s="6" t="inlineStr"/>
       <c r="S17" s="6" t="inlineStr"/>
       <c r="T17" s="6" t="inlineStr"/>
       <c r="U17" s="6" t="inlineStr"/>
@@ -1656,10 +1656,10 @@
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="4" t="inlineStr"/>
       <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="inlineStr"/>
-      <c r="J18" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
@@ -1672,7 +1672,9 @@
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr"/>
       <c r="V18" s="4" t="inlineStr"/>
-      <c r="W18" s="4" t="inlineStr"/>
+      <c r="W18" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1704,34 +1706,34 @@
         <v>5</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M19" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="P19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q19" s="6" t="inlineStr"/>
-      <c r="R19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="S19" s="6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="P19" s="6" t="inlineStr"/>
+      <c r="Q19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R19" s="6" t="inlineStr"/>
+      <c r="S19" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="T19" s="6" t="n">
         <v>1</v>
       </c>
@@ -1772,29 +1774,27 @@
         <v>1</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="4" t="inlineStr"/>
       <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" s="4" t="inlineStr"/>
-      <c r="O20" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="N20" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O20" s="4" t="inlineStr"/>
       <c r="P20" s="4" t="inlineStr"/>
       <c r="Q20" s="4" t="inlineStr"/>
-      <c r="R20" s="4" t="inlineStr"/>
+      <c r="R20" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="S20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="T20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="U20" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="U20" s="4" t="inlineStr"/>
       <c r="V20" s="4" t="inlineStr"/>
       <c r="W20" s="4" t="inlineStr"/>
     </row>
@@ -1831,19 +1831,19 @@
         <v>22</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>13</v>
       </c>
       <c r="M21" s="6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="O21" s="6" t="n">
         <v>19</v>
@@ -1855,22 +1855,22 @@
         <v>19</v>
       </c>
       <c r="R21" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="S21" s="6" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="T21" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="U21" s="6" t="n">
         <v>21</v>
-      </c>
-      <c r="U21" s="6" t="n">
-        <v>20</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>21</v>
       </c>
       <c r="W21" s="6" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22">
@@ -1899,49 +1899,49 @@
         <v>100</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="J22" s="8" t="n">
         <v>106</v>
       </c>
       <c r="K22" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="L22" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="M22" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="N22" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="O22" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="P22" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="Q22" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="R22" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="S22" s="8" t="n">
         <v>106</v>
       </c>
-      <c r="L22" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="M22" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="N22" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="O22" s="8" t="n">
+      <c r="T22" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="P22" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="Q22" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="R22" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="S22" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="T22" s="8" t="n">
+      <c r="U22" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="V22" s="8" t="n">
         <v>106</v>
       </c>
-      <c r="U22" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="V22" s="8" t="n">
-        <v>105</v>
-      </c>
       <c r="W22" s="8" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1988,7 +1988,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-29</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-30</t>
         </is>
       </c>
     </row>
@@ -2030,77 +2030,77 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
     </row>
@@ -2129,37 +2129,37 @@
         <v>18</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="N4" s="4" t="n">
         <v>17</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>18</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>17</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>16</v>
       </c>
       <c r="R4" s="4" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="S4" s="4" t="n">
         <v>20</v>
@@ -2168,10 +2168,10 @@
         <v>20</v>
       </c>
       <c r="U4" s="4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -2208,37 +2208,37 @@
         <v>17</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="N5" s="6" t="n">
+      <c r="O5" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="O5" s="6" t="n">
-        <v>13</v>
-      </c>
       <c r="P5" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>14</v>
       </c>
       <c r="R5" s="6" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="S5" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>17</v>
       </c>
       <c r="U5" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="V5" s="6" t="n">
         <v>15</v>
@@ -2269,31 +2269,31 @@
         <v>6</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>4</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q6" s="4" t="n">
         <v>2</v>
@@ -2302,13 +2302,13 @@
         <v>2</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="U6" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V6" s="4" t="n">
         <v>4</v>
@@ -2345,7 +2345,7 @@
         <v>3</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>4</v>
@@ -2357,7 +2357,7 @@
         <v>4</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O7" s="6" t="n">
         <v>5</v>
@@ -2369,7 +2369,7 @@
         <v>5</v>
       </c>
       <c r="R7" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S7" s="6" t="n">
         <v>6</v>
@@ -2381,7 +2381,7 @@
         <v>6</v>
       </c>
       <c r="V7" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -2409,16 +2409,16 @@
         <v>5</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>1</v>
@@ -2427,7 +2427,7 @@
         <v>1</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>3</v>
@@ -2436,19 +2436,19 @@
         <v>3</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T8" s="4" t="n">
         <v>5</v>
       </c>
       <c r="U8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V8" s="4" t="n">
         <v>6</v>
@@ -2483,28 +2483,28 @@
         <v>6</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O9" s="6" t="n">
         <v>2</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R9" s="6" t="n">
         <v>3</v>
@@ -2513,10 +2513,10 @@
         <v>3</v>
       </c>
       <c r="T9" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U9" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V9" s="6" t="n">
         <v>2</v>
@@ -2547,25 +2547,25 @@
         <v>8</v>
       </c>
       <c r="H10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L10" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="I10" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>7</v>
-      </c>
       <c r="M10" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="N10" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>12</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>10</v>
@@ -2574,16 +2574,16 @@
         <v>10</v>
       </c>
       <c r="Q10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="R10" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="R10" s="4" t="n">
+      <c r="S10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="S10" s="4" t="n">
-        <v>10</v>
-      </c>
       <c r="T10" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="U10" s="4" t="n">
         <v>11</v>
@@ -2617,46 +2617,46 @@
         <v>39</v>
       </c>
       <c r="H11" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="K11" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="I11" s="10" t="n">
+      <c r="L11" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>47</v>
-      </c>
-      <c r="K11" s="10" t="n">
-        <v>49</v>
-      </c>
-      <c r="L11" s="10" t="n">
+      <c r="M11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="M11" s="10" t="n">
-        <v>46</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>50</v>
-      </c>
       <c r="O11" s="10" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="R11" s="10" t="n">
         <v>43</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="T11" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="U11" s="10" t="n">
         <v>40</v>
-      </c>
-      <c r="U11" s="10" t="n">
-        <v>38</v>
       </c>
       <c r="V11" s="10" t="n">
         <v>40</v>
@@ -2687,49 +2687,49 @@
         <v>100</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I12" s="8" t="n">
         <v>106</v>
       </c>
       <c r="J12" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>93</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>103</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>97</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="R12" s="8" t="n">
         <v>106</v>
       </c>
-      <c r="K12" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>93</v>
-      </c>
-      <c r="M12" s="8" t="n">
-        <v>95</v>
-      </c>
-      <c r="N12" s="8" t="n">
+      <c r="S12" s="8" t="n">
         <v>103</v>
       </c>
-      <c r="O12" s="8" t="n">
-        <v>97</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="Q12" s="8" t="n">
-        <v>99</v>
-      </c>
-      <c r="R12" s="8" t="n">
-        <v>96</v>
-      </c>
-      <c r="S12" s="8" t="n">
+      <c r="T12" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="U12" s="8" t="n">
         <v>106</v>
       </c>
-      <c r="T12" s="8" t="n">
-        <v>103</v>
-      </c>
-      <c r="U12" s="8" t="n">
-        <v>105</v>
-      </c>
       <c r="V12" s="8" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh SAT cache + report (2026-10-31)
</commit_message>
<xml_diff>
--- a/output/Evolucion_SAT.xlsx
+++ b/output/Evolucion_SAT.xlsx
@@ -528,7 +528,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por estado — 2026-10-30</t>
+          <t>Evolución abiertas SAT por estado — 2026-10-31</t>
         </is>
       </c>
     </row>
@@ -1988,7 +1988,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Evolución abiertas SAT por cadena — 2026-10-30</t>
+          <t>Evolución abiertas SAT por cadena — 2026-10-31</t>
         </is>
       </c>
     </row>

</xml_diff>